<commit_message>
Dania: wszystkie kluby Superligi i 1. Division 26/27, oceny akademii DBU, korekta FCK/Lyngby (R. Anker)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Be8XiCwvE6GnhZjaxWth9
</commit_message>
<xml_diff>
--- a/Kluby_Europa_Kontakty_Scouting.xlsx
+++ b/Kluby_Europa_Kontakty_Scouting.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Beşiktaş – korekta" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Beşiktaş – korekta'!$A$1:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -542,19 +542,19 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A2)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A2)</f>
         <v/>
       </c>
       <c r="C2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A2,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A2,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A2,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A2,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A2,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A2,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A3)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A3)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A3,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A3,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A3,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A3,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A3,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A3,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -588,19 +588,19 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A4)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A4)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A4,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A4,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A4,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A4,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A4,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A4,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -611,19 +611,19 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A5)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A5)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A5,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A5,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A5,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A5,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A5,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A5,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -634,19 +634,19 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A6)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A6)</f>
         <v/>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A6,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A6,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A6,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A6,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A6,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A6,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -657,19 +657,19 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A7)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A7)</f>
         <v/>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A7,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A7,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A7,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A7,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A7,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A7,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -680,19 +680,19 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$49,A8)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$71,A8)</f>
         <v/>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A8,Kontakty!$F$2:$F$49,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A8,Kontakty!$F$2:$F$71,"*@*")</f>
         <v/>
       </c>
       <c r="D8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A8,Kontakty!$I$2:$I$49,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A8,Kontakty!$I$2:$I$71,1)</f>
         <v/>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$49,A8,Kontakty!$J$2:$J$49,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$71,A8,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -763,6 +763,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Stan na: 26.09.2026. Stanowiska w klubach zmieniają się często – przed kampanią sprawdź źródło w kolumnie H.</t>
         </is>
@@ -779,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1417,7 +1424,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Mail widoczny na stronie, ukryty przed botami</t>
+          <t>Superliga. Najlepsza akademia w DK 2026 (DBU 5★, 97,0/100)</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1473,11 @@
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1476,29 +1487,37 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>F.C. København</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Christian Wilkens</t>
+          <t>Kristian Kjær</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Head of Recruitment (FCK Talent)</t>
+          <t>Director of Recruitment</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja akademii (starsze roczniki)</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
+          <t>Rekrutacja (dział rekrutacji)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>kfk@fcm.dk</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>uddannelse@fcm.dk</t>
+        </is>
+      </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>https://www.fck.dk/en/content/fck-talent-department-staff-and-officials</t>
+          <t>https://www.fcm.dk/drengeakademiet/</t>
         </is>
       </c>
       <c r="I14" s="9" t="n">
@@ -1506,12 +1525,12 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>Zakres roczników do potwierdzenia na stronie (U14–U17 wg strony FCK)</t>
+          <t>Superliga. DBU 5★. Head of Academy Recruitment: Mads Agner Veng (mail niepubliczny)</t>
         </is>
       </c>
     </row>
@@ -1528,28 +1547,24 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Rasmus Anker</t>
+          <t>Christian Wilkens</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Head Scout &amp; Recruitment Manager U12–U13</t>
+          <t>Head of Recruitment (FCK Talent)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja U12–U13</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>rsa@fck.dk</t>
-        </is>
-      </c>
+          <t>Rekrutacja akademii (starsze roczniki)</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr"/>
       <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
+          <t>https://www.fck.dk/en/content/fck-talent-department-staff-and-officials</t>
         </is>
       </c>
       <c r="I15" s="9" t="n">
@@ -1557,10 +1572,14 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Superliga. DBU 5★. Stanowisko U12–U13 wolne po odejściu R. Ankera do Lyngby (VIII 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1570,37 +1589,33 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Brøndby IF</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Kristian Kjær</t>
+          <t>Christian Morsing</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Director of Recruitment</t>
+          <t>Rekrutteringsansvarlig, Brøndby Masterclass</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja (dział rekrutacji)</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>kfk@fcm.dk</t>
-        </is>
-      </c>
+          <t>Kontakt z klubami ws. rekrutacji do akademii</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>uddannelse@fcm.dk</t>
+          <t>scouting.brondby.com; tel. +45 43 63 08 10</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcm.dk/drengeakademiet/</t>
+          <t>https://brondby.com/masterclass/om-masterclass/rekrutteringsprocedure-i-brondby-masterclass</t>
         </is>
       </c>
       <c r="I16" s="9" t="n">
@@ -1608,12 +1623,12 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>Head of Academy Recruitment: Mads Agner Veng (mail niepubliczny)</t>
+          <t>Superliga. DBU 4,5★ (89,39). Academy Director: Bjørn Holm; Head of Development: Jonas Bliksted</t>
         </is>
       </c>
     </row>
@@ -1625,44 +1640,48 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>FC Nordsjælland</t>
+          <t>Lyngby Boldklub</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>David Poulsen</t>
+          <t>Karsten Stiig Alnor</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Lead Scout U7–U10</t>
+          <t>Akademichef</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Scouting U7–U10</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+          <t>ks@lyngby-boldklub.dk</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr"/>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>https://fcn.dk/akademi/kontakt</t>
+          <t>https://lyngby-boldklub.dk/kontakt/</t>
         </is>
       </c>
       <c r="I17" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K17" s="7" t="inlineStr"/>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Superliga (beniaminek). DBU 4★</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1672,44 +1691,44 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>F.C. København</t>
+          <t>Lyngby Boldklub</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Rasmus Hahnemann</t>
+          <t>Rasmus Anker</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Head Scout &amp; Recruitment Manager U10–U11, ATK+</t>
+          <t>Chef for rekruttering og scouting</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja U10–U11</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>raha@fck.dk</t>
-        </is>
-      </c>
+          <t>Scouting/rekrutacja akademia → 1. zespół</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr"/>
       <c r="G18" s="7" t="inlineStr"/>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
+          <t>https://lyngby-boldklub.dk/2026/06/25/rasmus-anker-bliver-ny-chef-for-rekruttering-og-scouting/</t>
         </is>
       </c>
       <c r="I18" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K18" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>Od 01.08.2026 (wcześniej FCK). Nowy mail niepubliczny – stary rsa@fck.dk nieaktualny</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1719,37 +1738,33 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Brøndby IF</t>
+          <t>AGF</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Marc Søballe Pedersen</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Talentchef (AGF Talent)</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Portal dla scoutów/agentów</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr"/>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>scouting.brondby.com; tel. +45 43 63 08 10</t>
-        </is>
-      </c>
+      <c r="G19" s="7" t="inlineStr"/>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>https://scouting.brondby.com/</t>
+          <t>https://agf.dk/agf-talent</t>
         </is>
       </c>
       <c r="I19" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
@@ -1758,7 +1773,7 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do działu talentów</t>
+          <t>Superliga. Rekrutacja U13–U17: Kenneth Djoeneri; U10–U12: René Klok</t>
         </is>
       </c>
     </row>
@@ -1770,44 +1785,48 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>FC Nordsjælland</t>
+          <t>OB (Odense Boldklub)</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Henrik Surel</t>
+          <t>Ulrik Bredegaard</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Emerging Talent Scout U14–U19, Girls</t>
+          <t>Akademichef</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Scouting dziewcząt U14–U19</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+          <t>ulrik.bredegaard@ob.dk</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr"/>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>https://fcn.dk/akademi/kontakt</t>
+          <t>https://ob.dk/hold/akademi/akademiets-personale</t>
         </is>
       </c>
       <c r="I20" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="inlineStr"/>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Superliga. Talentchef: Benjamin Ajslev</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1817,44 +1836,52 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>F.C. København</t>
+          <t>Silkeborg IF</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Cornelius Scheel Hjeds</t>
+          <t>Nicolaj Bækgaard</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Head Scout U6–U9</t>
+          <t>Rekrutteringsansvarlig</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Scouting U6–U9</t>
+          <t>Zapytania ws. młodych zawodników</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>cohj@fck.dk</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr"/>
+          <t>nb@silkeborgif.com</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>tel. 22 98 96 10</t>
+        </is>
+      </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
+          <t>https://www.silkeborgif.com/talent/kontakt/</t>
         </is>
       </c>
       <c r="I21" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr"/>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1864,76 +1891,92 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>F.C. København</t>
+          <t>Silkeborg IF</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Casper Kåre Hansen</t>
+          <t>Peter Christian Hansen</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Talent Head, Girls/Women</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Akademia kobiet</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>cakh@fck.dk</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr"/>
+          <t>pc@silkeborgif.com</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>+45 20 27 58 35</t>
+        </is>
+      </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
+          <t>https://www.silkeborgif.com/talent/kontakt/</t>
         </is>
       </c>
       <c r="I22" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr"/>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Randers FC</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Massimiliano Notari</t>
+          <t>Peter Elstrup</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting</t>
+          <t>Talentchef &amp; Head of Coaching</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Scouting regionalny, krajowy, międzynarodowy</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>pe@randersfc.dk</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>+45 25 60 21 51; randersfc@randersfc.dk</t>
+        </is>
+      </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
+          <t>https://randersfc.dk/talent/kontakt/</t>
         </is>
       </c>
       <c r="I23" s="9" t="n">
@@ -1941,46 +1984,54 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>Potwierdzony na 2026/27, kontrakt do 30.06.2029</t>
+          <t>Superliga</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>AaB (Aalborg)</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Mattia Notari</t>
+          <t>Jakob Ahlmann</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Head of Men Youth Sector</t>
+          <t>Ansvarlig for kontraktspillere og rekruttering U15–U19</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Sektor młodzieżowy (mężczyźni)</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
+          <t>Rekrutacja do akademii</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>jah@aab-as.dk</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>tel. 28 40 15 89</t>
+        </is>
+      </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
+          <t>https://aabsport.dk/akademiet/om-aab-akademiet/</t>
         </is>
       </c>
       <c r="I24" s="9" t="n">
@@ -1988,46 +2039,50 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>Kontrakt do 30.06.2029</t>
+          <t>1. Division. Rola od 01.02.2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>AaB (Aalborg)</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Federico Crovari</t>
+          <t>Mathias Krogh</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Football Pathway Manager</t>
+          <t>Akademichef</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Ścieżka akademia → pierwszy zespół</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr"/>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>mak@aab-as.dk</t>
+        </is>
+      </c>
       <c r="G25" s="7" t="inlineStr"/>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
+          <t>https://aabsport.dk/akademiet/om-aab-akademiet/</t>
         </is>
       </c>
       <c r="I25" s="9" t="n">
@@ -2035,101 +2090,101 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>Nowa rola od 2026/27</t>
+          <t>1. Division</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Udinese Calcio</t>
+          <t>FC Nordsjælland</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Alec Bolla</t>
+          <t>David Poulsen</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Responsabile Udinese Academy</t>
+          <t>Lead Scout U7–U10</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Sieć klubów afiliowanych (60+), identyfikacja talentów</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>academy@udinesespa.it; +39 0432 544911</t>
-        </is>
-      </c>
+          <t>Scouting U7–U10</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr"/>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>https://www.udinese.it/academy/contacts</t>
+          <t>https://fcn.dk/akademi/kontakt</t>
         </is>
       </c>
       <c r="I26" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>Kontakt przez adres academy@</t>
+          <t>Superliga</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>F.C. København</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Gian Paolo Manighetti</t>
+          <t>Rasmus Hahnemann</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Responsabile Scouting (settore giovanile)</t>
+          <t>Head Scout &amp; Recruitment Manager U10–U11, ATK+</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Scouting sektora młodzieżowego</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr"/>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>settoregiovanile@atalanta.it</t>
-        </is>
-      </c>
+          <t>Scouting/rekrutacja U10–U11</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>raha@fck.dk</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr"/>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>https://www.calcioatalanta.it/category/news/approfondimenti/primavera-settore-giovanile-atalanta/</t>
+          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
         </is>
       </c>
       <c r="I27" s="9" t="n">
@@ -2137,50 +2192,54 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Dane z 2024/25 – sprawdzić aktualność</t>
+          <t>Superliga</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Empoli FC</t>
+          <t>Viborg FF</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Marco Bertelli</t>
+          <t>Mads Holm</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Responsabile Settore Giovanile</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Sektor młodzieżowy</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr"/>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>social@empolifc.com</t>
+          <t>kundeservice@vff.dk</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>https://www.empolifc.it/organigramma</t>
+          <t>https://www.vff.dk/viborg-f-f/kontaktinfo</t>
         </is>
       </c>
       <c r="I28" s="9" t="n">
@@ -2188,93 +2247,109 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>Scouting attività di base: Paolo Mussi</t>
+          <t>Superliga</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Włochy</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Sønderjyske Fodbold</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Gianluca Baschieri</t>
+          <t>Joshua Karesch</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Head of Grassroot</t>
+          <t>Scout &amp; Recruitment Manager</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Grassroots</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr"/>
+          <t>Scouting/rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>jk@soenderjyskefodbold.dk</t>
+        </is>
+      </c>
       <c r="G29" s="7" t="inlineStr"/>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
+          <t>https://soenderjyskefodbold.dk/scouting-rekruttering/</t>
         </is>
       </c>
       <c r="I29" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="inlineStr"/>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>Superliga. Scout: Steffen Dam – dam@soenderjyskefodbold.dk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Francja</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>RC Lens</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Alaeddine Yahia</t>
+          <t>Martin Bloch</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Responsable du recrutement de l'académie</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja akademii</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr"/>
-      <c r="G30" s="7" t="inlineStr"/>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>tel. 75 62 60 20</t>
+        </is>
+      </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>https://www.rclens.fr/fr/pros-cellule-de-recrutement</t>
+          <t>https://achorsens.dk/ansatte/akademiet</t>
         </is>
       </c>
       <c r="I30" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -2283,88 +2358,100 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>recrutement@rclens.fr to adres HR (oferty pracy) – nie do zgłoszeń zawodników</t>
+          <t>Superliga (beniaminek)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Francja</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Olympique Lyonnais</t>
+          <t>Vejle Boldklub</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Johann Louvel</t>
+          <t>Steen Thychosen</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Directeur de l'Academy</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr"/>
-      <c r="G31" s="7" t="inlineStr"/>
+          <t>VB Akademiet</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>st@vejle-boldklub.dk</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>+45 24 97 70 10</t>
+        </is>
+      </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>https://www.ol.fr/fr/academy/centre-de-formation/recrutement</t>
+          <t>https://vejle-boldklub.dk/vb-akademiet/staben</t>
         </is>
       </c>
       <c r="I31" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>Zastępca ds. technicznych/rekrutacji: Mathieu Seckinger</t>
+          <t>1. Division</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Francja</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Stade Rennais</t>
+          <t>Esbjerg fB</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Philippe Barraud</t>
+          <t>Anders Brynaa</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Chargé de coordination du recrutement</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja centrum szkoleniowego</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr"/>
+          <t>EfB Akademi</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
       <c r="G32" s="7" t="inlineStr"/>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
+          <t>https://efb.dk/efb-akademi/stab/</t>
         </is>
       </c>
       <c r="I32" s="9" t="n">
@@ -2372,50 +2459,54 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>Źródło nieoficjalne – potwierdzić na staderennais.com</t>
+          <t>1. Division</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Francja</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>LOSC Lille</t>
+          <t>HB Køge</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Steen Knudsen</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Formularz kontaktowy</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr"/>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>https://www.losc.fr/contact</t>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>sk@hbkoge.dk</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>+45 40 42 45 59</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>https://www.losc.fr/formation</t>
+          <t>https://www.hbkoge.dk/talentudvikling/</t>
         </is>
       </c>
       <c r="I33" s="9" t="n">
@@ -2423,446 +2514,470 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do rekrutacji młodzieży</t>
+          <t>1. Division. Klub stawia na wychowanków</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>KAA Gent</t>
+          <t>Hvidovre IF</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Jordi Maes</t>
+          <t>Christian Grønbæk</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Coördinator Scouting &amp; Rekrutering Jeugd</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja akademii</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr"/>
+          <t>Talentakademi</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>cg@hif.dk</t>
+        </is>
+      </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>formularz: kaagent.typeform.com/interessejeugd</t>
+          <t>hif@hif.dk; 36 78 17 72</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>https://www.kaagent.be/nl/jeugd/jeugdscouting</t>
+          <t>https://bredde.hif.dk/talentakademi/</t>
         </is>
       </c>
       <c r="I34" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>Brak otwartych testów – tylko zaproszenia</t>
+          <t>1. Division</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>KRC Genk</t>
+          <t>FC Nordsjælland</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Koen Daerden</t>
+          <t>Henrik Surel</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Technical Director Youth Academy</t>
+          <t>Emerging Talent Scout U14–U19, Girls</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr"/>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>https://www.krcgenk.be/en/contact</t>
-        </is>
-      </c>
+          <t>Scouting dziewcząt U14–U19</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr"/>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>https://www.krcgenk.be/en/contact</t>
+          <t>https://fcn.dk/akademi/kontakt</t>
         </is>
       </c>
       <c r="I35" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>Mail osoby tylko w bazach komercyjnych – nie podajemy</t>
+          <t>Superliga</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Cercle Brugge</t>
+          <t>F.C. København</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cornelius Scheel Hjeds</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Scouting manager jeugd</t>
+          <t>Head Scout U6–U9</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Scouting U8–U18</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr"/>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>scouting.jeugd@cerclebrugge.be</t>
-        </is>
-      </c>
+          <t>Scouting U6–U9</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>cohj@fck.dk</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr"/>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>https://cerclebrugge.be/en/teams/youth/jeugdacademie-scouting</t>
+          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
         </is>
       </c>
       <c r="I36" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K36" s="7" t="inlineStr"/>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>RSC Anderlecht</t>
+          <t>F.C. København</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Casper Kåre Hansen</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Neerpede Academy – scouting</t>
+          <t>Talent Head, Girls/Women</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Zgłoszenia zawodników</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr"/>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>formularz na rsca.be (FAQ Neerpede)</t>
-        </is>
-      </c>
+          <t>Akademia kobiet</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>cakh@fck.dk</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr"/>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>https://www.rsca.be/en/faqs/neerpede-academy</t>
+          <t>https://www.fck.dk/indhold/procedurer-rekruttering-i-talentafdelingen</t>
         </is>
       </c>
       <c r="I37" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K37" s="7" t="inlineStr"/>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Club Brugge</t>
+          <t>Akademisk Boldklub</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Simon Andresen</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Club NXT</t>
+          <t>Rekrutacja U17/U19</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Kontakt akademii</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr"/>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+          <t>Rekrutacja i testy U17–U19</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>formularz „Spillerhenvendelse” na stronie</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+          <t>https://www.akademiskboldklub.dk/klub/akademisk-boldklub--4/sider/spillerhenvendelser</t>
         </is>
       </c>
       <c r="I38" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K38" s="7" t="inlineStr"/>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>1. Division</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>LASK</t>
+          <t>Kolding IF</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Philipp Leeb</t>
+          <t>Jonas Illum</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchsleiter (Youth Director)</t>
+          <t>Talentchef (akademia chłopców i dziewcząt)</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Przyjęcia do akademii</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>p.leeb@lask.at</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>scouting@lask.at; 0699 111 879 00</t>
-        </is>
-      </c>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr"/>
+      <c r="G39" s="7" t="inlineStr"/>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>https://www.lask.at/en/m/ansprechpersonen</t>
+          <t>https://kolding-if.dk/sport/akademiet/kontakt-akademi/</t>
         </is>
       </c>
       <c r="I39" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K39" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>1. Division. Starszy kontakt jj@kolding-if.dk (Jacob Jensen, 2024) – nieaktualny</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>Hillerød Fodbold</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Hannes Thier</t>
+          <t>Peter Sørensen</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Scout (Akademie)</t>
+          <t>Talentchef</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Profile zawodników na testy</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>hannes.thier@sksturm.at</t>
-        </is>
-      </c>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr"/>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>office@akastmk-sturm.at</t>
+          <t>info@hilleroedfodbold.dk</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>http://www.akastmk-sturm.at/aufnahme.htm</t>
+          <t>https://www.hilleroedfodbold.dk/klubnyt/hilleroed-fodbold-ansaetter-peter-soerensen-som-ny-talentchef/</t>
         </is>
       </c>
       <c r="I40" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K40" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>1. Division. Od 01.01.2026</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>SK Rapid Wien</t>
+          <t>Hobro IK</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Nino Rauch</t>
+          <t>Peter Bøcher Christiansen</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Leiter Scouting</t>
+          <t>Rekrutteringsansvarlig</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr"/>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>nachwuchs@skrapid.com; info@skrapid.com</t>
-        </is>
-      </c>
+          <t>Rekrutacja do talentu</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>pbc@hikfodbold.dk</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr"/>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>https://www.skrapid.at/verein/gremien/sport-management/</t>
+          <t>https://hobroik.dk/forening/ungdom/talent/rekruttering-til-talent/</t>
         </is>
       </c>
       <c r="I41" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="inlineStr"/>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>1. Division. Od 01.07.2026. Talentchef: Martin Ingvorsen; testy U13–U19: NH@hikfodbold.dk</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>FC Red Bull Salzburg</t>
+          <t>Vendsyssel FF</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Riccardo Averini</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Akademie – Verwaltung</t>
+          <t>Head of Coaching &amp; Talentchef</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Administracja akademii</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr"/>
+          <t>Dział talentów, U17–U19</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
+          <t>tel. 30 49 66 71</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>https://www.redbullsalzburg.at/de/jungbullen/organisation-scouting.html</t>
+          <t>https://vendsysselff.dk/talent/stab/</t>
         </is>
       </c>
       <c r="I42" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
@@ -2871,190 +2986,190 @@
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do szefa scoutingu</t>
+          <t>1. Division</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>FC Fredericia</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Emil Bauer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>FC Fredericia Akademi – stab</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>emil.bauer@sksturm.at</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr"/>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcfredericia.org/Staben/</t>
+        </is>
+      </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://www.fcfredericia.org/Rekruttering/</t>
         </is>
       </c>
       <c r="I43" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K43" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>1. Division. Na stronie lista maili sztabu bez przypisanych ról – sprawdzić</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Dania</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>Aarhus Fremad</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Lukas Alterdinger</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>lukas.alterdinger@sksturm.at</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr"/>
+          <t>Formularz kontaktowy</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>https://www.aarhus-fremad.dk/kontakt/</t>
+        </is>
+      </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://www.aarhus-fremad.dk/kontakt/</t>
         </is>
       </c>
       <c r="I44" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K44" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>1. Division. Brak publicznego kontaktu do akademii</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Włochy</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Christoph Leitgeb</t>
+          <t>Massimiliano Notari</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Head of Scouting</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>christoph.leitgeb@sksturm.at</t>
-        </is>
-      </c>
+          <t>Scouting regionalny, krajowy, międzynarodowy</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr"/>
       <c r="G45" s="7" t="inlineStr"/>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
         </is>
       </c>
       <c r="I45" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K45" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>Potwierdzony na 2026/27, kontrakt do 30.06.2029</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Włochy</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>FC Zürich</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Balz Rau</t>
+          <t>Mattia Notari</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Koordinator Nachwuchsscouting</t>
+          <t>Head of Men Youth Sector</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Scouting młodzieżowy</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>balz.rau@fcz.ch</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>+41 43 521 12 12</t>
-        </is>
-      </c>
+          <t>Sektor młodzieżowy (mężczyźni)</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr"/>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcz.ch/pages/leitung-und-staff</t>
+          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
         </is>
       </c>
       <c r="I46" s="9" t="n">
@@ -3062,152 +3177,148 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>Ausbildungschef: Sascha Milicevic; Techn. Leiter: Claudio Calvi</t>
+          <t>Kontrakt do 30.06.2029</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Włochy</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>FC Basel</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Danique Stein</t>
+          <t>Federico Crovari</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Stiftung Nachwuchs-Campus Basel</t>
+          <t>Football Pathway Manager</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Campus młodzieżowy (administracja)</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>danique.stein@nachwuchs-campus.ch</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>info@fcb.ch; 061 375 10 10</t>
-        </is>
-      </c>
+          <t>Ścieżka akademia → pierwszy zespół</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr"/>
+      <c r="G47" s="7" t="inlineStr"/>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>https://www.nachwuchs-campus.ch/impressum</t>
+          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
         </is>
       </c>
       <c r="I47" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
-          <t>Rola administracyjna, nie scouting</t>
+          <t>Nowa rola od 2026/27</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Włochy</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>BSC Young Boys</t>
+          <t>Udinese Calcio</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Alec Bolla</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchsförderung</t>
+          <t>Responsabile Udinese Academy</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Sieć klubów afiliowanych (60+), identyfikacja talentów</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>info@bscyb.ch; +41 31 344 88 88</t>
+          <t>academy@udinesespa.it; +39 0432 544911</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>https://www.bscyb.ch/nachwuchsfoerderung</t>
+          <t>https://www.udinese.it/academy/contacts</t>
         </is>
       </c>
       <c r="I48" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K48" s="7" t="inlineStr"/>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt przez adres academy@</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Włochy</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Grasshopper Club Zürich</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Gian Paolo Manighetti</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchs / GC Campus</t>
+          <t>Responsabile Scouting (settore giovanile)</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Scouting sektora młodzieżowego</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>info@gcz.ch; +41 44 447 46 46</t>
+          <t>settoregiovanile@atalanta.it</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>https://www.gcz.ch/kontakt/</t>
+          <t>https://www.calcioatalanta.it/category/news/approfondimenti/primavera-settore-giovanile-atalanta/</t>
         </is>
       </c>
       <c r="I49" s="9" t="n">
@@ -3215,14 +3326,1092 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>Dane z 2024/25 – sprawdzić aktualność</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Włochy</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Empoli FC</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Marco Bertelli</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Responsabile Settore Giovanile</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Sektor młodzieżowy</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>social@empolifc.com</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>https://www.empolifc.it/organigramma</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>Scouting attività di base: Paolo Mussi</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Włochy</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Parma Calcio 1913</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Gianluca Baschieri</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Head of Grassroot</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Grassroots</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr"/>
+      <c r="G51" s="7" t="inlineStr"/>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K49" s="7" t="inlineStr"/>
+      <c r="K51" s="7" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>RC Lens</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Alaeddine Yahia</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Responsable du recrutement de l'académie</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>https://www.rclens.fr/fr/pros-cellule-de-recrutement</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>recrutement@rclens.fr to adres HR (oferty pracy) – nie do zgłoszeń zawodników</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Olympique Lyonnais</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Johann Louvel</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Directeur de l'Academy</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr"/>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ol.fr/fr/academy/centre-de-formation/recrutement</t>
+        </is>
+      </c>
+      <c r="I53" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>Zastępca ds. technicznych/rekrutacji: Mathieu Seckinger</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Philippe Barraud</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Chargé de coordination du recrutement</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja centrum szkoleniowego</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr"/>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>Źródło nieoficjalne – potwierdzić na staderennais.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>LOSC Lille</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Formularz kontaktowy</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr"/>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>https://www.losc.fr/contact</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>https://www.losc.fr/formation</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>Brak publicznego maila do rekrutacji młodzieży</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>KAA Gent</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Jordi Maes</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Coördinator Scouting &amp; Rekrutering Jeugd</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Scouting/rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>formularz: kaagent.typeform.com/interessejeugd</t>
+        </is>
+      </c>
+      <c r="H56" s="8" t="inlineStr">
+        <is>
+          <t>https://www.kaagent.be/nl/jeugd/jeugdscouting</t>
+        </is>
+      </c>
+      <c r="I56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>Brak otwartych testów – tylko zaproszenia</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>KRC Genk</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Koen Daerden</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Technical Director Youth Academy</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr"/>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>https://www.krcgenk.be/en/contact</t>
+        </is>
+      </c>
+      <c r="H57" s="8" t="inlineStr">
+        <is>
+          <t>https://www.krcgenk.be/en/contact</t>
+        </is>
+      </c>
+      <c r="I57" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>Mail osoby tylko w bazach komercyjnych – nie podajemy</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Cercle Brugge</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Scouting manager jeugd</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Scouting U8–U18</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>scouting.jeugd@cerclebrugge.be</t>
+        </is>
+      </c>
+      <c r="H58" s="8" t="inlineStr">
+        <is>
+          <t>https://cerclebrugge.be/en/teams/youth/jeugdacademie-scouting</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>RSC Anderlecht</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Neerpede Academy – scouting</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Zgłoszenia zawodników</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr"/>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>formularz na rsca.be (FAQ Neerpede)</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>https://www.rsca.be/en/faqs/neerpede-academy</t>
+        </is>
+      </c>
+      <c r="I59" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K59" s="7" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Club NXT</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt akademii</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr"/>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+        </is>
+      </c>
+      <c r="H60" s="8" t="inlineStr">
+        <is>
+          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K60" s="7" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>LASK</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Philipp Leeb</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchsleiter (Youth Director)</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Przyjęcia do akademii</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>p.leeb@lask.at</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>scouting@lask.at; 0699 111 879 00</t>
+        </is>
+      </c>
+      <c r="H61" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lask.at/en/m/ansprechpersonen</t>
+        </is>
+      </c>
+      <c r="I61" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Hannes Thier</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Scout (Akademie)</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Profile zawodników na testy</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>hannes.thier@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>office@akastmk-sturm.at</t>
+        </is>
+      </c>
+      <c r="H62" s="8" t="inlineStr">
+        <is>
+          <t>http://www.akastmk-sturm.at/aufnahme.htm</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>SK Rapid Wien</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Nino Rauch</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Leiter Scouting</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr"/>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>nachwuchs@skrapid.com; info@skrapid.com</t>
+        </is>
+      </c>
+      <c r="H63" s="8" t="inlineStr">
+        <is>
+          <t>https://www.skrapid.at/verein/gremien/sport-management/</t>
+        </is>
+      </c>
+      <c r="I63" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>FC Red Bull Salzburg</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Akademie – Verwaltung</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Administracja akademii</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr"/>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
+        </is>
+      </c>
+      <c r="H64" s="8" t="inlineStr">
+        <is>
+          <t>https://www.redbullsalzburg.at/de/jungbullen/organisation-scouting.html</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Brak publicznego maila do szefa scoutingu</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Emil Bauer</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>emil.bauer@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr"/>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+        </is>
+      </c>
+      <c r="I65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Lukas Alterdinger</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>lukas.alterdinger@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr"/>
+      <c r="H66" s="8" t="inlineStr">
+        <is>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K66" s="7" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Christoph Leitgeb</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>christoph.leitgeb@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr"/>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+        </is>
+      </c>
+      <c r="I67" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>FC Zürich</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Balz Rau</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Koordinator Nachwuchsscouting</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Scouting młodzieżowy</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>balz.rau@fcz.ch</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>+41 43 521 12 12</t>
+        </is>
+      </c>
+      <c r="H68" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcz.ch/pages/leitung-und-staff</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>Ausbildungschef: Sascha Milicevic; Techn. Leiter: Claudio Calvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>FC Basel</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Danique Stein</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Stiftung Nachwuchs-Campus Basel</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Campus młodzieżowy (administracja)</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>danique.stein@nachwuchs-campus.ch</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>info@fcb.ch; 061 375 10 10</t>
+        </is>
+      </c>
+      <c r="H69" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nachwuchs-campus.ch/impressum</t>
+        </is>
+      </c>
+      <c r="I69" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>Rola administracyjna, nie scouting</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>BSC Young Boys</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchsförderung</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr"/>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>info@bscyb.ch; +41 31 344 88 88</t>
+        </is>
+      </c>
+      <c r="H70" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bscyb.ch/nachwuchsfoerderung</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Grasshopper Club Zürich</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchs / GC Campus</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr"/>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>info@gcz.ch; +41 44 447 46 46</t>
+        </is>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
+        <is>
+          <t>https://www.gcz.ch/kontakt/</t>
+        </is>
+      </c>
+      <c r="I71" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K49"/>
-  <conditionalFormatting sqref="A2:K49">
+  <autoFilter ref="A1:K71"/>
+  <conditionalFormatting sqref="A2:K71">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Zweryfikowany"</formula>
     </cfRule>
@@ -3230,13 +4419,13 @@
       <formula>$J2="Do potwierdzenia"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I49">
+  <conditionalFormatting sqref="I2:I71">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>$I2=1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Zweryfikowany,Częściowo – brak maila osoby,Do potwierdzenia"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3272,26 +4461,50 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pelne ligi Belgii, Austrii i Szwajcarii 26/27 oraz topowe akademie wg rankingow CIES
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Be8XiCwvE6GnhZjaxWth9
</commit_message>
<xml_diff>
--- a/Kluby_Europa_Kontakty_Scouting.xlsx
+++ b/Kluby_Europa_Kontakty_Scouting.xlsx
@@ -10,10 +10,12 @@
     <sheet name="Podsumowanie" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Kontakty" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Beşiktaş – korekta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ranking CIES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Beşiktaş – korekta'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ranking CIES'!$A$1:$F$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +51,11 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -91,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +117,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -542,19 +550,19 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A2)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A2)</f>
         <v/>
       </c>
       <c r="C2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A2,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A2,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A2,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A2,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A2,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A2,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -565,19 +573,19 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A3)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A3)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A3,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A3,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A3,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A3,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A3,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A3,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -588,19 +596,19 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A4)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A4)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A4,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A4,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A4,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A4,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A4,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A4,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -611,19 +619,19 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A5)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A5)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A5,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A5,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A5,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A5,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A5,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A5,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -634,19 +642,19 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A6)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A6)</f>
         <v/>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A6,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A6,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A6,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A6,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A6,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A6,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -657,19 +665,19 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A7)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A7)</f>
         <v/>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A7,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A7,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A7,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A7,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A7,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A7,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -680,96 +688,264 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$71,A8)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A8)</f>
         <v/>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A8,Kontakty!$F$2:$F$71,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A8,Kontakty!$F$2:$F$119,"*@*")</f>
         <v/>
       </c>
       <c r="D8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A8,Kontakty!$I$2:$I$71,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A8,Kontakty!$I$2:$I$119,1)</f>
         <v/>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$71,A8,Kontakty!$J$2:$J$71,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A8,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A9,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D9" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A9,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E9" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A9,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A10,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D10" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A10,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E10" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A10,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A11,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D11" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A11,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E11" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A11,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Niemcy</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A12,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D12" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A12,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E12" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A12,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A13,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D13" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A13,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E13" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A13,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A14,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D14" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A14,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E14" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A14,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Ukraina</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$119,A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A15,Kontakty!$F$2:$F$119,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D15" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A15,Kontakty!$I$2:$I$119,1)</f>
+        <v/>
+      </c>
+      <c r="E15" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$119,A15,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>RAZEM</t>
         </is>
       </c>
-      <c r="B9" s="3">
-        <f>SUM(B2:B8)</f>
+      <c r="B16" s="3">
+        <f>SUM(B2:B15)</f>
         <v/>
       </c>
-      <c r="C9" s="3">
-        <f>SUM(C2:C8)</f>
+      <c r="C16" s="3">
+        <f>SUM(C2:C15)</f>
         <v/>
       </c>
-      <c r="D9" s="3">
-        <f>SUM(D2:D8)</f>
+      <c r="D16" s="3">
+        <f>SUM(D2:D15)</f>
         <v/>
       </c>
-      <c r="E9" s="3">
-        <f>SUM(E2:E8)</f>
+      <c r="E16" s="3">
+        <f>SUM(E2:E15)</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Legenda</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Stan na: 26.09.2026. Stanowiska w klubach zmieniają się często – przed kampanią sprawdź źródło w kolumnie H.</t>
         </is>
@@ -786,7 +962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3331,7 +3507,7 @@
       </c>
       <c r="K49" s="7" t="inlineStr">
         <is>
-          <t>Dane z 2024/25 – sprawdzić aktualność</t>
+          <t>Dane z 2024/25 – sprawdzić aktualność. CIES: w top 10 najbardziej dochodowych akademii (ranking 2024)</t>
         </is>
       </c>
     </row>
@@ -3437,29 +3613,29 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>RC Lens</t>
+          <t>Stade Rennais (CIES)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Alaeddine Yahia</t>
+          <t>Denis Arnaud</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Responsable du recrutement de l'académie</t>
+          <t>Directeur de l'académie</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja akademii</t>
+          <t>Centre de formation</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr"/>
       <c r="G52" s="7" t="inlineStr"/>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>https://www.rclens.fr/fr/pros-cellule-de-recrutement</t>
+          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
         </is>
       </c>
       <c r="I52" s="9" t="n">
@@ -3467,12 +3643,12 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>recrutement@rclens.fr to adres HR (oferty pracy) – nie do zgłoszeń zawodników</t>
+          <t>CIES 2026: 4. miejsce w Europie – 29 wychowanków w lidze Big-5. Nazwisko dyrektora do potwierdzenia</t>
         </is>
       </c>
     </row>
@@ -3484,29 +3660,33 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Olympique Lyonnais</t>
+          <t>AS Monaco (CIES)</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Johann Louvel</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Directeur de l'Academy</t>
+          <t>Cellule recrutement Academy (La Diagonale)</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Rekrutacja do centrum szkoleniowego</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr"/>
-      <c r="G53" s="7" t="inlineStr"/>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>https://www.asmonaco.com/encadrement/</t>
+        </is>
+      </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>https://www.ol.fr/fr/academy/centre-de-formation/recrutement</t>
+          <t>https://www.asmonaco.com/en/academy/la-diagonale-centre-de-formation-de-las-monaco</t>
         </is>
       </c>
       <c r="I53" s="9" t="n">
@@ -3514,12 +3694,12 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
         <is>
-          <t>Zastępca ds. technicznych/rekrutacji: Mathieu Seckinger</t>
+          <t>CIES: top 10 najbardziej dochodowych akademii (10 lat). Nie przyjmują zgłoszeń spontanicznych</t>
         </is>
       </c>
     </row>
@@ -3531,42 +3711,42 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Stade Rennais</t>
+          <t>RC Lens</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Philippe Barraud</t>
+          <t>Alaeddine Yahia</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Chargé de coordination du recrutement</t>
+          <t>Responsable du recrutement de l'académie</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja centrum szkoleniowego</t>
+          <t>Rekrutacja akademii</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr"/>
       <c r="G54" s="7" t="inlineStr"/>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
+          <t>https://www.rclens.fr/fr/pros-cellule-de-recrutement</t>
         </is>
       </c>
       <c r="I54" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>Źródło nieoficjalne – potwierdzić na staderennais.com</t>
+          <t>recrutement@rclens.fr to adres HR (oferty pracy) – nie do zgłoszeń zawodników</t>
         </is>
       </c>
     </row>
@@ -3578,148 +3758,140 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>LOSC Lille</t>
+          <t>Olympique Lyonnais</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Johann Louvel</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Directeur de l'Academy</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Formularz kontaktowy</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr"/>
-      <c r="G55" s="8" t="inlineStr">
-        <is>
-          <t>https://www.losc.fr/contact</t>
-        </is>
-      </c>
+      <c r="G55" s="7" t="inlineStr"/>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>https://www.losc.fr/formation</t>
+          <t>https://www.ol.fr/fr/academy/centre-de-formation/recrutement</t>
         </is>
       </c>
       <c r="I55" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do rekrutacji młodzieży</t>
+          <t>CIES: top 10 dochodów ze sprzedaży wychowanków; 34 wychowanków w Big-5. Zastępca ds. technicznych/rekrutacji: Mathieu Seckinger</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Francja</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>KAA Gent</t>
+          <t>Stade Rennais</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Jordi Maes</t>
+          <t>Philippe Barraud</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Coördinator Scouting &amp; Rekrutering Jeugd</t>
+          <t>Chargé de coordination du recrutement</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja akademii</t>
+          <t>Rekrutacja centrum szkoleniowego</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr"/>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>formularz: kaagent.typeform.com/interessejeugd</t>
-        </is>
-      </c>
+      <c r="G56" s="7" t="inlineStr"/>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>https://www.kaagent.be/nl/jeugd/jeugdscouting</t>
+          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
         </is>
       </c>
       <c r="I56" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>Brak otwartych testów – tylko zaproszenia</t>
+          <t>Źródło nieoficjalne – potwierdzić na staderennais.com</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Francja</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>KRC Genk</t>
+          <t>LOSC Lille</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Koen Daerden</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Technical Director Youth Academy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Formularz kontaktowy</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr"/>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>https://www.krcgenk.be/en/contact</t>
+          <t>https://www.losc.fr/contact</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>https://www.krcgenk.be/en/contact</t>
+          <t>https://www.losc.fr/formation</t>
         </is>
       </c>
       <c r="I57" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr">
         <is>
-          <t>Mail osoby tylko w bazach komercyjnych – nie podajemy</t>
+          <t>Brak publicznego maila do rekrutacji młodzieży</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3903,7 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Cercle Brugge</t>
+          <t>Club Brugge</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
@@ -3741,34 +3913,38 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Scouting manager jeugd</t>
+          <t>Club NXT – akademia</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Scouting U8–U18</t>
+          <t>Kontakt akademii</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr"/>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>scouting.jeugd@cerclebrugge.be</t>
+      <c r="G58" s="8" t="inlineStr">
+        <is>
+          <t>https://www.clubbrugge.be/en/nxt-contact</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>https://cerclebrugge.be/en/teams/youth/jeugdacademie-scouting</t>
+          <t>https://www.clubbrugge.be/en/nxt-contact</t>
         </is>
       </c>
       <c r="I58" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K58" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Club NXT – najlepsza akademia w Belgii 2 lata z rzędu</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3783,17 +3959,17 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Afrim Salievski</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Neerpede Academy – scouting</t>
+          <t>Academy Talent Director</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Zgłoszenia zawodników</t>
+          <t>Rekrutacja i scouting wszystkich kategorii młodzieżowych</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr"/>
@@ -3804,18 +3980,22 @@
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>https://www.rsca.be/en/faqs/neerpede-academy</t>
+          <t>https://www.rsca.be/en/afrim-salievski</t>
         </is>
       </c>
       <c r="I59" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K59" s="7" t="inlineStr"/>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Chief Academy: Tim Borguet; Football Director U13–U23: Tim Scheers</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3825,84 +4005,84 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Club Brugge</t>
+          <t>KRC Genk</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Koen Daerden</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Club NXT</t>
+          <t>Technical Director Youth Academy</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Kontakt akademii</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr"/>
-      <c r="G60" s="8" t="inlineStr">
-        <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>jeugdsecretariaat@krcgenk.be</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+          <t>https://www.krcgenk.be/nl/contact/locatie/jeugdscouting</t>
         </is>
       </c>
       <c r="I60" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K60" s="7" t="inlineStr"/>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. ~20 scoutów młodzieżowych; mail osoby tylko w bazach komercyjnych – nie podajemy</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>LASK</t>
+          <t>KAA Gent</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Philipp Leeb</t>
+          <t>Jordi Maes</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchsleiter (Youth Director)</t>
+          <t>Coördinator Scouting &amp; Rekrutering Jeugd</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Przyjęcia do akademii</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>p.leeb@lask.at</t>
-        </is>
-      </c>
+          <t>Scouting/rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr"/>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>scouting@lask.at; 0699 111 879 00</t>
+          <t>formularz: kaagent.typeform.com/interessejeugd</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>https://www.lask.at/en/m/ansprechpersonen</t>
+          <t>https://www.kaagent.be/nl/jeugd/jeugdscouting</t>
         </is>
       </c>
       <c r="I61" s="9" t="n">
@@ -3910,50 +4090,50 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
-        </is>
-      </c>
-      <c r="K61" s="7" t="inlineStr"/>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Brak otwartych testów – tylko zaproszenia</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>Union Saint-Gilloise</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Hannes Thier</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Scout (Akademie)</t>
+          <t>Union Academy – scouting</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Profile zawodników na testy</t>
-        </is>
-      </c>
-      <c r="F62" s="7" t="inlineStr">
-        <is>
-          <t>hannes.thier@sksturm.at</t>
-        </is>
-      </c>
+          <t>Scouting akademii</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>office@akastmk-sturm.at</t>
+          <t>scouting@rusgacademy.be; tel. 02 332 04 73</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>http://www.akastmk-sturm.at/aufnahme.htm</t>
+          <t>https://rusg.brussels/en/union-academy/contact-union-academy</t>
         </is>
       </c>
       <c r="I62" s="9" t="n">
@@ -3964,43 +4144,47 @@
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K62" s="7" t="inlineStr"/>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>SK Rapid Wien</t>
+          <t>Standard de Liège</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Nino Rauch</t>
+          <t>Christophe Lonnoy</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Leiter Scouting</t>
+          <t>Directeur Recrutement ARLD</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Rekrutacja Académie Robert Louis-Dreyfus</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>nachwuchs@skrapid.com; info@skrapid.com</t>
+          <t>i.vanherle@standard.be (Ingrid Vanherle, manager adm.); tel. +32 4 385 94 00</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>https://www.skrapid.at/verein/gremien/sport-management/</t>
+          <t>https://standard.be/fr/news/academie-robert-louis-dreyfus</t>
         </is>
       </c>
       <c r="I63" s="9" t="n">
@@ -4011,43 +4195,51 @@
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K63" s="7" t="inlineStr"/>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>FC Red Bull Salzburg</t>
+          <t>Royal Antwerp FC</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ralph Rust</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Akademie – Verwaltung</t>
+          <t>Head of Scouting &amp; Recruitment U13–U18</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Administracja akademii</t>
-        </is>
-      </c>
-      <c r="F64" s="7" t="inlineStr"/>
+          <t>Scouting/rekrutacja U13–U18</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>ralph.rust@rafc.be</t>
+        </is>
+      </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
+          <t>formularz: form.jotformeu.com/RoyalAntwerpFC/scouting-request-rafc</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>https://www.redbullsalzburg.at/de/jungbullen/organisation-scouting.html</t>
+          <t>https://jeugd.royalantwerpfc.be/contact/</t>
         </is>
       </c>
       <c r="I64" s="9" t="n">
@@ -4055,97 +4247,101 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do szefa scoutingu</t>
+          <t>Pro League</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>KV Mechelen</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Emil Bauer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Scouting jeugdacademie</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>emil.bauer@sksturm.at</t>
-        </is>
-      </c>
-      <c r="G65" s="7" t="inlineStr"/>
+          <t>Rekrutacja do akademii</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr"/>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>scouting@kvmechelen.be; info@kvmechelenjeugd.be</t>
+        </is>
+      </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://kvmechelen.be/academie/contact/</t>
         </is>
       </c>
       <c r="I65" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K65" s="7" t="inlineStr"/>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>Royal Antwerp FC</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Lukas Alterdinger</t>
+          <t>Vincent Verbrugghe</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Head of Scouting &amp; Recruitment U10–U12</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Scouting/rekrutacja U10–U12</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>lukas.alterdinger@sksturm.at</t>
+          <t>vincent.verbrugghe@rafc.be</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr"/>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://jeugd.royalantwerpfc.be/contact/</t>
         </is>
       </c>
       <c r="I66" s="9" t="n">
@@ -4156,43 +4352,47 @@
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K66" s="7" t="inlineStr"/>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>OH Leuven</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Christoph Leitgeb</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Academy</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F67" s="7" t="inlineStr">
-        <is>
-          <t>christoph.leitgeb@sksturm.at</t>
-        </is>
-      </c>
-      <c r="G67" s="7" t="inlineStr"/>
+          <t>Akademia / scouting</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>jeugd@ohl.be</t>
+        </is>
+      </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://www.ohleuven.com/academy/scouting</t>
         </is>
       </c>
       <c r="I67" s="9" t="n">
@@ -4203,51 +4403,51 @@
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K67" s="7" t="inlineStr"/>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>FC Zürich</t>
+          <t>Cercle Brugge</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Balz Rau</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Koordinator Nachwuchsscouting</t>
+          <t>Scouting manager jeugd</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>Scouting młodzieżowy</t>
-        </is>
-      </c>
-      <c r="F68" s="7" t="inlineStr">
-        <is>
-          <t>balz.rau@fcz.ch</t>
-        </is>
-      </c>
+          <t>Scouting U8–U18</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr"/>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>+41 43 521 12 12</t>
+          <t>scouting.jeugd@cerclebrugge.be</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcz.ch/pages/leitung-und-staff</t>
+          <t>https://cerclebrugge.be/en/teams/youth/jeugdacademie-scouting</t>
         </is>
       </c>
       <c r="I68" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
@@ -4256,49 +4456,49 @@
       </c>
       <c r="K68" s="7" t="inlineStr">
         <is>
-          <t>Ausbildungschef: Sascha Milicevic; Techn. Leiter: Claudio Calvi</t>
+          <t>Pro League</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>FC Basel</t>
+          <t>KV Kortrijk</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Danique Stein</t>
+          <t>Niels Bulcaen</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Stiftung Nachwuchs-Campus Basel</t>
+          <t>KVK Scouting (jeugdacademie)</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Campus młodzieżowy (administracja)</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>danique.stein@nachwuchs-campus.ch</t>
+          <t>niels.bulcaen@kvk.be</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>info@fcb.ch; 061 375 10 10</t>
+          <t>+32 56 96 01 90</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>https://www.nachwuchs-campus.ch/impressum</t>
+          <t>https://www.kvk.be/club/jeugdacademie/kvk-scouting/</t>
         </is>
       </c>
       <c r="I69" s="9" t="n">
@@ -4311,45 +4511,45 @@
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>Rola administracyjna, nie scouting</t>
+          <t>Pro League (beniaminek)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>BSC Young Boys</t>
+          <t>Lommel SK</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Kevin Wielockx</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchsförderung</t>
+          <t>Head of Youth Scouting</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Scouting młodzieżowy</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr"/>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>info@bscyb.ch; +41 31 344 88 88</t>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lommelsk.be/nl/talent-scouting.php</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>https://www.bscyb.ch/nachwuchsfoerderung</t>
+          <t>https://www.lommelsk.be/nl/talent-scouting.php</t>
         </is>
       </c>
       <c r="I70" s="9" t="n">
@@ -4360,17 +4560,21 @@
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K70" s="7" t="inlineStr"/>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>Pro League (beniaminek). Klub City Football Group</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Grasshopper Club Zürich</t>
+          <t>SK Beveren</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
@@ -4380,23 +4584,23 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchs / GC Campus</t>
+          <t>Jeugdwerking</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Akademia (tylko e-mail)</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr"/>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>info@gcz.ch; +41 44 447 46 46</t>
+          <t>jeugd@skbeveren.be</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>https://www.gcz.ch/kontakt/</t>
+          <t>https://www.skbeveren.be/contact/</t>
         </is>
       </c>
       <c r="I71" s="9" t="n">
@@ -4404,14 +4608,2498 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>Pro League (beniaminek, mistrz CPL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Sporting Charleroi</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Zebra Academy</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Akademia U15–U23</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>info@sporting-charleroi.be; 071 23 97 50</t>
+        </is>
+      </c>
+      <c r="H72" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sporting-charleroi.be/contact/</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K71" s="7" t="inlineStr"/>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Brak publicznego maila akademii</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Royal Antwerp FC</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Matthias De Ridder</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Head of Scouting &amp; Recruitment U7–U9</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Scouting U7–U9</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>matthias.deridder@rafcjeugd.be</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr"/>
+      <c r="H73" s="8" t="inlineStr">
+        <is>
+          <t>https://jeugd.royalantwerpfc.be/contact/</t>
+        </is>
+      </c>
+      <c r="I73" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>KVC Westerlo</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr"/>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>info@kvcwesterlo.be; +32 14 54 52 88</t>
+        </is>
+      </c>
+      <c r="H74" s="8" t="inlineStr">
+        <is>
+          <t>https://kvcwesterlo.be/nl/contact/</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Brak publicznego maila scoutingu młodzieży</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Sint-Truidense VV</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Luc Bormans</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Hoofd jeugdopleiding</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr"/>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>info@stvv.com; 011 71 38 19</t>
+        </is>
+      </c>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>https://stvv.com/en/contact</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Dane osoby z nieoficjalnej strony – potwierdzić</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>SV Zulte Waregem</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Essevee Academie</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr"/>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>formularz: essevee.be/nl/team-essevee/contact</t>
+        </is>
+      </c>
+      <c r="H76" s="8" t="inlineStr">
+        <is>
+          <t>https://www.essevee.be/nl/team-essevee/contact</t>
+        </is>
+      </c>
+      <c r="I76" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>Pro League. Brak publicznego maila akademii</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>RAAL La Louvière</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Wolves Academy</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja młodzieży</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr"/>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>jeunes@raal.be; zgłoszenia: raal.be/recrutement-2/</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>https://www.raal.be/ufaq/jaimerais-realiser-un-test-pour-integrer-lecole-des-jeunes-comment-faire/</t>
+        </is>
+      </c>
+      <c r="I77" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>Pro League</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>FC Red Bull Salzburg</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Manfred Pamminger</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Gesamtleiter Nachwuchs (w tym scouting)</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>Akademia, FC Liefering, scouting, współpraca międzynarodowa</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>https://www.redbullsalzburg.at/de/jungbullen-und-akademie</t>
+        </is>
+      </c>
+      <c r="I78" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga. Sportlicher Leiter Akademie: Raphael Ikache</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Hannes Thier</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Scout (Akademie)</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Profile zawodników na testy</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>hannes.thier@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>office@akastmk-sturm.at</t>
+        </is>
+      </c>
+      <c r="H79" s="8" t="inlineStr">
+        <is>
+          <t>http://www.akastmk-sturm.at/aufnahme.htm</t>
+        </is>
+      </c>
+      <c r="I79" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>SK Rapid Wien</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Nino Rauch</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Leiter Scouting</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr"/>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>nachwuchs@skrapid.com; info@skrapid.com</t>
+        </is>
+      </c>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>https://www.skrapid.at/verein/gremien/sport-management/</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K80" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>FK Austria Wien</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Manuel Takacs</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Leiter Akademie</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr"/>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>https://fk-austria.at/en/akademie-2/kontakt-2</t>
+        </is>
+      </c>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>https://fk-austria.at/en/news/die-sportdirektion-von-austria-wien</t>
+        </is>
+      </c>
+      <c r="I81" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga. Technical Director: Robert Urbanek</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>LASK</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Philipp Leeb</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchsleiter</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Przyjęcia do akademii</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>p.leeb@lask.at</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>scouting@lask.at; 0699 111 879 00</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lask.at/en/m/ansprechpersonen</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J82" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K82" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Emil Bauer</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>emil.bauer@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr"/>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+        </is>
+      </c>
+      <c r="I83" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K83" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Lukas Alterdinger</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>lukas.alterdinger@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr"/>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+        </is>
+      </c>
+      <c r="I84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K84" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Christoph Leitgeb</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>christoph.leitgeb@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr"/>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+        </is>
+      </c>
+      <c r="I85" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J85" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K85" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Grazer AK</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Christian Zach</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>Sportlicher Leiter Akademie</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>christian.zach@grazerak.at</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>office@grazerak.at</t>
+        </is>
+      </c>
+      <c r="H86" s="8" t="inlineStr">
+        <is>
+          <t>https://grazerak.at/verein/ansprechpartner-nachwuchs</t>
+        </is>
+      </c>
+      <c r="I86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J86" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K86" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga. Jugend &amp; Schulkoop.: Philipp Albrecht – philipp.albrecht@grazerak.at</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Wolfsberger AC</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr"/>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>office@rzpelletswac.at; +43 4352 30688</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
+          <t>https://rzpelletswac.at/kontakt/</t>
+        </is>
+      </c>
+      <c r="I87" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J87" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K87" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga. Brak publicznego maila akademii</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>TSV Hartberg</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>Hartberg Fußball Akademie</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F88" s="7" t="inlineStr"/>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>akademie@tsv-hartberg-fussball.at</t>
+        </is>
+      </c>
+      <c r="H88" s="8" t="inlineStr">
+        <is>
+          <t>https://tsv-hartberg-fussball.at/nachwuchs/kontakt-nachwuchs/</t>
+        </is>
+      </c>
+      <c r="I88" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J88" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K88" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>AKA-Geschäftsstelle</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>Akademia Ried</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr"/>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>office@akaried.at; +43 7752 88164</t>
+        </is>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
+        <is>
+          <t>https://www.svried.at/aka-geschaeftsstelle/</t>
+        </is>
+      </c>
+      <c r="I89" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J89" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K89" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>WSG Tirol</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchs</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>Młodzież, testy</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr"/>
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>jugendfussball@wsg-fussball.at; 0699 108 619 35</t>
+        </is>
+      </c>
+      <c r="H90" s="8" t="inlineStr">
+        <is>
+          <t>https://www.wsg-fussball.at/de/nachwuchs/infos/</t>
+        </is>
+      </c>
+      <c r="I90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J90" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K90" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>SCR Altach</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>SCRA Nachwuchs</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>Młodzież (największa w Vorarlbergu)</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr"/>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>https://www.scra.at/teams/nachwuchs/scra-nachwuchs</t>
+        </is>
+      </c>
+      <c r="H91" s="8" t="inlineStr">
+        <is>
+          <t>https://www.scra.at/teams/nachwuchs/scra-nachwuchs</t>
+        </is>
+      </c>
+      <c r="I91" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J91" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K91" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga. Brak publicznego maila</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>SC Austria Lustenau</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Mike Urschitz</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>Sportlicher Nachwuchsleiter</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Młodzież</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr"/>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>info@austria-lustenau.at; +43 5577 86250</t>
+        </is>
+      </c>
+      <c r="H92" s="8" t="inlineStr">
+        <is>
+          <t>https://www.austria-lustenau.at/kontakt</t>
+        </is>
+      </c>
+      <c r="I92" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J92" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K92" s="7" t="inlineStr">
+        <is>
+          <t>Bundesliga (beniaminek). Tel. do osoby: +43 699 19202012</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>BSC Young Boys</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Christian Franke</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>Technischer Direktor Youth Base</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Akademia (U15–U21)</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr"/>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>info@bscyb.ch; +41 31 344 88 88</t>
+        </is>
+      </c>
+      <c r="H93" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bscyb.ch/youth-base-staff</t>
+        </is>
+      </c>
+      <c r="I93" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J93" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K93" s="7" t="inlineStr">
+        <is>
+          <t>Super League</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>FC Basel</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Timo Jankowski</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>Leiter Nachwuchs</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchs-Campus</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr"/>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>info@fcb.ch; 061 375 10 10</t>
+        </is>
+      </c>
+      <c r="H94" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcb.ch/aktuell/news/nachwuchs/veraenderungen-auf-dem-campus-januar-2026</t>
+        </is>
+      </c>
+      <c r="I94" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J94" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K94" s="7" t="inlineStr">
+        <is>
+          <t>Super League. Administracja Campusu: danique.stein@nachwuchs-campus.ch</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>FC Zürich</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Balz Rau</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>Koordinator Nachwuchsscouting</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>Scouting młodzieżowy</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>balz.rau@fcz.ch</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>+41 43 521 12 12</t>
+        </is>
+      </c>
+      <c r="H95" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcz.ch/pages/leitung-und-staff</t>
+        </is>
+      </c>
+      <c r="I95" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J95" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K95" s="7" t="inlineStr">
+        <is>
+          <t>Super League. Ausbildungschef: Sascha Milicevic; Techn. Leiter: Claudio Calvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>FC Thun</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Jürg Frey</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>Leiter Nachwuchs</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>Młodzież</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>juerg.frey@fcthun.ch</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="inlineStr">
+        <is>
+          <t>033 225 18 98; info@fcthun.ch</t>
+        </is>
+      </c>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcthun.ch/de/teams/nachwuchs</t>
+        </is>
+      </c>
+      <c r="I96" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J96" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K96" s="7" t="inlineStr">
+        <is>
+          <t>Super League – aktualny mistrz Szwajcarii</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>FC Lugano</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Roman Hangarter</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Direttore Academy</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>Akademia + Partenariato Ticino (od 26/27)</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr"/>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>+41 91 922 86 72</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>https://fclugano.com/en/academy/</t>
+        </is>
+      </c>
+      <c r="I97" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J97" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K97" s="7" t="inlineStr">
+        <is>
+          <t>Super League. Chief Sports Officer: Sebastian Pelzer</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>FC Lausanne-Sport</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Massimo Ceccaroni</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>Directeur Technique Académie</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F98" s="7" t="inlineStr"/>
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>+41 21 641 05 30</t>
+        </is>
+      </c>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lausanne-sport.ch/contact/</t>
+        </is>
+      </c>
+      <c r="I98" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J98" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K98" s="7" t="inlineStr">
+        <is>
+          <t>Super League</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>FC Vaduz</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>Lorenz Gassner</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>Leiter Nachwuchs</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>Młodzież</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>lorenz.gassner@fcvaduz.li</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>+41 78 773 76 13; info@fcvaduz.li</t>
+        </is>
+      </c>
+      <c r="H99" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcvaduz.li/kontakt</t>
+        </is>
+      </c>
+      <c r="I99" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J99" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K99" s="7" t="inlineStr">
+        <is>
+          <t>Super League (beniaminek)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>FC St. Gallen</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>David Garcia</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>Academy Director – Future Champs Ostschweiz</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>Akademia regionu Ostschweiz</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr"/>
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>info@futurechamps.ch; +41 71 314 14 14</t>
+        </is>
+      </c>
+      <c r="H100" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcsg.ch/future-champs/organisation/kontakt/</t>
+        </is>
+      </c>
+      <c r="I100" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J100" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K100" s="7" t="inlineStr">
+        <is>
+          <t>Super League</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>Servette FC</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>Académie SFC</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F101" s="7" t="inlineStr"/>
+      <c r="G101" s="7" t="inlineStr">
+        <is>
+          <t>tel. +41 22 340 54 74</t>
+        </is>
+      </c>
+      <c r="H101" s="8" t="inlineStr">
+        <is>
+          <t>https://servettefc.ch/academie/je-veux-jouer-au-sfc/</t>
+        </is>
+      </c>
+      <c r="I101" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J101" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K101" s="7" t="inlineStr">
+        <is>
+          <t>Super League</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>FC Sion</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>Xavier Henriques</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="inlineStr">
+        <is>
+          <t>Coordinateur Académie/Formation</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F102" s="7" t="inlineStr"/>
+      <c r="G102" s="7" t="inlineStr">
+        <is>
+          <t>secretariat@fcsion.ch; 027 747 13 13</t>
+        </is>
+      </c>
+      <c r="H102" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcsion.ch/fr/administration/</t>
+        </is>
+      </c>
+      <c r="I102" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J102" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K102" s="7" t="inlineStr">
+        <is>
+          <t>Super League</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>FC Luzern</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchs</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
+          <t>Młodzież</t>
+        </is>
+      </c>
+      <c r="F103" s="7" t="inlineStr"/>
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>kontakt@fcl-verein.ch; 0848 317 000</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
+        <is>
+          <t>https://fcl.ch/role/nachwuchs/</t>
+        </is>
+      </c>
+      <c r="I103" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J103" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K103" s="7" t="inlineStr">
+        <is>
+          <t>Super League. Brak publicznego maila akademii</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>Szwajcaria</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>Grasshopper Club Zürich</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t>Nachwuchs / GC Campus</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F104" s="7" t="inlineStr"/>
+      <c r="G104" s="7" t="inlineStr">
+        <is>
+          <t>info@gcz.ch; +41 44 447 46 46</t>
+        </is>
+      </c>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>https://www.gcz.ch/kontakt/</t>
+        </is>
+      </c>
+      <c r="I104" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J104" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K104" s="7" t="inlineStr">
+        <is>
+          <t>Super League</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>SL Benfica</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>Departamento de Scouting e Avaliação de Jogadores</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>Scouting U10–U19 (bez otwartych testów)</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr"/>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>formularz: slbenfica.pt/en-us/apoio/contactos</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
+        <is>
+          <t>https://www.slbenfica.pt/en-us/futebol-formacao/formacao/prospecao/recrutamento-jogadores</t>
+        </is>
+      </c>
+      <c r="I105" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J105" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K105" s="7" t="inlineStr">
+        <is>
+          <t>CIES 2026: nr 1 na świecie wg przychodów ze sprzedaży wychowanków (589 mln € / 10 lat); 73 wychowanków w 31 ligach UEFA (2. miejsce)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr">
+        <is>
+          <t>Academia Cristiano Ronaldo</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>Scouting akademii (Alcochete)</t>
+        </is>
+      </c>
+      <c r="F106" s="7" t="inlineStr"/>
+      <c r="G106" s="8" t="inlineStr">
+        <is>
+          <t>https://escolasacademia.sporting.pt</t>
+        </is>
+      </c>
+      <c r="H106" s="8" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Academia_Cristiano_Ronaldo</t>
+        </is>
+      </c>
+      <c r="I106" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J106" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K106" s="7" t="inlineStr">
+        <is>
+          <t>CIES 2026: 3. miejsce w Training Index; najlepsza akademia spoza Big-5 wg wychowanków w Big-5 (24); top 10 dochodów ze sprzedaży</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>Nelson Oliveira</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>Head of Recruitment</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>Scouting – zgłaszanie zawodników</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr"/>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>geral.scouting@fcporto.pt</t>
+        </is>
+      </c>
+      <c r="H107" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcporto.pt/pt/contactos</t>
+        </is>
+      </c>
+      <c r="I107" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J107" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K107" s="7" t="inlineStr">
+        <is>
+          <t>Oficjalny adres działu scoutingu do przesyłania informacji o zawodnikach. Uznana akademia sprzedażowa (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>AFC Ajax</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>Kelvin de Lang</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr">
+        <is>
+          <t>Head of Scouting &amp; Recruitment, Academy De Toekomst</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>Scouting akademii</t>
+        </is>
+      </c>
+      <c r="F108" s="7" t="inlineStr"/>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ajax.nl/club/jeugdopleiding</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ajax.nl/artikelen/ajax-doc-scouten-voor-de-toekomst</t>
+        </is>
+      </c>
+      <c r="I108" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J108" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K108" s="7" t="inlineStr">
+        <is>
+          <t>CIES 2026: nr 1 w Europie – 85 wychowanków w 31 ligach UEFA, 1. miejsce Training Index; 2. na świecie w sprzedaży wychowanków (454 mln €)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>Rini de Groot</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr">
+        <is>
+          <t>Hoofd jeugdscouting</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>Scouting akademii (De Herdgang)</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr"/>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>Oirschotsedijk 12a, 5651 GC Eindhoven</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t>https://www.psv.nl/en/club/psv-campus-de-herdgang-1/psv-campus</t>
+        </is>
+      </c>
+      <c r="I109" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J109" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K109" s="7" t="inlineStr">
+        <is>
+          <t>Head of Scouting klubu: Jan Vennegoor of Hesselink. Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>Feyenoord</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="inlineStr">
+        <is>
+          <t>Ricardo Kern</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="inlineStr">
+        <is>
+          <t>Coördinator wedstrijdzaken Feyenoord Academy</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="inlineStr">
+        <is>
+          <t>Scouting / sprawy drużyn akademii</t>
+        </is>
+      </c>
+      <c r="F110" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G110" s="7" t="inlineStr">
+        <is>
+          <t>Olympiaweg 280, 3078 HT Rotterdam</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
+        <is>
+          <t>https://www.feyenoord.com/nl/academy/contact</t>
+        </is>
+      </c>
+      <c r="I110" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J110" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K110" s="7" t="inlineStr">
+        <is>
+          <t>Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D111" s="7" t="inlineStr">
+        <is>
+          <t>AZ Jeugdopleiding</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="inlineStr">
+        <is>
+          <t>Akademia, dni selekcji U8–U13</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr"/>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>https://www.az.nl/jeugdopleiding</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
+        <is>
+          <t>https://www.az.nl/jeugdopleiding/az-voetbalschool</t>
+        </is>
+      </c>
+      <c r="I111" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J111" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K111" s="7" t="inlineStr">
+        <is>
+          <t>Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>Real Sociedad</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="inlineStr">
+        <is>
+          <t>Zubieta (cantera)</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>Akademia – głównie talenty z Gipuzkoa</t>
+        </is>
+      </c>
+      <c r="F112" s="7" t="inlineStr"/>
+      <c r="G112" s="7" t="inlineStr">
+        <is>
+          <t>realsociedad.eus</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Real_Sociedad_Cantera</t>
+        </is>
+      </c>
+      <c r="I112" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J112" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K112" s="7" t="inlineStr">
+        <is>
+          <t>CIES 2026: top 10 w Europie wg wychowanków w Big-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>Villarreal CF</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t>Cantera Grogueta</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>Akademia (36 drużyn, ~650 zawodników)</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr"/>
+      <c r="G113" s="7" t="inlineStr">
+        <is>
+          <t>formularz: villarrealcf.es/en/formulario-contacto/</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
+        <is>
+          <t>https://villarrealcf.es/es/cantera-grogueta/</t>
+        </is>
+      </c>
+      <c r="I113" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J113" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K113" s="7" t="inlineStr">
+        <is>
+          <t>Bez otwartych testów dla chłopców. Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>Valencia CF</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>Academia VCF (Paterna)</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr"/>
+      <c r="G114" s="8" t="inlineStr">
+        <is>
+          <t>https://formacion.valenciacf.com/en/contacto/</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
+        <is>
+          <t>https://www.valenciacf.com/vcf-academy</t>
+        </is>
+      </c>
+      <c r="I114" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J114" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K114" s="7" t="inlineStr">
+        <is>
+          <t>Wg klubu: 4. najlepsza akademia w Europie (ranking CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>Niemcy</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>Bayer 04 Leverkusen</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>Jennifer Weber</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>Geschäftsstelle Nachwuchsabteilung (NLZ)</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>Biuro akademii, testy tylko przez e-mail</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>Jennifer.Weber@bayer04.de</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>tel. 0214 866 03 43</t>
+        </is>
+      </c>
+      <c r="H115" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bayer04.de/en-us/page/youth/trial-sessions</t>
+        </is>
+      </c>
+      <c r="I115" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J115" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K115" s="7" t="inlineStr">
+        <is>
+          <t>CIES: top 10 dochodów ze sprzedaży wychowanków (10 lat). Mail z organigramu NLZ – sprawdzić aktualność</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>GNK Dinamo Zagreb</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>Dinamo Akademija</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr"/>
+      <c r="G116" s="7" t="inlineStr">
+        <is>
+          <t>dinamo@gnkdinamo.hr; 01 238 6111</t>
+        </is>
+      </c>
+      <c r="H116" s="8" t="inlineStr">
+        <is>
+          <t>https://gnkdinamo.hr/hr/info/kontakt</t>
+        </is>
+      </c>
+      <c r="I116" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J116" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K116" s="7" t="inlineStr">
+        <is>
+          <t>Czołowa akademia sprzedażowa regionu (poza top 10 CIES 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>FK Partizan</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>Omladinska škola</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr"/>
+      <c r="G117" s="8" t="inlineStr">
+        <is>
+          <t>https://partizan.rs/en</t>
+        </is>
+      </c>
+      <c r="H117" s="8" t="inlineStr">
+        <is>
+          <t>http://www.en.partizan.rs/omladinska-skola-fudbala/</t>
+        </is>
+      </c>
+      <c r="I117" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J117" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K117" s="7" t="inlineStr">
+        <is>
+          <t>CIES: wcześniej nr 1 rocznego rankingu akademii (przed Ajaxem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>FK Crvena zvezda</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t>Omladinska škola</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F118" s="7" t="inlineStr"/>
+      <c r="G118" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crvenazvezdafk.com/en/klub/kontakt-i-lokacija</t>
+        </is>
+      </c>
+      <c r="H118" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crvenazvezdafk.com/en/vesti-kategorija/omladinska-shkola</t>
+        </is>
+      </c>
+      <c r="I118" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J118" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K118" s="7" t="inlineStr">
+        <is>
+          <t>Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t>Ukraina</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>Dynamo Kijów</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>Dział scoutingu</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F119" s="7" t="inlineStr"/>
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>tel. +38 044 278 06 28</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="inlineStr">
+        <is>
+          <t>https://fcdynamo.com/en/pages/contacts</t>
+        </is>
+      </c>
+      <c r="I119" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J119" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K119" s="7" t="inlineStr">
+        <is>
+          <t>CIES 2026: 3. miejsce w Europie – 72 wychowanków w 31 ligach UEFA. Uwaga: sytuacja wojenna</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K71"/>
-  <conditionalFormatting sqref="A2:K71">
+  <autoFilter ref="A1:K119"/>
+  <conditionalFormatting sqref="A2:K119">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Zweryfikowany"</formula>
     </cfRule>
@@ -4419,13 +7107,13 @@
       <formula>$J2="Do potwierdzenia"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I71">
+  <conditionalFormatting sqref="I2:I119">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>$I2=1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Zweryfikowany,Częściowo – brak maila osoby,Do potwierdzenia"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4483,16 +7171,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId66"/>
@@ -4503,8 +7191,65 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId132"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4725,4 +7470,550 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Ranking CIES</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Miejsce</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Klub</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Kraj</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Wynik</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Status w bazie</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w ligach Big-5 (WP529, 2026)</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>FC Barcelona</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>40 zawodników</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Poza zasięgiem – tylko informacyjnie</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w ligach Big-5 (WP529, 2026)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>35 zawodników</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Poza zasięgiem – tylko informacyjnie</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w ligach Big-5 (WP529, 2026)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>31 zawodników</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Poza zasięgiem – tylko informacyjnie</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w ligach Big-5 (WP529, 2026)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>29 zawodników</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w ligach Big-5 (WP529, 2026)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>AFC Ajax</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>27 zawodników (1. spoza Big-5)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w ligach Big-5 (WP529, 2026)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>6–10</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Chelsea, Real Sociedad, Man. United, Man. City, Arsenal</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Anglia/Hiszpania</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Real Sociedad w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w 31 ligach UEFA (2026)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>AFC Ajax</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>85 zawodników</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w 31 ligach UEFA (2026)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>SL Benfica</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>73 zawodników</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w 31 ligach UEFA (2026)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Dynamo Kijów</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Ukraina</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>72 zawodników</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Training Index (ważony poziomem)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>3. miejsce w obu tabelach</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Przychody ze sprzedaży wychowanków – 10 lat (WP540, 2026)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>SL Benfica</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Portugalia</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>589 mln €</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Przychody ze sprzedaży wychowanków – 10 lat (WP540, 2026)</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>AFC Ajax</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Holandia</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>454 mln €</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Przychody ze sprzedaży wychowanków – 10 lat (WP540, 2026)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Chelsea FC</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Anglia</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>442 mln €</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Poza zasięgiem – tylko informacyjnie</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Przychody ze sprzedaży wychowanków – 10 lat (WP540, 2026)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>4–10</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Olympique Lyonnais, AS Monaco, Sporting CP, Man. City, Real Madrid, Palmeiras, Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Lyon, Monaco, Sporting, Leverkusen w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Przychody ze sprzedaży wychowanków – 5 lat (WP540, 2026)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Chelsea FC</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Anglia</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>366 mln €</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Poza zasięgiem – tylko informacyjnie</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Przychody ze sprzedaży wychowanków – 5 lat (WP540, 2026)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Anglia</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>318 mln €</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Poza zasięgiem – tylko informacyjnie</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Źródła: CIES Football Observatory – Weekly Post 529 (training clubs), Weekly Post 540 (most profitable academies), 2026. football-observatory.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Kluby z CIES Monthly Report 99: Athletic, Barcelona, Real Madrid, PSG, Man United; Atalanta 2026/27
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Be8XiCwvE6GnhZjaxWth9
</commit_message>
<xml_diff>
--- a/Kluby_Europa_Kontakty_Scouting.xlsx
+++ b/Kluby_Europa_Kontakty_Scouting.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Ranking CIES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$124</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Beşiktaş – korekta'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ranking CIES'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ranking CIES'!$A$1:$F$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A2)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A2)</f>
         <v/>
       </c>
       <c r="C2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A2,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A2,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A2,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A2,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A2,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A2,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -573,19 +573,19 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A3)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A3)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A3,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A3,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A3,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A3,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A3,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A3,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -596,19 +596,19 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A4)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A4)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A4,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A4,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A4,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A4,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A4,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A4,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -619,19 +619,19 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A5)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A5)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A5,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A5,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A5,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A5,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A5,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A5,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -642,19 +642,19 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A6)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A6)</f>
         <v/>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A6,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A6,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A6,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A6,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A6,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A6,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -665,19 +665,19 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A7)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A7)</f>
         <v/>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A7,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A7,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A7,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A7,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A7,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A7,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -688,19 +688,19 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A8)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A8)</f>
         <v/>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A8,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A8,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A8,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A8,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A8,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A8,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -711,19 +711,19 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A9)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A9)</f>
         <v/>
       </c>
       <c r="C9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A9,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A9,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A9,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A9,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A9,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A9,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -734,19 +734,19 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A10)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A10)</f>
         <v/>
       </c>
       <c r="C10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A10,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A10,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A10,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A10,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A10,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A10,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -757,19 +757,19 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A11)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A11)</f>
         <v/>
       </c>
       <c r="C11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A11,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A11,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A11,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A11,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A11,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A11,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -780,19 +780,19 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A12)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A12)</f>
         <v/>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A12,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A12,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A12,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A12,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A12,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A12,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A13)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A13)</f>
         <v/>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A13,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A13,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A13,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A13,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A13,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A13,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A14)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A14)</f>
         <v/>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A14,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A14,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A14,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A14,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A14,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A14,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -849,103 +849,126 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$119,A15)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A15)</f>
         <v/>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A15,Kontakty!$F$2:$F$119,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A15,Kontakty!$F$2:$F$124,"*@*")</f>
         <v/>
       </c>
       <c r="D15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A15,Kontakty!$I$2:$I$119,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A15,Kontakty!$I$2:$I$124,1)</f>
         <v/>
       </c>
       <c r="E15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$119,A15,Kontakty!$J$2:$J$119,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A15,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Anglia</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$124,A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A16,Kontakty!$F$2:$F$124,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D16" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A16,Kontakty!$I$2:$I$124,1)</f>
+        <v/>
+      </c>
+      <c r="E16" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$124,A16,Kontakty!$J$2:$J$124,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>RAZEM</t>
         </is>
       </c>
-      <c r="B16" s="3">
-        <f>SUM(B2:B15)</f>
+      <c r="B17" s="3">
+        <f>SUM(B2:B16)</f>
         <v/>
       </c>
-      <c r="C16" s="3">
-        <f>SUM(C2:C15)</f>
+      <c r="C17" s="3">
+        <f>SUM(C2:C16)</f>
         <v/>
       </c>
-      <c r="D16" s="3">
-        <f>SUM(D2:D15)</f>
+      <c r="D17" s="3">
+        <f>SUM(D2:D16)</f>
         <v/>
       </c>
-      <c r="E16" s="3">
-        <f>SUM(E2:E15)</f>
+      <c r="E17" s="3">
+        <f>SUM(E2:E16)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Legenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
+          <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
+          <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
+          <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
+          <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
+          <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Stan na: 26.09.2026. Stanowiska w klubach zmieniają się często – przed kampanią sprawdź źródło w kolumnie H.</t>
         </is>
@@ -962,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:K124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3473,17 +3496,17 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Gian Paolo Manighetti</t>
+          <t>Roberto Samaden</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Responsabile Scouting (settore giovanile)</t>
+          <t>Responsabile Settore Giovanile (2026/27)</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Scouting sektora młodzieżowego</t>
+          <t>Sektor młodzieżowy</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
@@ -3494,20 +3517,20 @@
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>https://www.calcioatalanta.it/category/news/approfondimenti/primavera-settore-giovanile-atalanta/</t>
+          <t>https://www.zonacalciofaidate.it/news-dai-campi-e-sedi-settori-giovanili/settore-giovanile-atalanta-2026-2027-tutti-gli-allenatori-e-la-nuova-squadra-di-roberto-samaden</t>
         </is>
       </c>
       <c r="I49" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr">
         <is>
-          <t>Dane z 2024/25 – sprawdzić aktualność. CIES: w top 10 najbardziej dochodowych akademii (ranking 2024)</t>
+          <t>CIES MR99: 94 wychowanków w Big-5 w 20 lat, top 10 wg minut. Wcześniejszy szef scoutingu młodzieży: Gian Paolo Manighetti (2024/25)</t>
         </is>
       </c>
     </row>
@@ -3898,12 +3921,12 @@
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Belgia</t>
+          <t>Francja</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Club Brugge</t>
+          <t>Paris Saint-Germain</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
@@ -3913,27 +3936,27 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Club NXT – akademia</t>
+          <t>Centre de formation – cellule recrutement</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Kontakt akademii</t>
+          <t>Rekrutacja tylko przez obserwacje scoutów</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr"/>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+          <t>https://www.psg.fr/en/youth-football</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+          <t>https://www.psg.fr/en/youth-football</t>
         </is>
       </c>
       <c r="I58" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
@@ -3942,7 +3965,7 @@
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Club NXT – najlepsza akademia w Belgii 2 lata z rzędu</t>
+          <t>CIES MR99: 3. miejsce – 111 wychowanków w Big-5 (20 lat). Klub nie przyjmuje zgłoszeń spontanicznych</t>
         </is>
       </c>
     </row>
@@ -3954,33 +3977,33 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>RSC Anderlecht</t>
+          <t>Club Brugge</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Afrim Salievski</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Academy Talent Director</t>
+          <t>Club NXT – akademia</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja i scouting wszystkich kategorii młodzieżowych</t>
+          <t>Kontakt akademii</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr"/>
-      <c r="G59" s="7" t="inlineStr">
-        <is>
-          <t>formularz na rsca.be (FAQ Neerpede)</t>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>https://www.clubbrugge.be/en/nxt-contact</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>https://www.rsca.be/en/afrim-salievski</t>
+          <t>https://www.clubbrugge.be/en/nxt-contact</t>
         </is>
       </c>
       <c r="I59" s="9" t="n">
@@ -3993,7 +4016,7 @@
       </c>
       <c r="K59" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Chief Academy: Tim Borguet; Football Director U13–U23: Tim Scheers</t>
+          <t>Pro League. Club NXT – najlepsza akademia w Belgii 2 lata z rzędu</t>
         </is>
       </c>
     </row>
@@ -4005,33 +4028,33 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>KRC Genk</t>
+          <t>RSC Anderlecht</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Koen Daerden</t>
+          <t>Afrim Salievski</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Technical Director Youth Academy</t>
+          <t>Academy Talent Director</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Rekrutacja i scouting wszystkich kategorii młodzieżowych</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr"/>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>jeugdsecretariaat@krcgenk.be</t>
+          <t>formularz na rsca.be (FAQ Neerpede)</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>https://www.krcgenk.be/nl/contact/locatie/jeugdscouting</t>
+          <t>https://www.rsca.be/en/afrim-salievski</t>
         </is>
       </c>
       <c r="I60" s="9" t="n">
@@ -4044,7 +4067,7 @@
       </c>
       <c r="K60" s="7" t="inlineStr">
         <is>
-          <t>Pro League. ~20 scoutów młodzieżowych; mail osoby tylko w bazach komercyjnych – nie podajemy</t>
+          <t>Pro League. Chief Academy: Tim Borguet; Football Director U13–U23: Tim Scheers</t>
         </is>
       </c>
     </row>
@@ -4056,33 +4079,33 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>KAA Gent</t>
+          <t>KRC Genk</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Jordi Maes</t>
+          <t>Koen Daerden</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Coördinator Scouting &amp; Rekrutering Jeugd</t>
+          <t>Technical Director Youth Academy</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja akademii</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr"/>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>formularz: kaagent.typeform.com/interessejeugd</t>
+          <t>jeugdsecretariaat@krcgenk.be</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>https://www.kaagent.be/nl/jeugd/jeugdscouting</t>
+          <t>https://www.krcgenk.be/nl/contact/locatie/jeugdscouting</t>
         </is>
       </c>
       <c r="I61" s="9" t="n">
@@ -4095,7 +4118,7 @@
       </c>
       <c r="K61" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Brak otwartych testów – tylko zaproszenia</t>
+          <t>Pro League. ~20 scoutów młodzieżowych; mail osoby tylko w bazach komercyjnych – nie podajemy</t>
         </is>
       </c>
     </row>
@@ -4107,33 +4130,33 @@
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Union Saint-Gilloise</t>
+          <t>KAA Gent</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Jordi Maes</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Union Academy – scouting</t>
+          <t>Coördinator Scouting &amp; Rekrutering Jeugd</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii</t>
+          <t>Scouting/rekrutacja akademii</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>scouting@rusgacademy.be; tel. 02 332 04 73</t>
+          <t>formularz: kaagent.typeform.com/interessejeugd</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>https://rusg.brussels/en/union-academy/contact-union-academy</t>
+          <t>https://www.kaagent.be/nl/jeugd/jeugdscouting</t>
         </is>
       </c>
       <c r="I62" s="9" t="n">
@@ -4141,12 +4164,12 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>Pro League</t>
+          <t>Pro League. Brak otwartych testów – tylko zaproszenia</t>
         </is>
       </c>
     </row>
@@ -4158,33 +4181,33 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Standard de Liège</t>
+          <t>Union Saint-Gilloise</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Christophe Lonnoy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Directeur Recrutement ARLD</t>
+          <t>Union Academy – scouting</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja Académie Robert Louis-Dreyfus</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>i.vanherle@standard.be (Ingrid Vanherle, manager adm.); tel. +32 4 385 94 00</t>
+          <t>scouting@rusgacademy.be; tel. 02 332 04 73</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>https://standard.be/fr/news/academie-robert-louis-dreyfus</t>
+          <t>https://rusg.brussels/en/union-academy/contact-union-academy</t>
         </is>
       </c>
       <c r="I63" s="9" t="n">
@@ -4192,7 +4215,7 @@
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr">
@@ -4209,37 +4232,33 @@
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Royal Antwerp FC</t>
+          <t>Standard de Liège</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Ralph Rust</t>
+          <t>Christophe Lonnoy</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting &amp; Recruitment U13–U18</t>
+          <t>Directeur Recrutement ARLD</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja U13–U18</t>
-        </is>
-      </c>
-      <c r="F64" s="7" t="inlineStr">
-        <is>
-          <t>ralph.rust@rafc.be</t>
-        </is>
-      </c>
+          <t>Rekrutacja Académie Robert Louis-Dreyfus</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr"/>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>formularz: form.jotformeu.com/RoyalAntwerpFC/scouting-request-rafc</t>
+          <t>i.vanherle@standard.be (Ingrid Vanherle, manager adm.); tel. +32 4 385 94 00</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>https://jeugd.royalantwerpfc.be/contact/</t>
+          <t>https://standard.be/fr/news/academie-robert-louis-dreyfus</t>
         </is>
       </c>
       <c r="I64" s="9" t="n">
@@ -4247,7 +4266,7 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr">
@@ -4264,33 +4283,37 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>KV Mechelen</t>
+          <t>Royal Antwerp FC</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ralph Rust</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Scouting jeugdacademie</t>
+          <t>Head of Scouting &amp; Recruitment U13–U18</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja do akademii</t>
-        </is>
-      </c>
-      <c r="F65" s="7" t="inlineStr"/>
+          <t>Scouting/rekrutacja U13–U18</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>ralph.rust@rafc.be</t>
+        </is>
+      </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>scouting@kvmechelen.be; info@kvmechelenjeugd.be</t>
+          <t>formularz: form.jotformeu.com/RoyalAntwerpFC/scouting-request-rafc</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>https://kvmechelen.be/academie/contact/</t>
+          <t>https://jeugd.royalantwerpfc.be/contact/</t>
         </is>
       </c>
       <c r="I65" s="9" t="n">
@@ -4315,37 +4338,37 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Royal Antwerp FC</t>
+          <t>KV Mechelen</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Vincent Verbrugghe</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting &amp; Recruitment U10–U12</t>
+          <t>Scouting jeugdacademie</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Scouting/rekrutacja U10–U12</t>
-        </is>
-      </c>
-      <c r="F66" s="7" t="inlineStr">
-        <is>
-          <t>vincent.verbrugghe@rafc.be</t>
-        </is>
-      </c>
-      <c r="G66" s="7" t="inlineStr"/>
+          <t>Rekrutacja do akademii</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr"/>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>scouting@kvmechelen.be; info@kvmechelenjeugd.be</t>
+        </is>
+      </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>https://jeugd.royalantwerpfc.be/contact/</t>
+          <t>https://kvmechelen.be/academie/contact/</t>
         </is>
       </c>
       <c r="I66" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
@@ -4366,33 +4389,33 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>OH Leuven</t>
+          <t>Royal Antwerp FC</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Vincent Verbrugghe</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Academy</t>
+          <t>Head of Scouting &amp; Recruitment U10–U12</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Akademia / scouting</t>
-        </is>
-      </c>
-      <c r="F67" s="7" t="inlineStr"/>
-      <c r="G67" s="7" t="inlineStr">
-        <is>
-          <t>jeugd@ohl.be</t>
-        </is>
-      </c>
+          <t>Scouting/rekrutacja U10–U12</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>vincent.verbrugghe@rafc.be</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr"/>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>https://www.ohleuven.com/academy/scouting</t>
+          <t>https://jeugd.royalantwerpfc.be/contact/</t>
         </is>
       </c>
       <c r="I67" s="9" t="n">
@@ -4417,7 +4440,7 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Cercle Brugge</t>
+          <t>OH Leuven</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
@@ -4427,23 +4450,23 @@
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Scouting manager jeugd</t>
+          <t>Academy</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>Scouting U8–U18</t>
+          <t>Akademia / scouting</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr"/>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>scouting.jeugd@cerclebrugge.be</t>
+          <t>jeugd@ohl.be</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>https://cerclebrugge.be/en/teams/youth/jeugdacademie-scouting</t>
+          <t>https://www.ohleuven.com/academy/scouting</t>
         </is>
       </c>
       <c r="I68" s="9" t="n">
@@ -4468,37 +4491,33 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>KV Kortrijk</t>
+          <t>Cercle Brugge</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Niels Bulcaen</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>KVK Scouting (jeugdacademie)</t>
+          <t>Scouting manager jeugd</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii</t>
-        </is>
-      </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>niels.bulcaen@kvk.be</t>
-        </is>
-      </c>
+          <t>Scouting U8–U18</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr"/>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>+32 56 96 01 90</t>
+          <t>scouting.jeugd@cerclebrugge.be</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>https://www.kvk.be/club/jeugdacademie/kvk-scouting/</t>
+          <t>https://cerclebrugge.be/en/teams/youth/jeugdacademie-scouting</t>
         </is>
       </c>
       <c r="I69" s="9" t="n">
@@ -4511,7 +4530,7 @@
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>Pro League (beniaminek)</t>
+          <t>Pro League</t>
         </is>
       </c>
     </row>
@@ -4523,33 +4542,37 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Lommel SK</t>
+          <t>KV Kortrijk</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Kevin Wielockx</t>
+          <t>Niels Bulcaen</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Head of Youth Scouting</t>
+          <t>KVK Scouting (jeugdacademie)</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Scouting młodzieżowy</t>
-        </is>
-      </c>
-      <c r="F70" s="7" t="inlineStr"/>
-      <c r="G70" s="8" t="inlineStr">
-        <is>
-          <t>https://www.lommelsk.be/nl/talent-scouting.php</t>
+          <t>Scouting akademii</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>niels.bulcaen@kvk.be</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>+32 56 96 01 90</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>https://www.lommelsk.be/nl/talent-scouting.php</t>
+          <t>https://www.kvk.be/club/jeugdacademie/kvk-scouting/</t>
         </is>
       </c>
       <c r="I70" s="9" t="n">
@@ -4557,12 +4580,12 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>Pro League (beniaminek). Klub City Football Group</t>
+          <t>Pro League (beniaminek)</t>
         </is>
       </c>
     </row>
@@ -4574,33 +4597,33 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>SK Beveren</t>
+          <t>Lommel SK</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Kevin Wielockx</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Jeugdwerking</t>
+          <t>Head of Youth Scouting</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Akademia (tylko e-mail)</t>
+          <t>Scouting młodzieżowy</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr"/>
-      <c r="G71" s="7" t="inlineStr">
-        <is>
-          <t>jeugd@skbeveren.be</t>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lommelsk.be/nl/talent-scouting.php</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>https://www.skbeveren.be/contact/</t>
+          <t>https://www.lommelsk.be/nl/talent-scouting.php</t>
         </is>
       </c>
       <c r="I71" s="9" t="n">
@@ -4608,12 +4631,12 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K71" s="7" t="inlineStr">
         <is>
-          <t>Pro League (beniaminek, mistrz CPL)</t>
+          <t>Pro League (beniaminek). Klub City Football Group</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4648,7 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Sporting Charleroi</t>
+          <t>SK Beveren</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -4635,23 +4658,23 @@
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Zebra Academy</t>
+          <t>Jeugdwerking</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>Akademia U15–U23</t>
+          <t>Akademia (tylko e-mail)</t>
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr"/>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>info@sporting-charleroi.be; 071 23 97 50</t>
+          <t>jeugd@skbeveren.be</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>https://www.sporting-charleroi.be/contact/</t>
+          <t>https://www.skbeveren.be/contact/</t>
         </is>
       </c>
       <c r="I72" s="9" t="n">
@@ -4659,12 +4682,12 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K72" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Brak publicznego maila akademii</t>
+          <t>Pro League (beniaminek, mistrz CPL)</t>
         </is>
       </c>
     </row>
@@ -4676,46 +4699,46 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Royal Antwerp FC</t>
+          <t>Sporting Charleroi</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Matthias De Ridder</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting &amp; Recruitment U7–U9</t>
+          <t>Zebra Academy</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Scouting U7–U9</t>
-        </is>
-      </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>matthias.deridder@rafcjeugd.be</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="inlineStr"/>
+          <t>Akademia U15–U23</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>info@sporting-charleroi.be; 071 23 97 50</t>
+        </is>
+      </c>
       <c r="H73" s="8" t="inlineStr">
         <is>
-          <t>https://jeugd.royalantwerpfc.be/contact/</t>
+          <t>https://www.sporting-charleroi.be/contact/</t>
         </is>
       </c>
       <c r="I73" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr">
         <is>
-          <t>Pro League</t>
+          <t>Pro League. Brak publicznego maila akademii</t>
         </is>
       </c>
     </row>
@@ -4727,33 +4750,33 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>KVC Westerlo</t>
+          <t>Royal Antwerp FC</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Matthias De Ridder</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Head of Scouting &amp; Recruitment U7–U9</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
-        </is>
-      </c>
-      <c r="F74" s="7" t="inlineStr"/>
-      <c r="G74" s="7" t="inlineStr">
-        <is>
-          <t>info@kvcwesterlo.be; +32 14 54 52 88</t>
-        </is>
-      </c>
+          <t>Scouting U7–U9</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>matthias.deridder@rafcjeugd.be</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr"/>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>https://kvcwesterlo.be/nl/contact/</t>
+          <t>https://jeugd.royalantwerpfc.be/contact/</t>
         </is>
       </c>
       <c r="I74" s="9" t="n">
@@ -4761,12 +4784,12 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K74" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Brak publicznego maila scoutingu młodzieży</t>
+          <t>Pro League</t>
         </is>
       </c>
     </row>
@@ -4778,33 +4801,33 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Sint-Truidense VV</t>
+          <t>KVC Westerlo</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Luc Bormans</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Hoofd jeugdopleiding</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Kontakt ogólny</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr"/>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>info@stvv.com; 011 71 38 19</t>
+          <t>info@kvcwesterlo.be; +32 14 54 52 88</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
         <is>
-          <t>https://stvv.com/en/contact</t>
+          <t>https://kvcwesterlo.be/nl/contact/</t>
         </is>
       </c>
       <c r="I75" s="9" t="n">
@@ -4812,12 +4835,12 @@
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K75" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Dane osoby z nieoficjalnej strony – potwierdzić</t>
+          <t>Pro League. Brak publicznego maila scoutingu młodzieży</t>
         </is>
       </c>
     </row>
@@ -4829,17 +4852,17 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>SV Zulte Waregem</t>
+          <t>Sint-Truidense VV</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Luc Bormans</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Essevee Academie</t>
+          <t>Hoofd jeugdopleiding</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -4850,12 +4873,12 @@
       <c r="F76" s="7" t="inlineStr"/>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>formularz: essevee.be/nl/team-essevee/contact</t>
+          <t>info@stvv.com; 011 71 38 19</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>https://www.essevee.be/nl/team-essevee/contact</t>
+          <t>https://stvv.com/en/contact</t>
         </is>
       </c>
       <c r="I76" s="9" t="n">
@@ -4863,12 +4886,12 @@
       </c>
       <c r="J76" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K76" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Brak publicznego maila akademii</t>
+          <t>Pro League. Dane osoby z nieoficjalnej strony – potwierdzić</t>
         </is>
       </c>
     </row>
@@ -4880,7 +4903,7 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>RAAL La Louvière</t>
+          <t>SV Zulte Waregem</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
@@ -4890,23 +4913,23 @@
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Wolves Academy</t>
+          <t>Essevee Academie</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja młodzieży</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr"/>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>jeunes@raal.be; zgłoszenia: raal.be/recrutement-2/</t>
+          <t>formularz: essevee.be/nl/team-essevee/contact</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
         <is>
-          <t>https://www.raal.be/ufaq/jaimerais-realiser-un-test-pour-integrer-lecole-des-jeunes-comment-faire/</t>
+          <t>https://www.essevee.be/nl/team-essevee/contact</t>
         </is>
       </c>
       <c r="I77" s="9" t="n">
@@ -4914,63 +4937,63 @@
       </c>
       <c r="J77" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K77" s="7" t="inlineStr">
         <is>
-          <t>Pro League</t>
+          <t>Pro League. Brak publicznego maila akademii</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>FC Red Bull Salzburg</t>
+          <t>RAAL La Louvière</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>Manfred Pamminger</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Gesamtleiter Nachwuchs (w tym scouting)</t>
+          <t>Wolves Academy</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>Akademia, FC Liefering, scouting, współpraca międzynarodowa</t>
+          <t>Rekrutacja młodzieży</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr"/>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
+          <t>jeunes@raal.be; zgłoszenia: raal.be/recrutement-2/</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>https://www.redbullsalzburg.at/de/jungbullen-und-akademie</t>
+          <t>https://www.raal.be/ufaq/jaimerais-realiser-un-test-pour-integrer-lecole-des-jeunes-comment-faire/</t>
         </is>
       </c>
       <c r="I78" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K78" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga. Sportlicher Leiter Akademie: Raphael Ikache</t>
+          <t>Pro League</t>
         </is>
       </c>
     </row>
@@ -4982,37 +5005,33 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>FC Red Bull Salzburg</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Hannes Thier</t>
+          <t>Manfred Pamminger</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Scout (Akademie)</t>
+          <t>Gesamtleiter Nachwuchs (w tym scouting)</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>Profile zawodników na testy</t>
-        </is>
-      </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>hannes.thier@sksturm.at</t>
-        </is>
-      </c>
+          <t>Akademia, FC Liefering, scouting, współpraca międzynarodowa</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr"/>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>office@akastmk-sturm.at</t>
+          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
         <is>
-          <t>http://www.akastmk-sturm.at/aufnahme.htm</t>
+          <t>https://www.redbullsalzburg.at/de/jungbullen-und-akademie</t>
         </is>
       </c>
       <c r="I79" s="9" t="n">
@@ -5020,12 +5039,12 @@
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K79" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Bundesliga. Sportlicher Leiter Akademie: Raphael Ikache</t>
         </is>
       </c>
     </row>
@@ -5037,33 +5056,37 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>SK Rapid Wien</t>
+          <t>SK Sturm Graz</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Nino Rauch</t>
+          <t>Hannes Thier</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Leiter Scouting</t>
+          <t>Scout (Akademie)</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
-        </is>
-      </c>
-      <c r="F80" s="7" t="inlineStr"/>
+          <t>Profile zawodników na testy</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>hannes.thier@sksturm.at</t>
+        </is>
+      </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>nachwuchs@skrapid.com; info@skrapid.com</t>
+          <t>office@akastmk-sturm.at</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>https://www.skrapid.at/verein/gremien/sport-management/</t>
+          <t>http://www.akastmk-sturm.at/aufnahme.htm</t>
         </is>
       </c>
       <c r="I80" s="9" t="n">
@@ -5071,7 +5094,7 @@
       </c>
       <c r="J80" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K80" s="7" t="inlineStr">
@@ -5088,33 +5111,33 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>FK Austria Wien</t>
+          <t>SK Rapid Wien</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Manuel Takacs</t>
+          <t>Nino Rauch</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Leiter Akademie</t>
+          <t>Leiter Scouting</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Scouting</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr"/>
-      <c r="G81" s="8" t="inlineStr">
-        <is>
-          <t>https://fk-austria.at/en/akademie-2/kontakt-2</t>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>nachwuchs@skrapid.com; info@skrapid.com</t>
         </is>
       </c>
       <c r="H81" s="8" t="inlineStr">
         <is>
-          <t>https://fk-austria.at/en/news/die-sportdirektion-von-austria-wien</t>
+          <t>https://www.skrapid.at/verein/gremien/sport-management/</t>
         </is>
       </c>
       <c r="I81" s="9" t="n">
@@ -5127,7 +5150,7 @@
       </c>
       <c r="K81" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga. Technical Director: Robert Urbanek</t>
+          <t>Bundesliga</t>
         </is>
       </c>
     </row>
@@ -5139,37 +5162,33 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>LASK</t>
+          <t>FK Austria Wien</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>Philipp Leeb</t>
+          <t>Manuel Takacs</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchsleiter</t>
+          <t>Leiter Akademie</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>Przyjęcia do akademii</t>
-        </is>
-      </c>
-      <c r="F82" s="7" t="inlineStr">
-        <is>
-          <t>p.leeb@lask.at</t>
-        </is>
-      </c>
-      <c r="G82" s="7" t="inlineStr">
-        <is>
-          <t>scouting@lask.at; 0699 111 879 00</t>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr"/>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>https://fk-austria.at/en/akademie-2/kontakt-2</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
         <is>
-          <t>https://www.lask.at/en/m/ansprechpersonen</t>
+          <t>https://fk-austria.at/en/news/die-sportdirektion-von-austria-wien</t>
         </is>
       </c>
       <c r="I82" s="9" t="n">
@@ -5177,12 +5196,12 @@
       </c>
       <c r="J82" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K82" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Bundesliga. Technical Director: Robert Urbanek</t>
         </is>
       </c>
     </row>
@@ -5194,37 +5213,41 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>SK Sturm Graz</t>
+          <t>LASK</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Emil Bauer</t>
+          <t>Philipp Leeb</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Nachwuchsleiter</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Przyjęcia do akademii</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>emil.bauer@sksturm.at</t>
-        </is>
-      </c>
-      <c r="G83" s="7" t="inlineStr"/>
+          <t>p.leeb@lask.at</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>scouting@lask.at; 0699 111 879 00</t>
+        </is>
+      </c>
       <c r="H83" s="8" t="inlineStr">
         <is>
-          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
+          <t>https://www.lask.at/en/m/ansprechpersonen</t>
         </is>
       </c>
       <c r="I83" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J83" s="7" t="inlineStr">
         <is>
@@ -5250,7 +5273,7 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>Lukas Alterdinger</t>
+          <t>Emil Bauer</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
@@ -5265,7 +5288,7 @@
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>lukas.alterdinger@sksturm.at</t>
+          <t>emil.bauer@sksturm.at</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr"/>
@@ -5301,7 +5324,7 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Christoph Leitgeb</t>
+          <t>Lukas Alterdinger</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
@@ -5316,7 +5339,7 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>christoph.leitgeb@sksturm.at</t>
+          <t>lukas.alterdinger@sksturm.at</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr"/>
@@ -5347,37 +5370,33 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Grazer AK</t>
+          <t>SK Sturm Graz</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>Christian Zach</t>
+          <t>Christoph Leitgeb</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Sportlicher Leiter Akademie</t>
+          <t>Scouting</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Scouting</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
         <is>
-          <t>christian.zach@grazerak.at</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>office@grazerak.at</t>
-        </is>
-      </c>
+          <t>christoph.leitgeb@sksturm.at</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr"/>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t>https://grazerak.at/verein/ansprechpartner-nachwuchs</t>
+          <t>https://sksturm.at/en/c/geschaeftsstelle</t>
         </is>
       </c>
       <c r="I86" s="9" t="n">
@@ -5390,7 +5409,7 @@
       </c>
       <c r="K86" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga. Jugend &amp; Schulkoop.: Philipp Albrecht – philipp.albrecht@grazerak.at</t>
+          <t>Bundesliga</t>
         </is>
       </c>
     </row>
@@ -5402,33 +5421,37 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Wolfsberger AC</t>
+          <t>Grazer AK</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Christian Zach</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sportlicher Leiter Akademie</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
-        </is>
-      </c>
-      <c r="F87" s="7" t="inlineStr"/>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>christian.zach@grazerak.at</t>
+        </is>
+      </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>office@rzpelletswac.at; +43 4352 30688</t>
+          <t>office@grazerak.at</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
         <is>
-          <t>https://rzpelletswac.at/kontakt/</t>
+          <t>https://grazerak.at/verein/ansprechpartner-nachwuchs</t>
         </is>
       </c>
       <c r="I87" s="9" t="n">
@@ -5436,12 +5459,12 @@
       </c>
       <c r="J87" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K87" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga. Brak publicznego maila akademii</t>
+          <t>Bundesliga. Jugend &amp; Schulkoop.: Philipp Albrecht – philipp.albrecht@grazerak.at</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5476,7 @@
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>TSV Hartberg</t>
+          <t>Wolfsberger AC</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
@@ -5463,23 +5486,23 @@
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Hartberg Fußball Akademie</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Kontakt ogólny</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr"/>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>akademie@tsv-hartberg-fussball.at</t>
+          <t>office@rzpelletswac.at; +43 4352 30688</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
         <is>
-          <t>https://tsv-hartberg-fussball.at/nachwuchs/kontakt-nachwuchs/</t>
+          <t>https://rzpelletswac.at/kontakt/</t>
         </is>
       </c>
       <c r="I88" s="9" t="n">
@@ -5487,12 +5510,12 @@
       </c>
       <c r="J88" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K88" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Bundesliga. Brak publicznego maila akademii</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5527,7 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>SV Ried</t>
+          <t>TSV Hartberg</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
@@ -5514,23 +5537,23 @@
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>AKA-Geschäftsstelle</t>
+          <t>Hartberg Fußball Akademie</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>Akademia Ried</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr"/>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>office@akaried.at; +43 7752 88164</t>
+          <t>akademie@tsv-hartberg-fussball.at</t>
         </is>
       </c>
       <c r="H89" s="8" t="inlineStr">
         <is>
-          <t>https://www.svried.at/aka-geschaeftsstelle/</t>
+          <t>https://tsv-hartberg-fussball.at/nachwuchs/kontakt-nachwuchs/</t>
         </is>
       </c>
       <c r="I89" s="9" t="n">
@@ -5555,7 +5578,7 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>WSG Tirol</t>
+          <t>SV Ried</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
@@ -5565,27 +5588,27 @@
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchs</t>
+          <t>AKA-Geschäftsstelle</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>Młodzież, testy</t>
+          <t>Akademia Ried</t>
         </is>
       </c>
       <c r="F90" s="7" t="inlineStr"/>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>jugendfussball@wsg-fussball.at; 0699 108 619 35</t>
+          <t>office@akaried.at; +43 7752 88164</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
         <is>
-          <t>https://www.wsg-fussball.at/de/nachwuchs/infos/</t>
+          <t>https://www.svried.at/aka-geschaeftsstelle/</t>
         </is>
       </c>
       <c r="I90" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
@@ -5606,7 +5629,7 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>SCR Altach</t>
+          <t>WSG Tirol</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
@@ -5616,23 +5639,23 @@
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>SCRA Nachwuchs</t>
+          <t>Nachwuchs</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>Młodzież (największa w Vorarlbergu)</t>
+          <t>Młodzież, testy</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr"/>
-      <c r="G91" s="8" t="inlineStr">
-        <is>
-          <t>https://www.scra.at/teams/nachwuchs/scra-nachwuchs</t>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>jugendfussball@wsg-fussball.at; 0699 108 619 35</t>
         </is>
       </c>
       <c r="H91" s="8" t="inlineStr">
         <is>
-          <t>https://www.scra.at/teams/nachwuchs/scra-nachwuchs</t>
+          <t>https://www.wsg-fussball.at/de/nachwuchs/infos/</t>
         </is>
       </c>
       <c r="I91" s="9" t="n">
@@ -5640,12 +5663,12 @@
       </c>
       <c r="J91" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K91" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga. Brak publicznego maila</t>
+          <t>Bundesliga</t>
         </is>
       </c>
     </row>
@@ -5657,33 +5680,33 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>SC Austria Lustenau</t>
+          <t>SCR Altach</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>Mike Urschitz</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>Sportlicher Nachwuchsleiter</t>
+          <t>SCRA Nachwuchs</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>Młodzież</t>
+          <t>Młodzież (największa w Vorarlbergu)</t>
         </is>
       </c>
       <c r="F92" s="7" t="inlineStr"/>
-      <c r="G92" s="7" t="inlineStr">
-        <is>
-          <t>info@austria-lustenau.at; +43 5577 86250</t>
+      <c r="G92" s="8" t="inlineStr">
+        <is>
+          <t>https://www.scra.at/teams/nachwuchs/scra-nachwuchs</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
         <is>
-          <t>https://www.austria-lustenau.at/kontakt</t>
+          <t>https://www.scra.at/teams/nachwuchs/scra-nachwuchs</t>
         </is>
       </c>
       <c r="I92" s="9" t="n">
@@ -5696,49 +5719,49 @@
       </c>
       <c r="K92" s="7" t="inlineStr">
         <is>
-          <t>Bundesliga (beniaminek). Tel. do osoby: +43 699 19202012</t>
+          <t>Bundesliga. Brak publicznego maila</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>Szwajcaria</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>BSC Young Boys</t>
+          <t>SC Austria Lustenau</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Christian Franke</t>
+          <t>Mike Urschitz</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Technischer Direktor Youth Base</t>
+          <t>Sportlicher Nachwuchsleiter</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>Akademia (U15–U21)</t>
+          <t>Młodzież</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr"/>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>info@bscyb.ch; +41 31 344 88 88</t>
+          <t>info@austria-lustenau.at; +43 5577 86250</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
         <is>
-          <t>https://www.bscyb.ch/youth-base-staff</t>
+          <t>https://www.austria-lustenau.at/kontakt</t>
         </is>
       </c>
       <c r="I93" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J93" s="7" t="inlineStr">
         <is>
@@ -5747,7 +5770,7 @@
       </c>
       <c r="K93" s="7" t="inlineStr">
         <is>
-          <t>Super League</t>
+          <t>Bundesliga (beniaminek). Tel. do osoby: +43 699 19202012</t>
         </is>
       </c>
     </row>
@@ -5759,33 +5782,33 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>FC Basel</t>
+          <t>BSC Young Boys</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>Timo Jankowski</t>
+          <t>Christian Franke</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>Leiter Nachwuchs</t>
+          <t>Technischer Direktor Youth Base</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchs-Campus</t>
+          <t>Akademia (U15–U21)</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr"/>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>info@fcb.ch; 061 375 10 10</t>
+          <t>info@bscyb.ch; +41 31 344 88 88</t>
         </is>
       </c>
       <c r="H94" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcb.ch/aktuell/news/nachwuchs/veraenderungen-auf-dem-campus-januar-2026</t>
+          <t>https://www.bscyb.ch/youth-base-staff</t>
         </is>
       </c>
       <c r="I94" s="9" t="n">
@@ -5798,7 +5821,7 @@
       </c>
       <c r="K94" s="7" t="inlineStr">
         <is>
-          <t>Super League. Administracja Campusu: danique.stein@nachwuchs-campus.ch</t>
+          <t>Super League</t>
         </is>
       </c>
     </row>
@@ -5810,37 +5833,33 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>FC Zürich</t>
+          <t>FC Basel</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Balz Rau</t>
+          <t>Timo Jankowski</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Koordinator Nachwuchsscouting</t>
+          <t>Leiter Nachwuchs</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Scouting młodzieżowy</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>balz.rau@fcz.ch</t>
-        </is>
-      </c>
+          <t>Nachwuchs-Campus</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr"/>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>+41 43 521 12 12</t>
+          <t>info@fcb.ch; 061 375 10 10</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcz.ch/pages/leitung-und-staff</t>
+          <t>https://www.fcb.ch/aktuell/news/nachwuchs/veraenderungen-auf-dem-campus-januar-2026</t>
         </is>
       </c>
       <c r="I95" s="9" t="n">
@@ -5848,12 +5867,12 @@
       </c>
       <c r="J95" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K95" s="7" t="inlineStr">
         <is>
-          <t>Super League. Ausbildungschef: Sascha Milicevic; Techn. Leiter: Claudio Calvi</t>
+          <t>Super League. Administracja Campusu: danique.stein@nachwuchs-campus.ch</t>
         </is>
       </c>
     </row>
@@ -5865,37 +5884,37 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>FC Thun</t>
+          <t>FC Zürich</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>Jürg Frey</t>
+          <t>Balz Rau</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Leiter Nachwuchs</t>
+          <t>Koordinator Nachwuchsscouting</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>Młodzież</t>
+          <t>Scouting młodzieżowy</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
-          <t>juerg.frey@fcthun.ch</t>
+          <t>balz.rau@fcz.ch</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>033 225 18 98; info@fcthun.ch</t>
+          <t>+41 43 521 12 12</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcthun.ch/de/teams/nachwuchs</t>
+          <t>https://www.fcz.ch/pages/leitung-und-staff</t>
         </is>
       </c>
       <c r="I96" s="9" t="n">
@@ -5908,7 +5927,7 @@
       </c>
       <c r="K96" s="7" t="inlineStr">
         <is>
-          <t>Super League – aktualny mistrz Szwajcarii</t>
+          <t>Super League. Ausbildungschef: Sascha Milicevic; Techn. Leiter: Claudio Calvi</t>
         </is>
       </c>
     </row>
@@ -5920,33 +5939,37 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>FC Lugano</t>
+          <t>FC Thun</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>Roman Hangarter</t>
+          <t>Jürg Frey</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Direttore Academy</t>
+          <t>Leiter Nachwuchs</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>Akademia + Partenariato Ticino (od 26/27)</t>
-        </is>
-      </c>
-      <c r="F97" s="7" t="inlineStr"/>
+          <t>Młodzież</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>juerg.frey@fcthun.ch</t>
+        </is>
+      </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>+41 91 922 86 72</t>
+          <t>033 225 18 98; info@fcthun.ch</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t>https://fclugano.com/en/academy/</t>
+          <t>https://www.fcthun.ch/de/teams/nachwuchs</t>
         </is>
       </c>
       <c r="I97" s="9" t="n">
@@ -5954,12 +5977,12 @@
       </c>
       <c r="J97" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K97" s="7" t="inlineStr">
         <is>
-          <t>Super League. Chief Sports Officer: Sebastian Pelzer</t>
+          <t>Super League – aktualny mistrz Szwajcarii</t>
         </is>
       </c>
     </row>
@@ -5971,33 +5994,33 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>FC Lausanne-Sport</t>
+          <t>FC Lugano</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>Massimo Ceccaroni</t>
+          <t>Roman Hangarter</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Directeur Technique Académie</t>
+          <t>Direttore Academy</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Akademia + Partenariato Ticino (od 26/27)</t>
         </is>
       </c>
       <c r="F98" s="7" t="inlineStr"/>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>+41 21 641 05 30</t>
+          <t>+41 91 922 86 72</t>
         </is>
       </c>
       <c r="H98" s="8" t="inlineStr">
         <is>
-          <t>https://www.lausanne-sport.ch/contact/</t>
+          <t>https://fclugano.com/en/academy/</t>
         </is>
       </c>
       <c r="I98" s="9" t="n">
@@ -6010,7 +6033,7 @@
       </c>
       <c r="K98" s="7" t="inlineStr">
         <is>
-          <t>Super League</t>
+          <t>Super League. Chief Sports Officer: Sebastian Pelzer</t>
         </is>
       </c>
     </row>
@@ -6022,50 +6045,46 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>FC Vaduz</t>
+          <t>FC Lausanne-Sport</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>Lorenz Gassner</t>
+          <t>Massimo Ceccaroni</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Leiter Nachwuchs</t>
+          <t>Directeur Technique Académie</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>Młodzież</t>
-        </is>
-      </c>
-      <c r="F99" s="7" t="inlineStr">
-        <is>
-          <t>lorenz.gassner@fcvaduz.li</t>
-        </is>
-      </c>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr"/>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>+41 78 773 76 13; info@fcvaduz.li</t>
+          <t>+41 21 641 05 30</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcvaduz.li/kontakt</t>
+          <t>https://www.lausanne-sport.ch/contact/</t>
         </is>
       </c>
       <c r="I99" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J99" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K99" s="7" t="inlineStr">
         <is>
-          <t>Super League (beniaminek)</t>
+          <t>Super League</t>
         </is>
       </c>
     </row>
@@ -6077,33 +6096,37 @@
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>FC St. Gallen</t>
+          <t>FC Vaduz</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>David Garcia</t>
+          <t>Lorenz Gassner</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Academy Director – Future Champs Ostschweiz</t>
+          <t>Leiter Nachwuchs</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>Akademia regionu Ostschweiz</t>
-        </is>
-      </c>
-      <c r="F100" s="7" t="inlineStr"/>
+          <t>Młodzież</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>lorenz.gassner@fcvaduz.li</t>
+        </is>
+      </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>info@futurechamps.ch; +41 71 314 14 14</t>
+          <t>+41 78 773 76 13; info@fcvaduz.li</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcsg.ch/future-champs/organisation/kontakt/</t>
+          <t>https://www.fcvaduz.li/kontakt</t>
         </is>
       </c>
       <c r="I100" s="9" t="n">
@@ -6111,12 +6134,12 @@
       </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K100" s="7" t="inlineStr">
         <is>
-          <t>Super League</t>
+          <t>Super League (beniaminek)</t>
         </is>
       </c>
     </row>
@@ -6128,33 +6151,33 @@
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>Servette FC</t>
+          <t>FC St. Gallen</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>David Garcia</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Académie SFC</t>
+          <t>Academy Director – Future Champs Ostschweiz</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Akademia regionu Ostschweiz</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr"/>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>tel. +41 22 340 54 74</t>
+          <t>info@futurechamps.ch; +41 71 314 14 14</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
         <is>
-          <t>https://servettefc.ch/academie/je-veux-jouer-au-sfc/</t>
+          <t>https://www.fcsg.ch/future-champs/organisation/kontakt/</t>
         </is>
       </c>
       <c r="I101" s="9" t="n">
@@ -6179,17 +6202,17 @@
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>FC Sion</t>
+          <t>Servette FC</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>Xavier Henriques</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>Coordinateur Académie/Formation</t>
+          <t>Académie SFC</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
@@ -6200,12 +6223,12 @@
       <c r="F102" s="7" t="inlineStr"/>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>secretariat@fcsion.ch; 027 747 13 13</t>
+          <t>tel. +41 22 340 54 74</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcsion.ch/fr/administration/</t>
+          <t>https://servettefc.ch/academie/je-veux-jouer-au-sfc/</t>
         </is>
       </c>
       <c r="I102" s="9" t="n">
@@ -6230,33 +6253,33 @@
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>FC Luzern</t>
+          <t>FC Sion</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Xavier Henriques</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchs</t>
+          <t>Coordinateur Académie/Formation</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>Młodzież</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F103" s="7" t="inlineStr"/>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>kontakt@fcl-verein.ch; 0848 317 000</t>
+          <t>secretariat@fcsion.ch; 027 747 13 13</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>https://fcl.ch/role/nachwuchs/</t>
+          <t>https://www.fcsion.ch/fr/administration/</t>
         </is>
       </c>
       <c r="I103" s="9" t="n">
@@ -6269,7 +6292,7 @@
       </c>
       <c r="K103" s="7" t="inlineStr">
         <is>
-          <t>Super League. Brak publicznego maila akademii</t>
+          <t>Super League</t>
         </is>
       </c>
     </row>
@@ -6281,7 +6304,7 @@
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Grasshopper Club Zürich</t>
+          <t>FC Luzern</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
@@ -6291,23 +6314,23 @@
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>Nachwuchs / GC Campus</t>
+          <t>Nachwuchs</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Młodzież</t>
         </is>
       </c>
       <c r="F104" s="7" t="inlineStr"/>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>info@gcz.ch; +41 44 447 46 46</t>
+          <t>kontakt@fcl-verein.ch; 0848 317 000</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>https://www.gcz.ch/kontakt/</t>
+          <t>https://fcl.ch/role/nachwuchs/</t>
         </is>
       </c>
       <c r="I104" s="9" t="n">
@@ -6320,19 +6343,19 @@
       </c>
       <c r="K104" s="7" t="inlineStr">
         <is>
-          <t>Super League</t>
+          <t>Super League. Brak publicznego maila akademii</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>Portugalia</t>
+          <t>Szwajcaria</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>SL Benfica</t>
+          <t>Grasshopper Club Zürich</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
@@ -6342,27 +6365,27 @@
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>Departamento de Scouting e Avaliação de Jogadores</t>
+          <t>Nachwuchs / GC Campus</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>Scouting U10–U19 (bez otwartych testów)</t>
+          <t>Kontakt ogólny</t>
         </is>
       </c>
       <c r="F105" s="7" t="inlineStr"/>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>formularz: slbenfica.pt/en-us/apoio/contactos</t>
+          <t>info@gcz.ch; +41 44 447 46 46</t>
         </is>
       </c>
       <c r="H105" s="8" t="inlineStr">
         <is>
-          <t>https://www.slbenfica.pt/en-us/futebol-formacao/formacao/prospecao/recrutamento-jogadores</t>
+          <t>https://www.gcz.ch/kontakt/</t>
         </is>
       </c>
       <c r="I105" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J105" s="7" t="inlineStr">
         <is>
@@ -6371,7 +6394,7 @@
       </c>
       <c r="K105" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: nr 1 na świecie wg przychodów ze sprzedaży wychowanków (589 mln € / 10 lat); 73 wychowanków w 31 ligach UEFA (2. miejsce)</t>
+          <t>Super League</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6406,7 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>Sporting CP</t>
+          <t>SL Benfica</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -6393,23 +6416,23 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>Academia Cristiano Ronaldo</t>
+          <t>Departamento de Scouting e Avaliação de Jogadores</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii (Alcochete)</t>
+          <t>Scouting U10–U19 (bez otwartych testów)</t>
         </is>
       </c>
       <c r="F106" s="7" t="inlineStr"/>
-      <c r="G106" s="8" t="inlineStr">
-        <is>
-          <t>https://escolasacademia.sporting.pt</t>
+      <c r="G106" s="7" t="inlineStr">
+        <is>
+          <t>formularz: slbenfica.pt/en-us/apoio/contactos</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Academia_Cristiano_Ronaldo</t>
+          <t>https://www.slbenfica.pt/en-us/futebol-formacao/formacao/prospecao/recrutamento-jogadores</t>
         </is>
       </c>
       <c r="I106" s="9" t="n">
@@ -6422,7 +6445,7 @@
       </c>
       <c r="K106" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: 3. miejsce w Training Index; najlepsza akademia spoza Big-5 wg wychowanków w Big-5 (24); top 10 dochodów ze sprzedaży</t>
+          <t>CIES 2026: nr 1 na świecie wg przychodów ze sprzedaży wychowanków (589 mln € / 10 lat); 73 wychowanków w 31 ligach UEFA (2. miejsce)</t>
         </is>
       </c>
     </row>
@@ -6434,33 +6457,33 @@
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Sporting CP</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>Nelson Oliveira</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>Head of Recruitment</t>
+          <t>Academia Cristiano Ronaldo</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>Scouting – zgłaszanie zawodników</t>
+          <t>Scouting akademii (Alcochete)</t>
         </is>
       </c>
       <c r="F107" s="7" t="inlineStr"/>
-      <c r="G107" s="7" t="inlineStr">
-        <is>
-          <t>geral.scouting@fcporto.pt</t>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
+          <t>https://escolasacademia.sporting.pt</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcporto.pt/pt/contactos</t>
+          <t>https://en.wikipedia.org/wiki/Academia_Cristiano_Ronaldo</t>
         </is>
       </c>
       <c r="I107" s="9" t="n">
@@ -6468,50 +6491,50 @@
       </c>
       <c r="J107" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K107" s="7" t="inlineStr">
         <is>
-          <t>Oficjalny adres działu scoutingu do przesyłania informacji o zawodnikach. Uznana akademia sprzedażowa (poza top 10 CIES)</t>
+          <t>CIES 2026: 3. miejsce w Training Index; najlepsza akademia spoza Big-5 wg wychowanków w Big-5 (24); top 10 dochodów ze sprzedaży</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>Holandia</t>
+          <t>Portugalia</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>Kelvin de Lang</t>
+          <t>Nelson Oliveira</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting &amp; Recruitment, Academy De Toekomst</t>
+          <t>Head of Recruitment</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii</t>
+          <t>Scouting – zgłaszanie zawodników</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr"/>
-      <c r="G108" s="8" t="inlineStr">
-        <is>
-          <t>https://www.ajax.nl/club/jeugdopleiding</t>
+      <c r="G108" s="7" t="inlineStr">
+        <is>
+          <t>geral.scouting@fcporto.pt</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
         <is>
-          <t>https://www.ajax.nl/artikelen/ajax-doc-scouten-voor-de-toekomst</t>
+          <t>https://www.fcporto.pt/pt/contactos</t>
         </is>
       </c>
       <c r="I108" s="9" t="n">
@@ -6519,12 +6542,12 @@
       </c>
       <c r="J108" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K108" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: nr 1 w Europie – 85 wychowanków w 31 ligach UEFA, 1. miejsce Training Index; 2. na świecie w sprzedaży wychowanków (454 mln €)</t>
+          <t>Oficjalny adres działu scoutingu do przesyłania informacji o zawodnikach. Uznana akademia sprzedażowa (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
@@ -6536,37 +6559,37 @@
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>Rini de Groot</t>
+          <t>Kelvin de Lang</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>Hoofd jeugdscouting</t>
+          <t>Head of Scouting &amp; Recruitment, Academy De Toekomst</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii (De Herdgang)</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr"/>
-      <c r="G109" s="7" t="inlineStr">
-        <is>
-          <t>Oirschotsedijk 12a, 5651 GC Eindhoven</t>
+      <c r="G109" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ajax.nl/club/jeugdopleiding</t>
         </is>
       </c>
       <c r="H109" s="8" t="inlineStr">
         <is>
-          <t>https://www.psv.nl/en/club/psv-campus-de-herdgang-1/psv-campus</t>
+          <t>https://www.ajax.nl/artikelen/ajax-doc-scouten-voor-de-toekomst</t>
         </is>
       </c>
       <c r="I109" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J109" s="7" t="inlineStr">
         <is>
@@ -6575,7 +6598,7 @@
       </c>
       <c r="K109" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting klubu: Jan Vennegoor of Hesselink. Uznana akademia (poza top 10 CIES)</t>
+          <t>CIES 2026: nr 1 w Europie – 85 wychowanków w 31 ligach UEFA, 1. miejsce Training Index; 2. na świecie w sprzedaży wychowanków (454 mln €)</t>
         </is>
       </c>
     </row>
@@ -6587,37 +6610,33 @@
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>Feyenoord</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>Ricardo Kern</t>
+          <t>Rini de Groot</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>Coördinator wedstrijdzaken Feyenoord Academy</t>
+          <t>Hoofd jeugdscouting</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>Scouting / sprawy drużyn akademii</t>
-        </is>
-      </c>
-      <c r="F110" s="7" t="inlineStr">
-        <is>
-          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
-        </is>
-      </c>
+          <t>Scouting akademii (De Herdgang)</t>
+        </is>
+      </c>
+      <c r="F110" s="7" t="inlineStr"/>
       <c r="G110" s="7" t="inlineStr">
         <is>
-          <t>Olympiaweg 280, 3078 HT Rotterdam</t>
+          <t>Oirschotsedijk 12a, 5651 GC Eindhoven</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
         <is>
-          <t>https://www.feyenoord.com/nl/academy/contact</t>
+          <t>https://www.psv.nl/en/club/psv-campus-de-herdgang-1/psv-campus</t>
         </is>
       </c>
       <c r="I110" s="9" t="n">
@@ -6630,7 +6649,7 @@
       </c>
       <c r="K110" s="7" t="inlineStr">
         <is>
-          <t>Uznana akademia (poza top 10 CIES)</t>
+          <t>Head of Scouting klubu: Jan Vennegoor of Hesselink. Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
@@ -6642,33 +6661,37 @@
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>AZ Alkmaar</t>
+          <t>Feyenoord</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ricardo Kern</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>AZ Jeugdopleiding</t>
+          <t>Coördinator wedstrijdzaken Feyenoord Academy</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>Akademia, dni selekcji U8–U13</t>
-        </is>
-      </c>
-      <c r="F111" s="7" t="inlineStr"/>
-      <c r="G111" s="8" t="inlineStr">
-        <is>
-          <t>https://www.az.nl/jeugdopleiding</t>
+          <t>Scouting / sprawy drużyn akademii</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G111" s="7" t="inlineStr">
+        <is>
+          <t>Olympiaweg 280, 3078 HT Rotterdam</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>https://www.az.nl/jeugdopleiding/az-voetbalschool</t>
+          <t>https://www.feyenoord.com/nl/academy/contact</t>
         </is>
       </c>
       <c r="I111" s="9" t="n">
@@ -6688,12 +6711,12 @@
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>Hiszpania</t>
+          <t>Holandia</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>AZ Alkmaar</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
@@ -6703,23 +6726,23 @@
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>Zubieta (cantera)</t>
+          <t>AZ Jeugdopleiding</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>Akademia – głównie talenty z Gipuzkoa</t>
+          <t>Akademia, dni selekcji U8–U13</t>
         </is>
       </c>
       <c r="F112" s="7" t="inlineStr"/>
-      <c r="G112" s="7" t="inlineStr">
-        <is>
-          <t>realsociedad.eus</t>
+      <c r="G112" s="8" t="inlineStr">
+        <is>
+          <t>https://www.az.nl/jeugdopleiding</t>
         </is>
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Real_Sociedad_Cantera</t>
+          <t>https://www.az.nl/jeugdopleiding/az-voetbalschool</t>
         </is>
       </c>
       <c r="I112" s="9" t="n">
@@ -6732,7 +6755,7 @@
       </c>
       <c r="K112" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: top 10 w Europie wg wychowanków w Big-5</t>
+          <t>Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6767,7 @@
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Villarreal CF</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
@@ -6754,23 +6777,23 @@
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>Cantera Grogueta</t>
+          <t>Zubieta (cantera)</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>Akademia (36 drużyn, ~650 zawodników)</t>
+          <t>Akademia – głównie talenty z Gipuzkoa</t>
         </is>
       </c>
       <c r="F113" s="7" t="inlineStr"/>
       <c r="G113" s="7" t="inlineStr">
         <is>
-          <t>formularz: villarrealcf.es/en/formulario-contacto/</t>
+          <t>realsociedad.eus</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>https://villarrealcf.es/es/cantera-grogueta/</t>
+          <t>https://en.wikipedia.org/wiki/Real_Sociedad_Cantera</t>
         </is>
       </c>
       <c r="I113" s="9" t="n">
@@ -6783,7 +6806,7 @@
       </c>
       <c r="K113" s="7" t="inlineStr">
         <is>
-          <t>Bez otwartych testów dla chłopców. Uznana akademia (poza top 10 CIES)</t>
+          <t>CIES 2026: top 10 w Europie wg wychowanków w Big-5</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6818,7 @@
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>Valencia CF</t>
+          <t>Villarreal CF</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
@@ -6805,23 +6828,23 @@
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>Academia VCF (Paterna)</t>
+          <t>Cantera Grogueta</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Akademia (36 drużyn, ~650 zawodników)</t>
         </is>
       </c>
       <c r="F114" s="7" t="inlineStr"/>
-      <c r="G114" s="8" t="inlineStr">
-        <is>
-          <t>https://formacion.valenciacf.com/en/contacto/</t>
+      <c r="G114" s="7" t="inlineStr">
+        <is>
+          <t>formularz: villarrealcf.es/en/formulario-contacto/</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
         <is>
-          <t>https://www.valenciacf.com/vcf-academy</t>
+          <t>https://villarrealcf.es/es/cantera-grogueta/</t>
         </is>
       </c>
       <c r="I114" s="9" t="n">
@@ -6834,74 +6857,70 @@
       </c>
       <c r="K114" s="7" t="inlineStr">
         <is>
-          <t>Wg klubu: 4. najlepsza akademia w Europie (ranking CIES)</t>
+          <t>Bez otwartych testów dla chłopców. Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>Niemcy</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>Bayer 04 Leverkusen</t>
+          <t>Valencia CF</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>Jennifer Weber</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>Geschäftsstelle Nachwuchsabteilung (NLZ)</t>
+          <t>Academia VCF (Paterna)</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>Biuro akademii, testy tylko przez e-mail</t>
-        </is>
-      </c>
-      <c r="F115" s="7" t="inlineStr">
-        <is>
-          <t>Jennifer.Weber@bayer04.de</t>
-        </is>
-      </c>
-      <c r="G115" s="7" t="inlineStr">
-        <is>
-          <t>tel. 0214 866 03 43</t>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr"/>
+      <c r="G115" s="8" t="inlineStr">
+        <is>
+          <t>https://formacion.valenciacf.com/en/contacto/</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>https://www.bayer04.de/en-us/page/youth/trial-sessions</t>
+          <t>https://www.valenciacf.com/vcf-academy</t>
         </is>
       </c>
       <c r="I115" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J115" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K115" s="7" t="inlineStr">
         <is>
-          <t>CIES: top 10 dochodów ze sprzedaży wychowanków (10 lat). Mail z organigramu NLZ – sprawdzić aktualność</t>
+          <t>Wg klubu: 4. najlepsza akademia w Europie (ranking CIES)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>Chorwacja</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t>GNK Dinamo Zagreb</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
@@ -6911,27 +6930,27 @@
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>Dinamo Akademija</t>
+          <t>Lezama (cantera)</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Akademia – tylko zawodnicy z korzeniami baskijskimi</t>
         </is>
       </c>
       <c r="F116" s="7" t="inlineStr"/>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>dinamo@gnkdinamo.hr; 01 238 6111</t>
+          <t>Barrio Garaioltza 147, 48196 Lezama; https://www.athletic-club.eus/en/contact/</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
         <is>
-          <t>https://gnkdinamo.hr/hr/info/kontakt</t>
+          <t>https://www.athletic-club.eus/en/teams/lezama/</t>
         </is>
       </c>
       <c r="I116" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J116" s="7" t="inlineStr">
         <is>
@@ -6940,19 +6959,19 @@
       </c>
       <c r="K116" s="7" t="inlineStr">
         <is>
-          <t>Czołowa akademia sprzedażowa regionu (poza top 10 CIES 2026)</t>
+          <t>CIES MR99: 7. miejsce wg minut wychowanków w Big-5 (20 lat). Rekrutacja ograniczona do Kraju Basków</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>FK Partizan</t>
+          <t>FC Barcelona</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
@@ -6962,7 +6981,7 @@
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>Omladinska škola</t>
+          <t>La Masia</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
@@ -6971,18 +6990,18 @@
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr"/>
-      <c r="G117" s="8" t="inlineStr">
-        <is>
-          <t>https://partizan.rs/en</t>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>oab@fcbarcelona.cat (informacja ogólna)</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>http://www.en.partizan.rs/omladinska-skola-fudbala/</t>
+          <t>https://www.fcbarcelona.com/en/club/identity/la-masia</t>
         </is>
       </c>
       <c r="I117" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J117" s="7" t="inlineStr">
         <is>
@@ -6991,49 +7010,49 @@
       </c>
       <c r="K117" s="7" t="inlineStr">
         <is>
-          <t>CIES: wcześniej nr 1 rocznego rankingu akademii (przed Ajaxem)</t>
+          <t>CIES MR99: 2. miejsce – 156 wychowanków w Big-5 (20 lat). barcaescola@fcbarcelona.cat to szkółka FCBEscola, nie scouting</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t>FK Crvena zvezda</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Juni Calafat</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>Omladinska škola</t>
+          <t>Chief Scout</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Scouting (głównie 1. zespół)</t>
         </is>
       </c>
       <c r="F118" s="7" t="inlineStr"/>
-      <c r="G118" s="8" t="inlineStr">
-        <is>
-          <t>https://www.crvenazvezdafk.com/en/klub/kontakt-i-lokacija</t>
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>realmadrid.com – sekcja cantera</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr">
         <is>
-          <t>https://www.crvenazvezdafk.com/en/vesti-kategorija/omladinska-shkola</t>
+          <t>https://en.wikipedia.org/wiki/Juni_Calafat</t>
         </is>
       </c>
       <c r="I118" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J118" s="7" t="inlineStr">
         <is>
@@ -7042,64 +7061,323 @@
       </c>
       <c r="K118" s="7" t="inlineStr">
         <is>
-          <t>Uznana akademia (poza top 10 CIES)</t>
+          <t>CIES MR99: 1. miejsce – 166 wychowanków w Big-5 (20 lat), 103 w 55 ligach. Brak publicznego kontaktu scoutingu</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
         <is>
+          <t>Niemcy</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>Bayer 04 Leverkusen</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>Jennifer Weber</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>Geschäftsstelle Nachwuchsabteilung (NLZ)</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>Biuro akademii, testy tylko przez e-mail</t>
+        </is>
+      </c>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>Jennifer.Weber@bayer04.de</t>
+        </is>
+      </c>
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>tel. 0214 866 03 43</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="inlineStr">
+        <is>
+          <t>https://www.bayer04.de/en-us/page/youth/trial-sessions</t>
+        </is>
+      </c>
+      <c r="I119" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J119" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K119" s="7" t="inlineStr">
+        <is>
+          <t>CIES: top 10 dochodów ze sprzedaży wychowanków (10 lat). Mail z organigramu NLZ – sprawdzić aktualność</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>GNK Dinamo Zagreb</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>Dinamo Akademija</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F120" s="7" t="inlineStr"/>
+      <c r="G120" s="7" t="inlineStr">
+        <is>
+          <t>dinamo@gnkdinamo.hr; 01 238 6111</t>
+        </is>
+      </c>
+      <c r="H120" s="8" t="inlineStr">
+        <is>
+          <t>https://gnkdinamo.hr/hr/info/kontakt</t>
+        </is>
+      </c>
+      <c r="I120" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J120" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K120" s="7" t="inlineStr">
+        <is>
+          <t>Czołowa akademia sprzedażowa regionu (poza top 10 CIES 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>FK Partizan</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Omladinska škola</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr"/>
+      <c r="G121" s="8" t="inlineStr">
+        <is>
+          <t>https://partizan.rs/en</t>
+        </is>
+      </c>
+      <c r="H121" s="8" t="inlineStr">
+        <is>
+          <t>http://www.en.partizan.rs/omladinska-skola-fudbala/</t>
+        </is>
+      </c>
+      <c r="I121" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J121" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K121" s="7" t="inlineStr">
+        <is>
+          <t>CIES: wcześniej nr 1 rocznego rankingu akademii (przed Ajaxem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>FK Crvena zvezda</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t>Omladinska škola</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr"/>
+      <c r="G122" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crvenazvezdafk.com/en/klub/kontakt-i-lokacija</t>
+        </is>
+      </c>
+      <c r="H122" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crvenazvezdafk.com/en/vesti-kategorija/omladinska-shkola</t>
+        </is>
+      </c>
+      <c r="I122" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J122" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K122" s="7" t="inlineStr">
+        <is>
+          <t>Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
           <t>Ukraina</t>
         </is>
       </c>
-      <c r="B119" s="7" t="inlineStr">
+      <c r="B123" s="7" t="inlineStr">
         <is>
           <t>Dynamo Kijów</t>
         </is>
       </c>
-      <c r="C119" s="7" t="inlineStr">
+      <c r="C123" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D119" s="7" t="inlineStr">
+      <c r="D123" s="7" t="inlineStr">
         <is>
           <t>Dział scoutingu</t>
         </is>
       </c>
-      <c r="E119" s="7" t="inlineStr">
+      <c r="E123" s="7" t="inlineStr">
         <is>
           <t>Scouting</t>
         </is>
       </c>
-      <c r="F119" s="7" t="inlineStr"/>
-      <c r="G119" s="7" t="inlineStr">
+      <c r="F123" s="7" t="inlineStr"/>
+      <c r="G123" s="7" t="inlineStr">
         <is>
           <t>tel. +38 044 278 06 28</t>
         </is>
       </c>
-      <c r="H119" s="8" t="inlineStr">
+      <c r="H123" s="8" t="inlineStr">
         <is>
           <t>https://fcdynamo.com/en/pages/contacts</t>
         </is>
       </c>
-      <c r="I119" s="9" t="n">
+      <c r="I123" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J119" s="7" t="inlineStr">
+      <c r="J123" s="7" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K119" s="7" t="inlineStr">
+      <c r="K123" s="7" t="inlineStr">
         <is>
           <t>CIES 2026: 3. miejsce w Europie – 72 wychowanków w 31 ligach UEFA. Uwaga: sytuacja wojenna</t>
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>Anglia</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t>David Harrison</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="inlineStr">
+        <is>
+          <t>Head of Academy Recruitment</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr"/>
+      <c r="G124" s="7" t="inlineStr">
+        <is>
+          <t>Carrington Training Complex, Birch Road, Manchester M31 4BH</t>
+        </is>
+      </c>
+      <c r="H124" s="8" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/help/faqs/club-information2</t>
+        </is>
+      </c>
+      <c r="I124" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J124" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K124" s="7" t="inlineStr">
+        <is>
+          <t>CIES MR99: 103 wychowanków w Big-5 (20 lat), top 10 wg minut. Nazwisko ze źródła nieoficjalnego – potwierdzić</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K119"/>
-  <conditionalFormatting sqref="A2:K119">
+  <autoFilter ref="A1:K124"/>
+  <conditionalFormatting sqref="A2:K124">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Zweryfikowany"</formula>
     </cfRule>
@@ -7107,13 +7385,13 @@
       <formula>$J2="Do potwierdzenia"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I119">
+  <conditionalFormatting sqref="I2:I124">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>$I2=1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Zweryfikowany,Częściowo – brak maila osoby,Do potwierdzenia"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7180,76 +7458,82 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId138"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7478,7 +7762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -8005,15 +8289,265 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>MR99 (II 2025): wychowankowie w Big-5, 20 lat</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>166 zawodników</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Źródła: CIES Football Observatory – Weekly Post 529 (training clubs), Weekly Post 540 (most profitable academies), 2026. football-observatory.com</t>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>MR99 (II 2025): wychowankowie w Big-5, 20 lat</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>FC Barcelona</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Hiszpania</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>MR99 (II 2025): wychowankowie w Big-5, 20 lat</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Francja</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>MR99 (II 2025): wychowankowie w Big-5, 20 lat</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>4–5</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Olympique Lyonnais, Manchester United</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Francja/Anglia</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>po 103</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>MR99 (II 2025): wychowankowie w Big-5, 20 lat</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>6–7</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Stade Rennais, Atalanta</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Francja/Włochy</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>po 94</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>MR99 (II 2025): minuty wychowanków w Big-5, 20 lat</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>top 10</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Real Madrid (1), Barcelona (2), Lyon, PSG, Rennes, Man. United, Athletic Club (7), Atalanta, Real Sociedad (9), Valencia (10)</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Wszystkie w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w 55 ligach (VI 2025)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Real Madrid 103, Benfica 102, Barcelona 94</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>W arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Wychowankowie w 55 ligach (VI 2025)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>4–10</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Ajax, Sporting CP, River Plate, Defensor, Crvena zvezda, Dinamo Zagreb, Boca Juniors</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Europejskie kluby w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Źródła: CIES Football Observatory – Weekly Post 529 (training clubs), Weekly Post 540 (most profitable academies), 2026; Monthly Report 99 (II 2025). football-observatory.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dodatkowe akademie aktywnie scoutujace: Norwegia, Niemcy, Holandia, Chorwacja, Slowenia, Slowacja, Czechy, Braga
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Be8XiCwvE6GnhZjaxWth9
</commit_message>
<xml_diff>
--- a/Kluby_Europa_Kontakty_Scouting.xlsx
+++ b/Kluby_Europa_Kontakty_Scouting.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Ranking CIES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Beşiktaş – korekta'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ranking CIES'!$A$1:$F$32</definedName>
   </definedNames>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A2)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A2)</f>
         <v/>
       </c>
       <c r="C2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A2,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A2,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A2,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A2,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A2,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A2,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -573,19 +573,19 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A3)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A3)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A3,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A3,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A3,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A3,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A3,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A3,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -596,19 +596,19 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A4)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A4)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A4,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A4,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A4,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A4,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A4,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A4,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -619,19 +619,19 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A5)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A5)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A5,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A5,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A5,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A5,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A5,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A5,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -642,19 +642,19 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A6)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A6)</f>
         <v/>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A6,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A6,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A6,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A6,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A6,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A6,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -665,19 +665,19 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A7)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A7)</f>
         <v/>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A7,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A7,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A7,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A7,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A7,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A7,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -688,19 +688,19 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A8)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A8)</f>
         <v/>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A8,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A8,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A8,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A8,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A8,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A8,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -711,19 +711,19 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A9)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A9)</f>
         <v/>
       </c>
       <c r="C9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A9,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A9,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A9,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A9,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A9,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A9,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -734,19 +734,19 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A10)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A10)</f>
         <v/>
       </c>
       <c r="C10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A10,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A10,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A10,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A10,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A10,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A10,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -757,19 +757,19 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A11)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A11)</f>
         <v/>
       </c>
       <c r="C11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A11,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A11,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A11,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A11,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A11,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A11,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -780,19 +780,19 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A12)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A12)</f>
         <v/>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A12,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A12,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A12,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A12,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A12,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A12,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A13)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A13)</f>
         <v/>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A13,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A13,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A13,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A13,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A13,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A13,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A14)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A14)</f>
         <v/>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A14,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A14,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A14,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A14,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A14,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A14,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -849,19 +849,19 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A15)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A15)</f>
         <v/>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A15,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A15,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A15,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A15,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A15,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A15,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -872,19 +872,19 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A16)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A16)</f>
         <v/>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A16,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A16,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D16" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A16,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A16,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E16" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A16,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A16,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -895,103 +895,172 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$129,A17)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A17)</f>
         <v/>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A17,Kontakty!$F$2:$F$129,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A17,Kontakty!$F$2:$F$148,"*@*")</f>
         <v/>
       </c>
       <c r="D17" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A17,Kontakty!$I$2:$I$129,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A17,Kontakty!$I$2:$I$148,1)</f>
         <v/>
       </c>
       <c r="E17" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$129,A17,Kontakty!$J$2:$J$129,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A17,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A18)</f>
+        <v/>
+      </c>
+      <c r="C18" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A18,Kontakty!$F$2:$F$148,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D18" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A18,Kontakty!$I$2:$I$148,1)</f>
+        <v/>
+      </c>
+      <c r="E18" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A18,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Słowacja</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A19)</f>
+        <v/>
+      </c>
+      <c r="C19" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A19,Kontakty!$F$2:$F$148,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D19" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A19,Kontakty!$I$2:$I$148,1)</f>
+        <v/>
+      </c>
+      <c r="E19" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A19,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Słowenia</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$148,A20)</f>
+        <v/>
+      </c>
+      <c r="C20" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A20,Kontakty!$F$2:$F$148,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D20" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A20,Kontakty!$I$2:$I$148,1)</f>
+        <v/>
+      </c>
+      <c r="E20" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$148,A20,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>RAZEM</t>
         </is>
       </c>
-      <c r="B18" s="3">
-        <f>SUM(B2:B17)</f>
+      <c r="B21" s="3">
+        <f>SUM(B2:B20)</f>
         <v/>
       </c>
-      <c r="C18" s="3">
-        <f>SUM(C2:C17)</f>
+      <c r="C21" s="3">
+        <f>SUM(C2:C20)</f>
         <v/>
       </c>
-      <c r="D18" s="3">
-        <f>SUM(D2:D17)</f>
+      <c r="D21" s="3">
+        <f>SUM(D2:D20)</f>
         <v/>
       </c>
-      <c r="E18" s="3">
-        <f>SUM(E2:E17)</f>
+      <c r="E21" s="3">
+        <f>SUM(E2:E20)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Legenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
+          <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
+          <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
+          <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+          <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Stan na: 26.09.2026. Stanowiska w klubach zmieniają się często – przed kampanią sprawdź źródło w kolumnie H.</t>
         </is>
@@ -1008,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:K148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6632,42 +6701,42 @@
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>Holandia</t>
+          <t>Portugalia</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>SC Braga</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>Kelvin de Lang</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting &amp; Recruitment, Academy De Toekomst</t>
+          <t>Formação – scouting</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii</t>
+          <t>Akademia (Cidade Desportiva)</t>
         </is>
       </c>
       <c r="F110" s="7" t="inlineStr"/>
-      <c r="G110" s="8" t="inlineStr">
-        <is>
-          <t>https://www.ajax.nl/club/jeugdopleiding</t>
+      <c r="G110" s="7" t="inlineStr">
+        <is>
+          <t>mail@scbraga.pt; tel. 253 261 259 (formação)</t>
         </is>
       </c>
       <c r="H110" s="8" t="inlineStr">
         <is>
-          <t>https://www.ajax.nl/artikelen/ajax-doc-scouten-voor-de-toekomst</t>
+          <t>https://scbraga.pt/formacao/</t>
         </is>
       </c>
       <c r="I110" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J110" s="7" t="inlineStr">
         <is>
@@ -6676,7 +6745,7 @@
       </c>
       <c r="K110" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: nr 1 w Europie – 85 wychowanków w 31 ligach UEFA, 1. miejsce Training Index; 2. na świecie w sprzedaży wychowanków (454 mln €)</t>
+          <t>CIES 2025: 95. miejsce w globalnym rankingu akademii</t>
         </is>
       </c>
     </row>
@@ -6688,37 +6757,37 @@
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>PSV Eindhoven</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>Rini de Groot</t>
+          <t>Kelvin de Lang</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>Hoofd jeugdscouting</t>
+          <t>Head of Scouting &amp; Recruitment, Academy De Toekomst</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii (De Herdgang)</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr"/>
-      <c r="G111" s="7" t="inlineStr">
-        <is>
-          <t>Oirschotsedijk 12a, 5651 GC Eindhoven</t>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>https://www.ajax.nl/club/jeugdopleiding</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
         <is>
-          <t>https://www.psv.nl/en/club/psv-campus-de-herdgang-1/psv-campus</t>
+          <t>https://www.ajax.nl/artikelen/ajax-doc-scouten-voor-de-toekomst</t>
         </is>
       </c>
       <c r="I111" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J111" s="7" t="inlineStr">
         <is>
@@ -6727,7 +6796,7 @@
       </c>
       <c r="K111" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting klubu: Jan Vennegoor of Hesselink. Uznana akademia (poza top 10 CIES)</t>
+          <t>CIES 2026: nr 1 w Europie – 85 wychowanków w 31 ligach UEFA, 1. miejsce Training Index; 2. na świecie w sprzedaży wychowanków (454 mln €)</t>
         </is>
       </c>
     </row>
@@ -6739,50 +6808,46 @@
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>Feyenoord</t>
+          <t>FC Twente / Heracles Academie</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>Ricardo Kern</t>
+          <t>Koen Fleer</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>Coördinator wedstrijdzaken Feyenoord Academy</t>
+          <t>Head of Youth Scouting</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>Scouting / sprawy drużyn akademii</t>
-        </is>
-      </c>
-      <c r="F112" s="7" t="inlineStr">
-        <is>
-          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
-        </is>
-      </c>
+          <t>Scouting akademii</t>
+        </is>
+      </c>
+      <c r="F112" s="7" t="inlineStr"/>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>Olympiaweg 280, 3078 HT Rotterdam</t>
+          <t>info@fctwenteheraclesacademie.nl; +31 53 852 5679</t>
         </is>
       </c>
       <c r="H112" s="8" t="inlineStr">
         <is>
-          <t>https://www.feyenoord.com/nl/academy/contact</t>
+          <t>https://fctwenteheraclesacademie.nl/over-de-academie/organisatie/</t>
         </is>
       </c>
       <c r="I112" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J112" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K112" s="7" t="inlineStr">
         <is>
-          <t>Uznana akademia (poza top 10 CIES)</t>
+          <t>Koordynator scoutingu: Jorn Nijhof</t>
         </is>
       </c>
     </row>
@@ -6794,33 +6859,33 @@
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>AZ Alkmaar</t>
+          <t>PSV Eindhoven</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rini de Groot</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>AZ Jeugdopleiding</t>
+          <t>Hoofd jeugdscouting</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>Akademia, dni selekcji U8–U13</t>
+          <t>Scouting akademii (De Herdgang)</t>
         </is>
       </c>
       <c r="F113" s="7" t="inlineStr"/>
-      <c r="G113" s="8" t="inlineStr">
-        <is>
-          <t>https://www.az.nl/jeugdopleiding</t>
+      <c r="G113" s="7" t="inlineStr">
+        <is>
+          <t>Oirschotsedijk 12a, 5651 GC Eindhoven</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>https://www.az.nl/jeugdopleiding/az-voetbalschool</t>
+          <t>https://www.psv.nl/en/club/psv-campus-de-herdgang-1/psv-campus</t>
         </is>
       </c>
       <c r="I113" s="9" t="n">
@@ -6833,7 +6898,7 @@
       </c>
       <c r="K113" s="7" t="inlineStr">
         <is>
-          <t>Uznana akademia (poza top 10 CIES)</t>
+          <t>Head of Scouting klubu: Jan Vennegoor of Hesselink. Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
@@ -6845,33 +6910,37 @@
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>sc Heerenveen</t>
+          <t>Feyenoord</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ricardo Kern</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>Jeugdopleiding / Akademy</t>
+          <t>Coördinator wedstrijdzaken Feyenoord Academy</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
-        </is>
-      </c>
-      <c r="F114" s="7" t="inlineStr"/>
+          <t>Scouting / sprawy drużyn akademii</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>tel. 0513 612 100; https://www.sc-heerenveen.nl/contact</t>
+          <t>Olympiaweg 280, 3078 HT Rotterdam</t>
         </is>
       </c>
       <c r="H114" s="8" t="inlineStr">
         <is>
-          <t>https://www.sc-heerenveen.nl/teams/akademy</t>
+          <t>https://www.feyenoord.com/nl/academy/contact</t>
         </is>
       </c>
       <c r="I114" s="9" t="n">
@@ -6884,19 +6953,19 @@
       </c>
       <c r="K114" s="7" t="inlineStr">
         <is>
-          <t>CIES MR98: Oliver Braude w top 10 bocznych obrońców U21</t>
+          <t>Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>Hiszpania</t>
+          <t>Holandia</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>AZ Alkmaar</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
@@ -6906,23 +6975,23 @@
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>Zubieta (cantera)</t>
+          <t>AZ Jeugdopleiding</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>Akademia – głównie talenty z Gipuzkoa</t>
+          <t>Akademia, dni selekcji U8–U13</t>
         </is>
       </c>
       <c r="F115" s="7" t="inlineStr"/>
-      <c r="G115" s="7" t="inlineStr">
-        <is>
-          <t>realsociedad.eus</t>
+      <c r="G115" s="8" t="inlineStr">
+        <is>
+          <t>https://www.az.nl/jeugdopleiding</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Real_Sociedad_Cantera</t>
+          <t>https://www.az.nl/jeugdopleiding/az-voetbalschool</t>
         </is>
       </c>
       <c r="I115" s="9" t="n">
@@ -6935,19 +7004,19 @@
       </c>
       <c r="K115" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: top 10 w Europie wg wychowanków w Big-5</t>
+          <t>Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>Hiszpania</t>
+          <t>Holandia</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t>Villarreal CF</t>
+          <t>sc Heerenveen</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
@@ -6957,23 +7026,23 @@
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>Cantera Grogueta</t>
+          <t>Jeugdopleiding / Akademy</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>Akademia (36 drużyn, ~650 zawodników)</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F116" s="7" t="inlineStr"/>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>formularz: villarrealcf.es/en/formulario-contacto/</t>
+          <t>tel. 0513 612 100; https://www.sc-heerenveen.nl/contact</t>
         </is>
       </c>
       <c r="H116" s="8" t="inlineStr">
         <is>
-          <t>https://villarrealcf.es/es/cantera-grogueta/</t>
+          <t>https://www.sc-heerenveen.nl/teams/akademy</t>
         </is>
       </c>
       <c r="I116" s="9" t="n">
@@ -6986,45 +7055,45 @@
       </c>
       <c r="K116" s="7" t="inlineStr">
         <is>
-          <t>Bez otwartych testów dla chłopców. Uznana akademia (poza top 10 CIES)</t>
+          <t>CIES MR98: Oliver Braude w top 10 bocznych obrońców U21</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>Hiszpania</t>
+          <t>Holandia</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>Valencia CF</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rudy Jansen</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>Academia VCF (Paterna)</t>
+          <t>Head of Scouting Youth Academy</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Scouting akademii (sieć klubów RAC)</t>
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr"/>
-      <c r="G117" s="8" t="inlineStr">
-        <is>
-          <t>https://formacion.valenciacf.com/en/contacto/</t>
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>fcutrecht.nl</t>
         </is>
       </c>
       <c r="H117" s="8" t="inlineStr">
         <is>
-          <t>https://www.valenciacf.com/vcf-academy</t>
+          <t>https://www.voetbaltrainer.nl/coachvak/talentherkenning-en-scouting-bij-fc-utrecht/</t>
         </is>
       </c>
       <c r="I117" s="9" t="n">
@@ -7032,12 +7101,12 @@
       </c>
       <c r="J117" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K117" s="7" t="inlineStr">
         <is>
-          <t>Wg klubu: 4. najlepsza akademia w Europie (ranking CIES)</t>
+          <t>Nazwisko ze źródła branżowego – potwierdzić</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7118,7 @@
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
@@ -7059,27 +7128,27 @@
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>Lezama (cantera)</t>
+          <t>Zubieta (cantera)</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>Akademia – tylko zawodnicy z korzeniami baskijskimi</t>
+          <t>Akademia – głównie talenty z Gipuzkoa</t>
         </is>
       </c>
       <c r="F118" s="7" t="inlineStr"/>
       <c r="G118" s="7" t="inlineStr">
         <is>
-          <t>Barrio Garaioltza 147, 48196 Lezama; https://www.athletic-club.eus/en/contact/</t>
+          <t>realsociedad.eus</t>
         </is>
       </c>
       <c r="H118" s="8" t="inlineStr">
         <is>
-          <t>https://www.athletic-club.eus/en/teams/lezama/</t>
+          <t>https://en.wikipedia.org/wiki/Real_Sociedad_Cantera</t>
         </is>
       </c>
       <c r="I118" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J118" s="7" t="inlineStr">
         <is>
@@ -7088,7 +7157,7 @@
       </c>
       <c r="K118" s="7" t="inlineStr">
         <is>
-          <t>CIES MR99: 7. miejsce wg minut wychowanków w Big-5 (20 lat). Rekrutacja ograniczona do Kraju Basków</t>
+          <t>CIES 2026: top 10 w Europie wg wychowanków w Big-5</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7169,7 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>FC Barcelona</t>
+          <t>Villarreal CF</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
@@ -7110,27 +7179,27 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>La Masia</t>
+          <t>Cantera Grogueta</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Akademia (36 drużyn, ~650 zawodników)</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr"/>
       <c r="G119" s="7" t="inlineStr">
         <is>
-          <t>oab@fcbarcelona.cat (informacja ogólna)</t>
+          <t>formularz: villarrealcf.es/en/formulario-contacto/</t>
         </is>
       </c>
       <c r="H119" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcbarcelona.com/en/club/identity/la-masia</t>
+          <t>https://villarrealcf.es/es/cantera-grogueta/</t>
         </is>
       </c>
       <c r="I119" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J119" s="7" t="inlineStr">
         <is>
@@ -7139,7 +7208,7 @@
       </c>
       <c r="K119" s="7" t="inlineStr">
         <is>
-          <t>CIES MR99: 2. miejsce – 156 wychowanków w Big-5 (20 lat). barcaescola@fcbarcelona.cat to szkółka FCBEscola, nie scouting</t>
+          <t>Bez otwartych testów dla chłopców. Uznana akademia (poza top 10 CIES)</t>
         </is>
       </c>
     </row>
@@ -7151,37 +7220,37 @@
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Valencia CF</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>Juni Calafat</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>Chief Scout</t>
+          <t>Academia VCF (Paterna)</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>Scouting (głównie 1. zespół)</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F120" s="7" t="inlineStr"/>
-      <c r="G120" s="7" t="inlineStr">
-        <is>
-          <t>realmadrid.com – sekcja cantera</t>
+      <c r="G120" s="8" t="inlineStr">
+        <is>
+          <t>https://formacion.valenciacf.com/en/contacto/</t>
         </is>
       </c>
       <c r="H120" s="8" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Juni_Calafat</t>
+          <t>https://www.valenciacf.com/vcf-academy</t>
         </is>
       </c>
       <c r="I120" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J120" s="7" t="inlineStr">
         <is>
@@ -7190,155 +7259,147 @@
       </c>
       <c r="K120" s="7" t="inlineStr">
         <is>
-          <t>CIES MR99: 1. miejsce – 166 wychowanków w Big-5 (20 lat), 103 w 55 ligach. Brak publicznego kontaktu scoutingu</t>
+          <t>Wg klubu: 4. najlepsza akademia w Europie (ranking CIES)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
         <is>
-          <t>Niemcy</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t>Bayer 04 Leverkusen</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>Jennifer Weber</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>Geschäftsstelle Nachwuchsabteilung (NLZ)</t>
+          <t>Lezama (cantera)</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>Biuro akademii, testy tylko przez e-mail</t>
-        </is>
-      </c>
-      <c r="F121" s="7" t="inlineStr">
-        <is>
-          <t>Jennifer.Weber@bayer04.de</t>
-        </is>
-      </c>
+          <t>Akademia – tylko zawodnicy z korzeniami baskijskimi</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr"/>
       <c r="G121" s="7" t="inlineStr">
         <is>
-          <t>tel. 0214 866 03 43</t>
+          <t>Barrio Garaioltza 147, 48196 Lezama; https://www.athletic-club.eus/en/contact/</t>
         </is>
       </c>
       <c r="H121" s="8" t="inlineStr">
         <is>
-          <t>https://www.bayer04.de/en-us/page/youth/trial-sessions</t>
+          <t>https://www.athletic-club.eus/en/teams/lezama/</t>
         </is>
       </c>
       <c r="I121" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J121" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K121" s="7" t="inlineStr">
         <is>
-          <t>CIES: top 10 dochodów ze sprzedaży wychowanków (10 lat). Mail z organigramu NLZ – sprawdzić aktualność</t>
+          <t>CIES MR99: 7. miejsce wg minut wychowanków w Big-5 (20 lat). Rekrutacja ograniczona do Kraju Basków</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
         <is>
-          <t>Niemcy</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>FC Barcelona</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>Ramtin Mehdibehesht</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>Leiter Scouting (NLZ)</t>
+          <t>La Masia</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii, region Rhein-Main</t>
-        </is>
-      </c>
-      <c r="F122" s="7" t="inlineStr">
-        <is>
-          <t>m.ramtin@eintrachtfrankfurt.de</t>
-        </is>
-      </c>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr"/>
       <c r="G122" s="7" t="inlineStr">
         <is>
-          <t>info@eintracht-frankfurt.de; nachwuchs.eintracht.de</t>
+          <t>oab@fcbarcelona.cat (informacja ogólna)</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>https://nachwuchs.eintracht.de/leistungszentrum/team/</t>
+          <t>https://www.fcbarcelona.com/en/club/identity/la-masia</t>
         </is>
       </c>
       <c r="I122" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J122" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K122" s="7" t="inlineStr">
         <is>
-          <t>CIES MR98: Hugo Larsson wśród najlepszych defensywnych pomocników U21. Mail do potwierdzenia na stronie NLZ</t>
+          <t>CIES MR99: 2. miejsce – 156 wychowanków w Big-5 (20 lat). barcaescola@fcbarcelona.cat to szkółka FCBEscola, nie scouting</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
         <is>
-          <t>Niemcy</t>
+          <t>Hiszpania</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
         <is>
-          <t>FC Bayern München</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Juni Calafat</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>FC Bayern Campus</t>
+          <t>Chief Scout</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>Akademia – tylko własny scouting, brak testów</t>
+          <t>Scouting (głównie 1. zespół)</t>
         </is>
       </c>
       <c r="F123" s="7" t="inlineStr"/>
-      <c r="G123" s="8" t="inlineStr">
-        <is>
-          <t>https://fcbayern.com/de/teams/fc-bayern-campus/info-und-kontakt</t>
+      <c r="G123" s="7" t="inlineStr">
+        <is>
+          <t>realmadrid.com – sekcja cantera</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
         <is>
-          <t>https://fcbayern.com/de/teams/fc-bayern-campus/info-und-kontakt</t>
+          <t>https://en.wikipedia.org/wiki/Juni_Calafat</t>
         </is>
       </c>
       <c r="I123" s="9" t="n">
@@ -7351,45 +7412,49 @@
       </c>
       <c r="K123" s="7" t="inlineStr">
         <is>
-          <t>CIES MR98: Aleksandar Pavlović w top pomocników U21</t>
+          <t>CIES MR99: 1. miejsce – 166 wychowanków w Big-5 (20 lat), 103 w 55 ligach. Brak publicznego kontaktu scoutingu</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>Chorwacja</t>
+          <t>Niemcy</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t>GNK Dinamo Zagreb</t>
+          <t>Bayer 04 Leverkusen</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Jennifer Weber</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>Dinamo Akademija</t>
+          <t>Geschäftsstelle Nachwuchsabteilung (NLZ)</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
-        </is>
-      </c>
-      <c r="F124" s="7" t="inlineStr"/>
+          <t>Biuro akademii, testy tylko przez e-mail</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr">
+        <is>
+          <t>Jennifer.Weber@bayer04.de</t>
+        </is>
+      </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
-          <t>dinamo@gnkdinamo.hr; 01 238 6111</t>
+          <t>tel. 0214 866 03 43</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
         <is>
-          <t>https://gnkdinamo.hr/hr/info/kontakt</t>
+          <t>https://www.bayer04.de/en-us/page/youth/trial-sessions</t>
         </is>
       </c>
       <c r="I124" s="9" t="n">
@@ -7397,54 +7462,54 @@
       </c>
       <c r="J124" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K124" s="7" t="inlineStr">
         <is>
-          <t>Czołowa akademia sprzedażowa regionu (poza top 10 CIES 2026)</t>
+          <t>CIES: top 10 dochodów ze sprzedaży wychowanków (10 lat). Mail z organigramu NLZ – sprawdzić aktualność</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Niemcy</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
         <is>
-          <t>FK Partizan</t>
+          <t>TSG Hoffenheim</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Jonathan Hader</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>Omladinska škola</t>
+          <t>Leiter Scouting &amp; Kadermanagement (Akademie)</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F125" s="7" t="inlineStr"/>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>https://partizan.rs/en</t>
+          <t>https://www.tsg-hoffenheim.de/akademie/services/kontakt-akademie</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
         <is>
-          <t>http://www.en.partizan.rs/omladinska-skola-fudbala/</t>
+          <t>https://www.tsg-hoffenheim.de/aktuelles/news/2025/08/kurzpass-kw32</t>
         </is>
       </c>
       <c r="I125" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J125" s="7" t="inlineStr">
         <is>
@@ -7453,45 +7518,49 @@
       </c>
       <c r="K125" s="7" t="inlineStr">
         <is>
-          <t>CIES: wcześniej nr 1 rocznego rankingu akademii (przed Ajaxem)</t>
+          <t>Od VIII 2025. Jedna z czołowych akademii w Niemczech</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Niemcy</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
         <is>
-          <t>FK Crvena zvezda</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ramtin Mehdibehesht</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Omladinska škola</t>
+          <t>Leiter Scouting (NLZ)</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
-        </is>
-      </c>
-      <c r="F126" s="7" t="inlineStr"/>
-      <c r="G126" s="8" t="inlineStr">
-        <is>
-          <t>https://www.crvenazvezdafk.com/en/klub/kontakt-i-lokacija</t>
+          <t>Scouting akademii, region Rhein-Main</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr">
+        <is>
+          <t>m.ramtin@eintrachtfrankfurt.de</t>
+        </is>
+      </c>
+      <c r="G126" s="7" t="inlineStr">
+        <is>
+          <t>info@eintracht-frankfurt.de; nachwuchs.eintracht.de</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>https://www.crvenazvezdafk.com/en/vesti-kategorija/omladinska-shkola</t>
+          <t>https://nachwuchs.eintracht.de/leistungszentrum/team/</t>
         </is>
       </c>
       <c r="I126" s="9" t="n">
@@ -7499,54 +7568,54 @@
       </c>
       <c r="J126" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K126" s="7" t="inlineStr">
         <is>
-          <t>Uznana akademia (poza top 10 CIES)</t>
+          <t>CIES MR98: Hugo Larsson wśród najlepszych defensywnych pomocników U21. Mail do potwierdzenia na stronie NLZ</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
         <is>
-          <t>Ukraina</t>
+          <t>Niemcy</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>Dynamo Kijów</t>
+          <t>Borussia Mönchengladbach</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Markus Hausweiler</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>Dział scoutingu</t>
+          <t>Bereichsleiter Scouting NLZ (od U14)</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>Scouting</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F127" s="7" t="inlineStr"/>
-      <c r="G127" s="7" t="inlineStr">
-        <is>
-          <t>tel. +38 044 278 06 28</t>
+      <c r="G127" s="8" t="inlineStr">
+        <is>
+          <t>https://www.borussia.de/de/allgemeines/kontakt</t>
         </is>
       </c>
       <c r="H127" s="8" t="inlineStr">
         <is>
-          <t>https://fcdynamo.com/en/pages/contacts</t>
+          <t>https://www.borussia.de/nlz-scouting</t>
         </is>
       </c>
       <c r="I127" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J127" s="7" t="inlineStr">
         <is>
@@ -7555,70 +7624,66 @@
       </c>
       <c r="K127" s="7" t="inlineStr">
         <is>
-          <t>CIES 2026: 3. miejsce w Europie – 72 wychowanków w 31 ligach UEFA. Uwaga: sytuacja wojenna</t>
+          <t>Scouting najmłodszych: Christian Wagner</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t>Anglia</t>
+          <t>Niemcy</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>1. FSV Mainz 05</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>David Harrison</t>
+          <t>Volker Kersting</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>Head of Academy Recruitment</t>
+          <t>Direktor Nachwuchs</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja akademii</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F128" s="7" t="inlineStr"/>
-      <c r="G128" s="7" t="inlineStr">
-        <is>
-          <t>Carrington Training Complex, Birch Road, Manchester M31 4BH</t>
+      <c r="G128" s="8" t="inlineStr">
+        <is>
+          <t>https://www.mainz05.de/mitarbeiter</t>
         </is>
       </c>
       <c r="H128" s="8" t="inlineStr">
         <is>
-          <t>https://www.manutd.com/en/help/faqs/club-information2</t>
+          <t>https://www.mainz05.de/mitarbeiter</t>
         </is>
       </c>
       <c r="I128" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J128" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
-        </is>
-      </c>
-      <c r="K128" s="7" t="inlineStr">
-        <is>
-          <t>CIES MR99: 103 wychowanków w Big-5 (20 lat), top 10 wg minut. Nazwisko ze źródła nieoficjalnego – potwierdzić</t>
-        </is>
-      </c>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K128" s="7" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
-          <t>Czechy</t>
+          <t>Niemcy</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>SK Slavia Praha</t>
+          <t>VfB Stuttgart</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
@@ -7628,23 +7693,23 @@
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>Slávistická akademie – vedení mládeže</t>
+          <t>NLZ – Scouting</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>Akademia (Eden, Horní Měcholupy, Xaverov)</t>
+          <t>Rocznik 2009 i młodsi tylko przez scouting; młodsi przez zapisy na Talentsichtung</t>
         </is>
       </c>
       <c r="F129" s="7" t="inlineStr"/>
-      <c r="G129" s="8" t="inlineStr">
-        <is>
-          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
+      <c r="G129" s="7" t="inlineStr">
+        <is>
+          <t>Mercedesstraße 109, 70372 Stuttgart</t>
         </is>
       </c>
       <c r="H129" s="8" t="inlineStr">
         <is>
-          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
+          <t>https://www.vfb.de/de/1893/junge-wilde/jugendkonzept/seite/leistungszentrum/</t>
         </is>
       </c>
       <c r="I129" s="9" t="n">
@@ -7657,13 +7722,974 @@
       </c>
       <c r="K129" s="7" t="inlineStr">
         <is>
+          <t>12 scoutów młodzieżowych w regionie</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t>Niemcy</t>
+        </is>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>FC Bayern München</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>FC Bayern Campus</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>Akademia – tylko własny scouting, brak testów</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr"/>
+      <c r="G130" s="8" t="inlineStr">
+        <is>
+          <t>https://fcbayern.com/de/teams/fc-bayern-campus/info-und-kontakt</t>
+        </is>
+      </c>
+      <c r="H130" s="8" t="inlineStr">
+        <is>
+          <t>https://fcbayern.com/de/teams/fc-bayern-campus/info-und-kontakt</t>
+        </is>
+      </c>
+      <c r="I130" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J130" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K130" s="7" t="inlineStr">
+        <is>
+          <t>CIES MR98: Aleksandar Pavlović w top pomocników U21</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="7" t="inlineStr">
+        <is>
+          <t>Niemcy</t>
+        </is>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>SC Freiburg</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>Jochen Saier</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t>Sportvorstand / szef scoutingu</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>Fußballschule (akademia)</t>
+        </is>
+      </c>
+      <c r="F131" s="7" t="inlineStr"/>
+      <c r="G131" s="7" t="inlineStr">
+        <is>
+          <t>formularz: scfreiburg.com/en/specials/service/contact/</t>
+        </is>
+      </c>
+      <c r="H131" s="8" t="inlineStr">
+        <is>
+          <t>https://www.scfreiburg.com/fussballschule/fussballschule/leitungsteam/</t>
+        </is>
+      </c>
+      <c r="I131" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J131" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K131" s="7" t="inlineStr">
+        <is>
+          <t>Klasyczny klub szkolący</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="7" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
+        <is>
+          <t>GNK Dinamo Zagreb</t>
+        </is>
+      </c>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="inlineStr">
+        <is>
+          <t>Dinamo Akademija</t>
+        </is>
+      </c>
+      <c r="E132" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F132" s="7" t="inlineStr"/>
+      <c r="G132" s="7" t="inlineStr">
+        <is>
+          <t>dinamo@gnkdinamo.hr; 01 238 6111</t>
+        </is>
+      </c>
+      <c r="H132" s="8" t="inlineStr">
+        <is>
+          <t>https://gnkdinamo.hr/hr/info/kontakt</t>
+        </is>
+      </c>
+      <c r="I132" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J132" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K132" s="7" t="inlineStr">
+        <is>
+          <t>Czołowa akademia sprzedażowa regionu (poza top 10 CIES 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t>HNK Hajduk Split</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t>Akademija</t>
+        </is>
+      </c>
+      <c r="E133" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F133" s="7" t="inlineStr"/>
+      <c r="G133" s="7" t="inlineStr">
+        <is>
+          <t>info@hajduk.hr; 021 323 650</t>
+        </is>
+      </c>
+      <c r="H133" s="8" t="inlineStr">
+        <is>
+          <t>https://hajduk.hr/akademija/struktura</t>
+        </is>
+      </c>
+      <c r="I133" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J133" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K133" s="7" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B134" s="7" t="inlineStr">
+        <is>
+          <t>HNK Rijeka</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t>Škola nogometa</t>
+        </is>
+      </c>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F134" s="7" t="inlineStr"/>
+      <c r="G134" s="7" t="inlineStr">
+        <is>
+          <t>skolanogometa@nk-rijeka.hr; +385 51 612 041</t>
+        </is>
+      </c>
+      <c r="H134" s="8" t="inlineStr">
+        <is>
+          <t>https://nk-rijeka.hr/skola/kontakt/</t>
+        </is>
+      </c>
+      <c r="I134" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J134" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K134" s="7" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>Chorwacja</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t>NK Osijek</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>Škola nogometa</t>
+        </is>
+      </c>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F135" s="7" t="inlineStr"/>
+      <c r="G135" s="7" t="inlineStr">
+        <is>
+          <t>skola.nogometa@nk-osijek.hr; +385 31 586 462</t>
+        </is>
+      </c>
+      <c r="H135" s="8" t="inlineStr">
+        <is>
+          <t>https://nk-osijek.hr/kontakt/</t>
+        </is>
+      </c>
+      <c r="I135" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J135" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K135" s="7" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B136" s="7" t="inlineStr">
+        <is>
+          <t>FK Partizan</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t>Omladinska škola</t>
+        </is>
+      </c>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F136" s="7" t="inlineStr"/>
+      <c r="G136" s="8" t="inlineStr">
+        <is>
+          <t>https://partizan.rs/en</t>
+        </is>
+      </c>
+      <c r="H136" s="8" t="inlineStr">
+        <is>
+          <t>http://www.en.partizan.rs/omladinska-skola-fudbala/</t>
+        </is>
+      </c>
+      <c r="I136" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J136" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K136" s="7" t="inlineStr">
+        <is>
+          <t>CIES: wcześniej nr 1 rocznego rankingu akademii (przed Ajaxem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="7" t="inlineStr">
+        <is>
+          <t>Serbia</t>
+        </is>
+      </c>
+      <c r="B137" s="7" t="inlineStr">
+        <is>
+          <t>FK Crvena zvezda</t>
+        </is>
+      </c>
+      <c r="C137" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t>Omladinska škola</t>
+        </is>
+      </c>
+      <c r="E137" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F137" s="7" t="inlineStr"/>
+      <c r="G137" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crvenazvezdafk.com/en/klub/kontakt-i-lokacija</t>
+        </is>
+      </c>
+      <c r="H137" s="8" t="inlineStr">
+        <is>
+          <t>https://www.crvenazvezdafk.com/en/vesti-kategorija/omladinska-shkola</t>
+        </is>
+      </c>
+      <c r="I137" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J137" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K137" s="7" t="inlineStr">
+        <is>
+          <t>Uznana akademia (poza top 10 CIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t>Ukraina</t>
+        </is>
+      </c>
+      <c r="B138" s="7" t="inlineStr">
+        <is>
+          <t>Dynamo Kijów</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr">
+        <is>
+          <t>Dział scoutingu</t>
+        </is>
+      </c>
+      <c r="E138" s="7" t="inlineStr">
+        <is>
+          <t>Scouting</t>
+        </is>
+      </c>
+      <c r="F138" s="7" t="inlineStr"/>
+      <c r="G138" s="7" t="inlineStr">
+        <is>
+          <t>tel. +38 044 278 06 28</t>
+        </is>
+      </c>
+      <c r="H138" s="8" t="inlineStr">
+        <is>
+          <t>https://fcdynamo.com/en/pages/contacts</t>
+        </is>
+      </c>
+      <c r="I138" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J138" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K138" s="7" t="inlineStr">
+        <is>
+          <t>CIES 2026: 3. miejsce w Europie – 72 wychowanków w 31 ligach UEFA. Uwaga: sytuacja wojenna</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
+          <t>Anglia</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>David Harrison</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>Head of Academy Recruitment</t>
+        </is>
+      </c>
+      <c r="E139" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F139" s="7" t="inlineStr"/>
+      <c r="G139" s="7" t="inlineStr">
+        <is>
+          <t>Carrington Training Complex, Birch Road, Manchester M31 4BH</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/help/faqs/club-information2</t>
+        </is>
+      </c>
+      <c r="I139" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J139" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K139" s="7" t="inlineStr">
+        <is>
+          <t>CIES MR99: 103 wychowanków w Big-5 (20 lat), top 10 wg minut. Nazwisko ze źródła nieoficjalnego – potwierdzić</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t>Czechy</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t>SK Slavia Praha</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t>Slávistická akademie – vedení mládeže</t>
+        </is>
+      </c>
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>Akademia (Eden, Horní Měcholupy, Xaverov)</t>
+        </is>
+      </c>
+      <c r="F140" s="7" t="inlineStr"/>
+      <c r="G140" s="8" t="inlineStr">
+        <is>
+          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
+        </is>
+      </c>
+      <c r="H140" s="8" t="inlineStr">
+        <is>
+          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
+        </is>
+      </c>
+      <c r="I140" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J140" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K140" s="7" t="inlineStr">
+        <is>
           <t>CIES MR98: El Hadji Malick Diouf w top 10 bocznych obrońców U21</t>
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t>Czechy</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>AC Sparta Praha</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>Akademie – nábory</t>
+        </is>
+      </c>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>Nabory roczników 2014–2020</t>
+        </is>
+      </c>
+      <c r="F141" s="7" t="inlineStr"/>
+      <c r="G141" s="7" t="inlineStr">
+        <is>
+          <t>WhatsApp +420 704 847 471</t>
+        </is>
+      </c>
+      <c r="H141" s="8" t="inlineStr">
+        <is>
+          <t>https://ac.sparta.cz/nabory</t>
+        </is>
+      </c>
+      <c r="I141" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J141" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K141" s="7" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="7" t="inlineStr">
+        <is>
+          <t>Czechy</t>
+        </is>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
+        <is>
+          <t>FC Viktoria Plzeň</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t>Mládež</t>
+        </is>
+      </c>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F142" s="7" t="inlineStr"/>
+      <c r="G142" s="7" t="inlineStr">
+        <is>
+          <t>fcviktoria@fcviktoria.cz; https://www.fcviktoria.cz/zobraz.asp?t=mladez-kontakty</t>
+        </is>
+      </c>
+      <c r="H142" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcviktoria.cz/zobraz.asp?t=mladez-kontakty</t>
+        </is>
+      </c>
+      <c r="I142" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J142" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K142" s="7" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>Rosenborg BK</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t>John Vik</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>Head of Scouting &amp; Recruitment</t>
+        </is>
+      </c>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>Scouting i rekrutacja</t>
+        </is>
+      </c>
+      <c r="F143" s="7" t="inlineStr">
+        <is>
+          <t>john.vik@rbk.no</t>
+        </is>
+      </c>
+      <c r="G143" s="7" t="inlineStr">
+        <is>
+          <t>Scout: Trond Henriksen – trond.henriksen@rbk.no, 915 91 031</t>
+        </is>
+      </c>
+      <c r="H143" s="8" t="inlineStr">
+        <is>
+          <t>https://www.rbk.no/om-rbk/ansatte/sport</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J143" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K143" s="7" t="inlineStr">
+        <is>
+          <t>Klub współpracuje z SciSports (scouting oparty na danych)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B144" s="7" t="inlineStr">
+        <is>
+          <t>Strømsgodset IF</t>
+        </is>
+      </c>
+      <c r="C144" s="7" t="inlineStr">
+        <is>
+          <t>Jan Vidar Haugstulen</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutteringsansvarlig, Eliteakademiet</t>
+        </is>
+      </c>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja do akademii</t>
+        </is>
+      </c>
+      <c r="F144" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G144" s="7" t="inlineStr">
+        <is>
+          <t>tel. 913 32 753</t>
+        </is>
+      </c>
+      <c r="H144" s="8" t="inlineStr">
+        <is>
+          <t>https://www.godset.no/utvikling/eliteakademiet</t>
+        </is>
+      </c>
+      <c r="I144" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J144" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K144" s="7" t="inlineStr">
+        <is>
+          <t>Znana akademia wprowadzająca młodzież do 1. zespołu</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t>FK Bodø/Glimt</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F145" s="7" t="inlineStr"/>
+      <c r="G145" s="7" t="inlineStr">
+        <is>
+          <t>bg@glimt.no</t>
+        </is>
+      </c>
+      <c r="H145" s="8" t="inlineStr">
+        <is>
+          <t>https://x.com/Glimt</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J145" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K145" s="7" t="inlineStr">
+        <is>
+          <t>Brak publicznego maila akademii</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B146" s="7" t="inlineStr">
+        <is>
+          <t>SK Brann</t>
+        </is>
+      </c>
+      <c r="C146" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D146" s="7" t="inlineStr">
+        <is>
+          <t>Akademiet</t>
+        </is>
+      </c>
+      <c r="E146" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F146" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G146" s="7" t="inlineStr">
+        <is>
+          <t>tel. +47 55 59 85 00</t>
+        </is>
+      </c>
+      <c r="H146" s="8" t="inlineStr">
+        <is>
+          <t>https://www.brann.no/lag/akademiet/ansatte</t>
+        </is>
+      </c>
+      <c r="I146" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J146" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K146" s="7" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t>Słowacja</t>
+        </is>
+      </c>
+      <c r="B147" s="7" t="inlineStr">
+        <is>
+          <t>MŠK Žilina</t>
+        </is>
+      </c>
+      <c r="C147" s="7" t="inlineStr">
+        <is>
+          <t>Viktor Miko</t>
+        </is>
+      </c>
+      <c r="D147" s="7" t="inlineStr">
+        <is>
+          <t>Skauting U7–U12</t>
+        </is>
+      </c>
+      <c r="E147" s="7" t="inlineStr">
+        <is>
+          <t>Nabór i scouting najmłodszych</t>
+        </is>
+      </c>
+      <c r="F147" s="7" t="inlineStr">
+        <is>
+          <t>Viktor.Miko@mskzilina.sk</t>
+        </is>
+      </c>
+      <c r="G147" s="7" t="inlineStr">
+        <is>
+          <t>mskzilina@mskzilina.sk; +421 41 54 24 958</t>
+        </is>
+      </c>
+      <c r="H147" s="8" t="inlineStr">
+        <is>
+          <t>http://mskzilina.sk/nabor</t>
+        </is>
+      </c>
+      <c r="I147" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J147" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K147" s="7" t="inlineStr">
+        <is>
+          <t>Jedna z najbardziej znanych akademii w Europie Środkowej</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="7" t="inlineStr">
+        <is>
+          <t>Słowenia</t>
+        </is>
+      </c>
+      <c r="B148" s="7" t="inlineStr">
+        <is>
+          <t>NK Maribor</t>
+        </is>
+      </c>
+      <c r="C148" s="7" t="inlineStr">
+        <is>
+          <t>Danijel Širec</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="inlineStr">
+        <is>
+          <t>Vodja skavtske službe (szef scoutingu)</t>
+        </is>
+      </c>
+      <c r="E148" s="7" t="inlineStr">
+        <is>
+          <t>Scouting akademii</t>
+        </is>
+      </c>
+      <c r="F148" s="7" t="inlineStr"/>
+      <c r="G148" s="7" t="inlineStr">
+        <is>
+          <t>nogometna.sola@nkmaribor.com; 02 620 97 05</t>
+        </is>
+      </c>
+      <c r="H148" s="8" t="inlineStr">
+        <is>
+          <t>https://www.nkmaribor.com/footballSchool/basic/contact</t>
+        </is>
+      </c>
+      <c r="I148" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J148" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K148" s="7" t="inlineStr">
+        <is>
+          <t>Dyrektor szkółki: Sebastijan Harc; dyr. sportowy: Boštjan Kreft</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K129"/>
-  <conditionalFormatting sqref="A2:K129">
+  <autoFilter ref="A1:K148"/>
+  <conditionalFormatting sqref="A2:K148">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Zweryfikowany"</formula>
     </cfRule>
@@ -7671,13 +8697,13 @@
       <formula>$J2="Do potwierdzenia"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I129">
+  <conditionalFormatting sqref="I2:I148">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>$I2=1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Zweryfikowany,Częściowo – brak maila osoby,Do potwierdzenia"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7800,33 +8826,55 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H147" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H148" r:id="rId167"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Uzupelnione maile scoutingu: Ajax, Genk, Elfsborg, Malmo, Salzburg, Club Brugge, Dinamo Zagreb i inne
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Be8XiCwvE6GnhZjaxWth9
</commit_message>
<xml_diff>
--- a/Kluby_Europa_Kontakty_Scouting.xlsx
+++ b/Kluby_Europa_Kontakty_Scouting.xlsx
@@ -1579,41 +1579,41 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Lars Hallengreen</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Scoutingansvarig MFF Ungdom</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>info@mff.se</t>
+          <t>Per Ågren (dyr. sportowy MFF Ungdom): per.agren@mff.se; info@mff.se</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>https://www.mff.se/om-malmo-ff/kontakt/</t>
+          <t>https://www.mff.se/nyheter/mot-lars-hallengreen-ny-scoutingansvarig-for-mff-ungdom/</t>
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do rekrutacji akademii</t>
+          <t>Szef scoutingu klubu: Jeffrey Aubynn</t>
         </is>
       </c>
     </row>
@@ -1630,23 +1630,23 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tony Lundqvist</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Akademichef</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Akademia / scouting</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>info@elfsborg.se; 033-13 91 91</t>
+          <t>scouting@elfsborg.se; info@elfsborg.se</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -1655,16 +1655,16 @@
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do rekrutacji akademii</t>
+          <t>Ungdomsansvarig: Andreas Klarström, 072-401 72 75</t>
         </is>
       </c>
     </row>
@@ -4129,12 +4129,12 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Jesper van Aarnhem</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Club NXT – akademia</t>
+          <t>Head Scout Club NXT</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -4143,9 +4143,9 @@
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr"/>
-      <c r="G60" s="8" t="inlineStr">
-        <is>
-          <t>https://www.clubbrugge.be/en/nxt-contact</t>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>info@clubbrugge.be; formularz: clubbrugge.be/en/nxt-contact</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="K61" s="7" t="inlineStr">
         <is>
-          <t>Pro League. Chief Academy: Tim Borguet; Football Director U13–U23: Tim Scheers</t>
+          <t>Pro League. Scouting, rekrutacja i retencja młodzieży: Peter Verbeke (zespół). Chief Academy: Tim Borguet</t>
         </is>
       </c>
     </row>
@@ -4231,12 +4231,12 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Koen Daerden</t>
+          <t>Wouter Vanbussel</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Technical Director Youth Academy</t>
+          <t>Jeugdscouting</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
@@ -4244,10 +4244,14 @@
           <t>Akademia</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr"/>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>wouter.vanbussel@krcgenk.be</t>
+        </is>
+      </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>jeugdsecretariaat@krcgenk.be</t>
+          <t>jeugdsecretariaat@krcgenk.be; scouting@krcgenk.be (scouting ogólny)</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
@@ -4260,12 +4264,12 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>Pro League. ~20 scoutów młodzieżowych; mail osoby tylko w bazach komercyjnych – nie podajemy</t>
+          <t>Pro League. Dyrektor techniczny akademii: Koen Daerden</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5177,7 @@
       <c r="F80" s="7" t="inlineStr"/>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>akademie.verwaltung@redbullsalzburg.at; 0662 433332 4603</t>
+          <t>academy@redbulls.com; akademie.verwaltung@redbullsalzburg.at; +43 662 433332 4603</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
@@ -5186,7 +5190,7 @@
       </c>
       <c r="J80" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K80" s="7" t="inlineStr">
@@ -6019,7 +6023,7 @@
       </c>
       <c r="K96" s="7" t="inlineStr">
         <is>
-          <t>Super League. Administracja Campusu: danique.stein@nachwuchs-campus.ch</t>
+          <t>Super League. Technischer Direktor (scouting/rekrutacja): Andreas Herrmann; Chief Scout: Marko Filipovic. Administracja Campusu: danique.stein@nachwuchs-campus.ch</t>
         </is>
       </c>
     </row>
@@ -6776,9 +6780,9 @@
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr"/>
-      <c r="G111" s="8" t="inlineStr">
-        <is>
-          <t>https://www.ajax.nl/club/jeugdopleiding</t>
+      <c r="G111" s="7" t="inlineStr">
+        <is>
+          <t>scouting@ajax.nl (dział scoutingu młodzieży)</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
@@ -6791,7 +6795,7 @@
       </c>
       <c r="J111" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K111" s="7" t="inlineStr">
@@ -6880,12 +6884,12 @@
       <c r="F113" s="7" t="inlineStr"/>
       <c r="G113" s="7" t="inlineStr">
         <is>
-          <t>Oirschotsedijk 12a, 5651 GC Eindhoven</t>
+          <t>fandesk@psv.nl; brak zgłoszeń – tylko scouting i otwarte treningi na De Herdgang</t>
         </is>
       </c>
       <c r="H113" s="8" t="inlineStr">
         <is>
-          <t>https://www.psv.nl/en/club/psv-campus-de-herdgang-1/psv-campus</t>
+          <t>https://fandesk.psv.nl/support/solutions/articles/80000304421-ik-wil-bij-psv-voetballen-kan-ik-mij-aanmelden-</t>
         </is>
       </c>
       <c r="I113" s="9" t="n">
@@ -6970,12 +6974,12 @@
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Aloys Wijnker</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>AZ Jeugdopleiding</t>
+          <t>Hoofd Jeugdopleiding</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
@@ -7841,17 +7845,17 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Luka Smiljanić</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>Dinamo Akademija</t>
+          <t>Voditelj skautinga (akademija)</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Scouting akademii</t>
         </is>
       </c>
       <c r="F132" s="7" t="inlineStr"/>
@@ -7862,7 +7866,7 @@
       </c>
       <c r="H132" s="8" t="inlineStr">
         <is>
-          <t>https://gnkdinamo.hr/hr/info/kontakt</t>
+          <t>https://gnkdinamo.hr/hr/dinamo-akademija/organizacija</t>
         </is>
       </c>
       <c r="I132" s="9" t="n">
@@ -7875,7 +7879,7 @@
       </c>
       <c r="K132" s="7" t="inlineStr">
         <is>
-          <t>Czołowa akademia sprzedażowa regionu (poza top 10 CIES 2026)</t>
+          <t>Scouci: Ivan Đurić, Igor Gabrijelić, Matej Žirović. Czołowa akademia sprzedażowa; CIES VI 2025: top 10 wg wychowanków w 55 ligach</t>
         </is>
       </c>
     </row>
@@ -8771,110 +8775,108 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H147" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H148" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H147" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H148" r:id="rId165"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Zakladka Akademie w SBS: 159 kontaktow do scoutingu i akademii z Europy + rankingi CIES (saldo transferow, pressing); nowe kluby: Lille, Udinese, Southampton, Tottenham, Sunderland, Leeds, Man City, Chelsea, Celtic, Szachtar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Be8XiCwvE6GnhZjaxWth9
</commit_message>
<xml_diff>
--- a/Kluby_Europa_Kontakty_Scouting.xlsx
+++ b/Kluby_Europa_Kontakty_Scouting.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Ranking CIES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kontakty'!$A$1:$K$156</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Beşiktaş – korekta'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ranking CIES'!$A$1:$F$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ranking CIES'!$A$1:$F$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A2)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A2)</f>
         <v/>
       </c>
       <c r="C2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A2,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A2,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A2,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A2,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E2" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A2,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A2,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -573,19 +573,19 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A3)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A3)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A3,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A3,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A3,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A3,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A3,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A3,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -596,19 +596,19 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A4)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A4)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A4,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A4,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A4,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A4,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A4,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A4,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -619,19 +619,19 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A5)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A5)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A5,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A5,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A5,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A5,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A5,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A5,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -642,19 +642,19 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A6)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A6)</f>
         <v/>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A6,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A6,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A6,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A6,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A6,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A6,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -665,19 +665,19 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A7)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A7)</f>
         <v/>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A7,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A7,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A7,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A7,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A7,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A7,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -688,19 +688,19 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A8)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A8)</f>
         <v/>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A8,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A8,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A8,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A8,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A8,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A8,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -711,19 +711,19 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A9)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A9)</f>
         <v/>
       </c>
       <c r="C9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A9,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A9,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A9,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A9,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E9" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A9,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A9,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -734,19 +734,19 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A10)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A10)</f>
         <v/>
       </c>
       <c r="C10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A10,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A10,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A10,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A10,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E10" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A10,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A10,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -757,19 +757,19 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A11)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A11)</f>
         <v/>
       </c>
       <c r="C11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A11,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A11,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A11,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A11,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E11" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A11,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A11,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -780,19 +780,19 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A12)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A12)</f>
         <v/>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A12,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A12,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A12,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A12,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E12" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A12,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A12,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A13)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A13)</f>
         <v/>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A13,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A13,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A13,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A13,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E13" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A13,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A13,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A14)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A14)</f>
         <v/>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A14,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A14,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A14,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A14,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E14" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A14,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A14,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -849,19 +849,19 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A15)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A15)</f>
         <v/>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A15,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A15,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A15,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A15,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E15" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A15,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A15,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -872,19 +872,19 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A16)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A16)</f>
         <v/>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A16,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A16,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D16" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A16,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A16,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E16" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A16,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A16,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -895,19 +895,19 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A17)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A17)</f>
         <v/>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A17,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A17,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D17" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A17,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A17,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E17" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A17,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A17,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -918,19 +918,19 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A18)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A18)</f>
         <v/>
       </c>
       <c r="C18" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A18,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A18,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D18" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A18,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A18,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E18" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A18,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A18,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A19)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A19)</f>
         <v/>
       </c>
       <c r="C19" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A19,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A19,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D19" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A19,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A19,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E19" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A19,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A19,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
@@ -964,103 +964,126 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <f>COUNTIF(Kontakty!$A$2:$A$148,A20)</f>
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A20)</f>
         <v/>
       </c>
       <c r="C20" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A20,Kontakty!$F$2:$F$148,"*@*")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A20,Kontakty!$F$2:$F$156,"*@*")</f>
         <v/>
       </c>
       <c r="D20" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A20,Kontakty!$I$2:$I$148,1)</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A20,Kontakty!$I$2:$I$156,1)</f>
         <v/>
       </c>
       <c r="E20" s="2">
-        <f>COUNTIFS(Kontakty!$A$2:$A$148,A20,Kontakty!$J$2:$J$148,"Zweryfikowany")</f>
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A20,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Szkocja</t>
+        </is>
+      </c>
+      <c r="B21" s="2">
+        <f>COUNTIF(Kontakty!$A$2:$A$156,A21)</f>
+        <v/>
+      </c>
+      <c r="C21" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A21,Kontakty!$F$2:$F$156,"*@*")</f>
+        <v/>
+      </c>
+      <c r="D21" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A21,Kontakty!$I$2:$I$156,1)</f>
+        <v/>
+      </c>
+      <c r="E21" s="2">
+        <f>COUNTIFS(Kontakty!$A$2:$A$156,A21,Kontakty!$J$2:$J$156,"Zweryfikowany")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>RAZEM</t>
         </is>
       </c>
-      <c r="B21" s="3">
-        <f>SUM(B2:B20)</f>
+      <c r="B22" s="3">
+        <f>SUM(B2:B21)</f>
         <v/>
       </c>
-      <c r="C21" s="3">
-        <f>SUM(C2:C20)</f>
+      <c r="C22" s="3">
+        <f>SUM(C2:C21)</f>
         <v/>
       </c>
-      <c r="D21" s="3">
-        <f>SUM(D2:D20)</f>
+      <c r="D22" s="3">
+        <f>SUM(D2:D21)</f>
         <v/>
       </c>
-      <c r="E21" s="3">
-        <f>SUM(E2:E20)</f>
+      <c r="E22" s="3">
+        <f>SUM(E2:E21)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Legenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
+          <t>Zweryfikowany – e-mail/kontakt opublikowany na oficjalnej stronie klubu (wiersz na zielono).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
+          <t>Częściowo – brak maila osoby – osoba i stanowisko potwierdzone, ale e-mail osoby nie jest publiczny lub jest ukryty przed botami; użyj kontaktu klubu.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
+          <t>Do potwierdzenia – dane ze źródła starszego lub nieoficjalnego; potwierdzić przed wysyłką (wiersz na pomarańczowo).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
+          <t>Priorytet: 1 = kontaktować w pierwszej kolejności, 3 = niski. Szwecja = kraj priorytetowy.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
+          <t>Nie podajemy maili z komercyjnych baz (RocketReach, Lusha itp.) ani maili zgadywanych z formatu domeny.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+          <t>Belgia: wszystkie 18 klubów Pro League 26/27; Austria: 12 klubów Bundesligi; Szwajcaria: 12 klubów Super League.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Dania: wszystkie 12 klubów Superligi i 12 klubów 1. Division (sezon 26/27, wg Transfermarkt). Oceny akademii: licencja DBU 2026–2028.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Stan na: 26.09.2026. Stanowiska w klubach zmieniają się często – przed kampanią sprawdź źródło w kolumnie H.</t>
         </is>
@@ -1077,7 +1100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K148"/>
+  <dimension ref="A1:K156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3638,17 +3661,17 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Empoli FC</t>
+          <t>Udinese Calcio (sektor młodzieżowy)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Marco Bertelli</t>
+          <t>José Ramón Rodríguez</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Responsabile Settore Giovanile</t>
+          <t>Responsabile Settore Giovanile (od V 2026)</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -3659,25 +3682,25 @@
       <c r="F50" s="7" t="inlineStr"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>social@empolifc.com</t>
+          <t>udinese@udinesespa.it; 0432 544911</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>https://www.empolifc.it/organigramma</t>
+          <t>https://www.udinese.it/club/organigramma</t>
         </is>
       </c>
       <c r="I50" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>Scouting attività di base: Paolo Mussi</t>
+          <t>CIES: +208 mln € salda transferów 2015–2024</t>
         </is>
       </c>
     </row>
@@ -3689,17 +3712,17 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Empoli FC</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Michele Sbravati</t>
+          <t>Marco Bertelli</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Youth Football Director</t>
+          <t>Responsabile Settore Giovanile</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -3710,12 +3733,12 @@
       <c r="F51" s="7" t="inlineStr"/>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>tel. 011 656 3629; Via Druento 175, Torino</t>
+          <t>social@empolifc.com</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>https://www.juventus.com/it/news/articoli/assetto-organizzativo-2024-2025-area-sportiva-juventus</t>
+          <t>https://www.empolifc.it/organigramma</t>
         </is>
       </c>
       <c r="I51" s="9" t="n">
@@ -3728,7 +3751,7 @@
       </c>
       <c r="K51" s="7" t="inlineStr">
         <is>
-          <t>CIES MR98: Kenan Yıldız w top skrzydłowych U21. Scouting Director: Stefano Stefanelli. Dane z 2024/25 – potwierdzić</t>
+          <t>Scouting attività di base: Paolo Mussi</t>
         </is>
       </c>
     </row>
@@ -3740,87 +3763,91 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Gianluca Baschieri</t>
+          <t>Michele Sbravati</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Head of Grassroot</t>
+          <t>Youth Football Director</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Grassroots</t>
+          <t>Sektor młodzieżowy</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr"/>
-      <c r="G52" s="7" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>tel. 011 656 3629; Via Druento 175, Torino</t>
+        </is>
+      </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
+          <t>https://www.juventus.com/it/news/articoli/assetto-organizzativo-2024-2025-area-sportiva-juventus</t>
         </is>
       </c>
       <c r="I52" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K52" s="7" t="inlineStr"/>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>CIES MR98: Kenan Yıldız w top skrzydłowych U21. Scouting Director: Stefano Stefanelli. Dane z 2024/25 – potwierdzić</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Francja</t>
+          <t>Włochy</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Stade Rennais (CIES)</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Denis Arnaud</t>
+          <t>Gianluca Baschieri</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Directeur de l'académie</t>
+          <t>Head of Grassroot</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Centre de formation</t>
+          <t>Grassroots</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr"/>
       <c r="G53" s="7" t="inlineStr"/>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
+          <t>https://www.parmacalcio1913.com/en/main-news/club-statement-new-football-department-structure-confirmed/</t>
         </is>
       </c>
       <c r="I53" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
-        </is>
-      </c>
-      <c r="K53" s="7" t="inlineStr">
-        <is>
-          <t>CIES 2026: 4. miejsce w Europie – 29 wychowanków w lidze Big-5. Nazwisko dyrektora do potwierdzenia</t>
-        </is>
-      </c>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3830,33 +3857,29 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>AS Monaco (CIES)</t>
+          <t>Stade Rennais</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Denis Arnaud</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Cellule recrutement Academy (La Diagonale)</t>
+          <t>Directeur de l'académie</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja do centrum szkoleniowego</t>
+          <t>Centre de formation</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr"/>
-      <c r="G54" s="8" t="inlineStr">
-        <is>
-          <t>https://www.asmonaco.com/encadrement/</t>
-        </is>
-      </c>
+      <c r="G54" s="7" t="inlineStr"/>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>https://www.asmonaco.com/en/academy/la-diagonale-centre-de-formation-de-las-monaco</t>
+          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
         </is>
       </c>
       <c r="I54" s="9" t="n">
@@ -3864,12 +3887,12 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>CIES: top 10 najbardziej dochodowych akademii (10 lat). Nie przyjmują zgłoszeń spontanicznych</t>
+          <t>CIES 2026: 4. miejsce w Europie – 29 wychowanków w lidze Big-5. Nazwisko dyrektora do potwierdzenia. Koordynacja rekrutacji: Philippe Barraud</t>
         </is>
       </c>
     </row>
@@ -3881,29 +3904,33 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>RC Lens</t>
+          <t>AS Monaco (CIES)</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Alaeddine Yahia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Responsable du recrutement de l'académie</t>
+          <t>Cellule recrutement Academy (La Diagonale)</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja akademii</t>
+          <t>Rekrutacja do centrum szkoleniowego</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr"/>
-      <c r="G55" s="7" t="inlineStr"/>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>https://www.asmonaco.com/encadrement/</t>
+        </is>
+      </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>https://www.rclens.fr/fr/pros-cellule-de-recrutement</t>
+          <t>https://www.asmonaco.com/en/academy/la-diagonale-centre-de-formation-de-las-monaco</t>
         </is>
       </c>
       <c r="I55" s="9" t="n">
@@ -3916,7 +3943,7 @@
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>recrutement@rclens.fr to adres HR (oferty pracy) – nie do zgłoszeń zawodników</t>
+          <t>CIES: top 10 najbardziej dochodowych akademii (10 lat). Nie przyjmują zgłoszeń spontanicznych</t>
         </is>
       </c>
     </row>
@@ -3928,29 +3955,29 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Olympique Lyonnais</t>
+          <t>RC Lens</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Johann Louvel</t>
+          <t>Alaeddine Yahia</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Directeur de l'Academy</t>
+          <t>Responsable du recrutement de l'académie</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Rekrutacja akademii</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr"/>
       <c r="G56" s="7" t="inlineStr"/>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>https://www.ol.fr/fr/academy/centre-de-formation/recrutement</t>
+          <t>https://www.rclens.fr/fr/pros-cellule-de-recrutement</t>
         </is>
       </c>
       <c r="I56" s="9" t="n">
@@ -3958,12 +3985,12 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>CIES: top 10 dochodów ze sprzedaży wychowanków; 34 wychowanków w Big-5. Zastępca ds. technicznych/rekrutacji: Mathieu Seckinger</t>
+          <t>recrutement@rclens.fr to adres HR (oferty pracy) – nie do zgłoszeń zawodników</t>
         </is>
       </c>
     </row>
@@ -3975,33 +4002,33 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Stade Rennais</t>
+          <t>Olympique Lyonnais</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Philippe Barraud</t>
+          <t>Johann Louvel</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Chargé de coordination du recrutement</t>
+          <t>Directeur de l'Academy</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja centrum szkoleniowego</t>
+          <t>Akademia</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr"/>
       <c r="G57" s="7" t="inlineStr"/>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>https://fr.wikipedia.org/wiki/Centre_de_formation_du_Stade_rennais_FC</t>
+          <t>https://www.ol.fr/fr/academy/centre-de-formation/recrutement</t>
         </is>
       </c>
       <c r="I57" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
@@ -4010,7 +4037,7 @@
       </c>
       <c r="K57" s="7" t="inlineStr">
         <is>
-          <t>Źródło nieoficjalne – potwierdzić na staderennais.com</t>
+          <t>CIES: top 10 dochodów ze sprzedaży wychowanków; 34 wychowanków w Big-5. Zastępca ds. technicznych/rekrutacji: Mathieu Seckinger</t>
         </is>
       </c>
     </row>
@@ -4027,32 +4054,32 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Philippe Liard</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Responsable cellule recrutement – centre de formation</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Formularz kontaktowy</t>
+          <t>Rekrutacja do akademii (Domaine de Luchin)</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr"/>
-      <c r="G58" s="8" t="inlineStr">
-        <is>
-          <t>https://www.losc.fr/contact</t>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>formularz: https://www.losc.fr/contact</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>https://www.losc.fr/formation</t>
+          <t>https://lepetitlillois.com/2024/07/27/philippe-liard-a-succede-a-mathieu-frison-a-la-cellule-de-recrutement-du-centre-de-formation-du-losc/</t>
         </is>
       </c>
       <c r="I58" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
@@ -4061,7 +4088,7 @@
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila do rekrutacji młodzieży</t>
+          <t>CIES: 4. w Europie wg salda transferów 2015–2024 (+391 mln €), 1. w Big-5. Dyrektor centrum: Jean-Michel Vandamme</t>
         </is>
       </c>
     </row>
@@ -8180,38 +8207,38 @@
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
         <is>
-          <t>Anglia</t>
+          <t>Ukraina</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>Szachtar Donieck</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>David Harrison</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>Head of Academy Recruitment</t>
+          <t>Shakhtar Football Academy</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja akademii</t>
+          <t>Akademia i szkółki</t>
         </is>
       </c>
       <c r="F139" s="7" t="inlineStr"/>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>Carrington Training Complex, Birch Road, Manchester M31 4BH</t>
+          <t>school@shakhtar.com; +380 800 300 314</t>
         </is>
       </c>
       <c r="H139" s="8" t="inlineStr">
         <is>
-          <t>https://www.manutd.com/en/help/faqs/club-information2</t>
+          <t>https://shakhtar.com/en/club/academy/</t>
         </is>
       </c>
       <c r="I139" s="9" t="n">
@@ -8219,24 +8246,24 @@
       </c>
       <c r="J139" s="7" t="inlineStr">
         <is>
-          <t>Do potwierdzenia</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K139" s="7" t="inlineStr">
         <is>
-          <t>CIES MR99: 103 wychowanków w Big-5 (20 lat), top 10 wg minut. Nazwisko ze źródła nieoficjalnego – potwierdzić</t>
+          <t>CIES: +190 mln € salda transferów 2015–2024. Uwaga: sytuacja wojenna</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
         <is>
-          <t>Czechy</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>SK Slavia Praha</t>
+          <t>Southampton FC</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
@@ -8246,48 +8273,48 @@
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>Slávistická akademie – vedení mládeže</t>
+          <t>Academy Recruitment – trials</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>Akademia (Eden, Horní Měcholupy, Xaverov)</t>
+          <t>Zgłoszenia zawodników na testy</t>
         </is>
       </c>
       <c r="F140" s="7" t="inlineStr"/>
-      <c r="G140" s="8" t="inlineStr">
-        <is>
-          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
+      <c r="G140" s="7" t="inlineStr">
+        <is>
+          <t>trials@saintsfc.co.uk</t>
         </is>
       </c>
       <c r="H140" s="8" t="inlineStr">
         <is>
-          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
+          <t>https://www.southamptonfc.com/en/academy-trials</t>
         </is>
       </c>
       <c r="I140" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J140" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
+          <t>Zweryfikowany</t>
         </is>
       </c>
       <c r="K140" s="7" t="inlineStr">
         <is>
-          <t>CIES MR98: El Hadji Malick Diouf w top 10 bocznych obrońców U21</t>
+          <t>Klub przyjmuje zgłoszenia (dane zawodnika + terminarz). CIES: czołówka pressingu</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
         <is>
-          <t>Czechy</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>AC Sparta Praha</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
@@ -8297,44 +8324,48 @@
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>Akademie – nábory</t>
+          <t>Academy Trials team</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>Nabory roczników 2014–2020</t>
+          <t>Zgłoszenia zawodników</t>
         </is>
       </c>
       <c r="F141" s="7" t="inlineStr"/>
       <c r="G141" s="7" t="inlineStr">
         <is>
-          <t>WhatsApp +420 704 847 471</t>
+          <t>academy.trials@tottenhamhotspur.com; academy@tottenhamhotspur.com</t>
         </is>
       </c>
       <c r="H141" s="8" t="inlineStr">
         <is>
-          <t>https://ac.sparta.cz/nabory</t>
+          <t>http://m.tottenhamhotspur.com/academy/trials/</t>
         </is>
       </c>
       <c r="I141" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J141" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K141" s="7" t="inlineStr"/>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K141" s="7" t="inlineStr">
+        <is>
+          <t>Adres ze starszej strony klubu – sprawdzić. Brak otwartych testów</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
         <is>
-          <t>Czechy</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t>FC Viktoria Plzeň</t>
+          <t>Sunderland AFC</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
@@ -8344,154 +8375,146 @@
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>Mládež</t>
+          <t>Academy of Light</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
+          <t>Zgłoszenia zawodników</t>
         </is>
       </c>
       <c r="F142" s="7" t="inlineStr"/>
       <c r="G142" s="7" t="inlineStr">
         <is>
-          <t>fcviktoria@fcviktoria.cz; https://www.fcviktoria.cz/zobraz.asp?t=mladez-kontakty</t>
+          <t>academy.feedback@safc.com</t>
         </is>
       </c>
       <c r="H142" s="8" t="inlineStr">
         <is>
-          <t>https://www.fcviktoria.cz/zobraz.asp?t=mladez-kontakty</t>
+          <t>https://www.safc.com/club/academy-of-light</t>
         </is>
       </c>
       <c r="I142" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J142" s="7" t="inlineStr">
         <is>
-          <t>Częściowo – brak maila osoby</t>
-        </is>
-      </c>
-      <c r="K142" s="7" t="inlineStr"/>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K142" s="7" t="inlineStr">
+        <is>
+          <t>Adres z przewodnika branżowego – potwierdzić</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
         <is>
-          <t>Norwegia</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
         <is>
-          <t>Rosenborg BK</t>
+          <t>Manchester United</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>John Vik</t>
+          <t>David Harrison</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>Head of Scouting &amp; Recruitment</t>
+          <t>Head of Academy Recruitment</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>Scouting i rekrutacja</t>
-        </is>
-      </c>
-      <c r="F143" s="7" t="inlineStr">
-        <is>
-          <t>john.vik@rbk.no</t>
-        </is>
-      </c>
+          <t>Rekrutacja akademii</t>
+        </is>
+      </c>
+      <c r="F143" s="7" t="inlineStr"/>
       <c r="G143" s="7" t="inlineStr">
         <is>
-          <t>Scout: Trond Henriksen – trond.henriksen@rbk.no, 915 91 031</t>
+          <t>Carrington Training Complex, Birch Road, Manchester M31 4BH</t>
         </is>
       </c>
       <c r="H143" s="8" t="inlineStr">
         <is>
-          <t>https://www.rbk.no/om-rbk/ansatte/sport</t>
+          <t>https://www.manutd.com/en/help/faqs/club-information2</t>
         </is>
       </c>
       <c r="I143" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J143" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Do potwierdzenia</t>
         </is>
       </c>
       <c r="K143" s="7" t="inlineStr">
         <is>
-          <t>Klub współpracuje z SciSports (scouting oparty na danych)</t>
+          <t>CIES MR99: 103 wychowanków w Big-5 (20 lat), top 10 wg minut. Nazwisko ze źródła nieoficjalnego – potwierdzić</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
         <is>
-          <t>Norwegia</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
         <is>
-          <t>Strømsgodset IF</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>Jan Vidar Haugstulen</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>Rekrutteringsansvarlig, Eliteakademiet</t>
+          <t>Academy (Thorp Arch)</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>Rekrutacja do akademii</t>
-        </is>
-      </c>
-      <c r="F144" s="7" t="inlineStr">
-        <is>
-          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
-        </is>
-      </c>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F144" s="7" t="inlineStr"/>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>tel. 913 32 753</t>
+          <t>tel. 01937 884400</t>
         </is>
       </c>
       <c r="H144" s="8" t="inlineStr">
         <is>
-          <t>https://www.godset.no/utvikling/eliteakademiet</t>
+          <t>https://www.leedsunited.com/en/club/careers</t>
         </is>
       </c>
       <c r="I144" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J144" s="7" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K144" s="7" t="inlineStr">
-        <is>
-          <t>Znana akademia wprowadzająca młodzież do 1. zespołu</t>
-        </is>
-      </c>
+      <c r="K144" s="7" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
         <is>
-          <t>Norwegia</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
         <is>
-          <t>FK Bodø/Glimt</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
@@ -8501,27 +8524,27 @@
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Academy – tylko własny scouting</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>Kontakt ogólny</t>
+          <t>Brak otwartych testów i zgłoszeń</t>
         </is>
       </c>
       <c r="F145" s="7" t="inlineStr"/>
-      <c r="G145" s="7" t="inlineStr">
-        <is>
-          <t>bg@glimt.no</t>
+      <c r="G145" s="8" t="inlineStr">
+        <is>
+          <t>https://www.mancity.com/club/safeguarding/scouts-and-scouting</t>
         </is>
       </c>
       <c r="H145" s="8" t="inlineStr">
         <is>
-          <t>https://x.com/Glimt</t>
+          <t>https://www.mancity.com/club/safeguarding/scouts-and-scouting</t>
         </is>
       </c>
       <c r="I145" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J145" s="7" t="inlineStr">
         <is>
@@ -8530,19 +8553,19 @@
       </c>
       <c r="K145" s="7" t="inlineStr">
         <is>
-          <t>Brak publicznego maila akademii</t>
+          <t>CIES: nr 1 pressingu (15,2/mecz); top 5 sprzedaży wychowanków (5 lat)</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
         <is>
-          <t>Norwegia</t>
+          <t>Anglia</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
         <is>
-          <t>SK Brann</t>
+          <t>Chelsea FC</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
@@ -8552,78 +8575,74 @@
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>Akademiet</t>
+          <t>Academy Player Recruitment Team</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>Akademia</t>
-        </is>
-      </c>
-      <c r="F146" s="7" t="inlineStr">
-        <is>
-          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
-        </is>
-      </c>
+          <t>Formularz zgłoszeniowy na stronie</t>
+        </is>
+      </c>
+      <c r="F146" s="7" t="inlineStr"/>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>tel. +47 55 59 85 00</t>
+          <t>formularz: chelseafc.com/en/about-the-academy</t>
         </is>
       </c>
       <c r="H146" s="8" t="inlineStr">
         <is>
-          <t>https://www.brann.no/lag/akademiet/ansatte</t>
+          <t>https://www.chelseafc.com/en/about-the-academy</t>
         </is>
       </c>
       <c r="I146" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J146" s="7" t="inlineStr">
         <is>
           <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
-      <c r="K146" s="7" t="inlineStr"/>
+      <c r="K146" s="7" t="inlineStr">
+        <is>
+          <t>CIES: nr 1 sprzedaży wychowanków w 5 lat (366 mln €)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>Słowacja</t>
+          <t>Czechy</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
         <is>
-          <t>MŠK Žilina</t>
+          <t>SK Slavia Praha</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>Viktor Miko</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>Skauting U7–U12</t>
+          <t>Slávistická akademie – vedení mládeže</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>Nabór i scouting najmłodszych</t>
-        </is>
-      </c>
-      <c r="F147" s="7" t="inlineStr">
-        <is>
-          <t>Viktor.Miko@mskzilina.sk</t>
-        </is>
-      </c>
-      <c r="G147" s="7" t="inlineStr">
-        <is>
-          <t>mskzilina@mskzilina.sk; +421 41 54 24 958</t>
+          <t>Akademia (Eden, Horní Měcholupy, Xaverov)</t>
+        </is>
+      </c>
+      <c r="F147" s="7" t="inlineStr"/>
+      <c r="G147" s="8" t="inlineStr">
+        <is>
+          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
         </is>
       </c>
       <c r="H147" s="8" t="inlineStr">
         <is>
-          <t>http://mskzilina.sk/nabor</t>
+          <t>https://www.slavia.cz/text/vedeni-mladeze</t>
         </is>
       </c>
       <c r="I147" s="9" t="n">
@@ -8631,69 +8650,481 @@
       </c>
       <c r="J147" s="7" t="inlineStr">
         <is>
-          <t>Zweryfikowany</t>
+          <t>Częściowo – brak maila osoby</t>
         </is>
       </c>
       <c r="K147" s="7" t="inlineStr">
         <is>
-          <t>Jedna z najbardziej znanych akademii w Europie Środkowej</t>
+          <t>CIES MR98: El Hadji Malick Diouf w top 10 bocznych obrońców U21</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
         <is>
-          <t>Słowenia</t>
+          <t>Czechy</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
         <is>
-          <t>NK Maribor</t>
+          <t>AC Sparta Praha</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>Danijel Širec</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>Vodja skavtske službe (szef scoutingu)</t>
+          <t>Akademie – nábory</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>Scouting akademii</t>
+          <t>Nabory roczników 2014–2020</t>
         </is>
       </c>
       <c r="F148" s="7" t="inlineStr"/>
       <c r="G148" s="7" t="inlineStr">
         <is>
+          <t>WhatsApp +420 704 847 471</t>
+        </is>
+      </c>
+      <c r="H148" s="8" t="inlineStr">
+        <is>
+          <t>https://ac.sparta.cz/nabory</t>
+        </is>
+      </c>
+      <c r="I148" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J148" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K148" s="7" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="7" t="inlineStr">
+        <is>
+          <t>Czechy</t>
+        </is>
+      </c>
+      <c r="B149" s="7" t="inlineStr">
+        <is>
+          <t>FC Viktoria Plzeň</t>
+        </is>
+      </c>
+      <c r="C149" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D149" s="7" t="inlineStr">
+        <is>
+          <t>Mládež</t>
+        </is>
+      </c>
+      <c r="E149" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F149" s="7" t="inlineStr"/>
+      <c r="G149" s="7" t="inlineStr">
+        <is>
+          <t>fcviktoria@fcviktoria.cz; https://www.fcviktoria.cz/zobraz.asp?t=mladez-kontakty</t>
+        </is>
+      </c>
+      <c r="H149" s="8" t="inlineStr">
+        <is>
+          <t>https://www.fcviktoria.cz/zobraz.asp?t=mladez-kontakty</t>
+        </is>
+      </c>
+      <c r="I149" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J149" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K149" s="7" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B150" s="7" t="inlineStr">
+        <is>
+          <t>Rosenborg BK</t>
+        </is>
+      </c>
+      <c r="C150" s="7" t="inlineStr">
+        <is>
+          <t>John Vik</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="inlineStr">
+        <is>
+          <t>Head of Scouting &amp; Recruitment</t>
+        </is>
+      </c>
+      <c r="E150" s="7" t="inlineStr">
+        <is>
+          <t>Scouting i rekrutacja</t>
+        </is>
+      </c>
+      <c r="F150" s="7" t="inlineStr">
+        <is>
+          <t>john.vik@rbk.no</t>
+        </is>
+      </c>
+      <c r="G150" s="7" t="inlineStr">
+        <is>
+          <t>Scout: Trond Henriksen – trond.henriksen@rbk.no, 915 91 031</t>
+        </is>
+      </c>
+      <c r="H150" s="8" t="inlineStr">
+        <is>
+          <t>https://www.rbk.no/om-rbk/ansatte/sport</t>
+        </is>
+      </c>
+      <c r="I150" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J150" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K150" s="7" t="inlineStr">
+        <is>
+          <t>Klub współpracuje z SciSports (scouting oparty na danych)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B151" s="7" t="inlineStr">
+        <is>
+          <t>Strømsgodset IF</t>
+        </is>
+      </c>
+      <c r="C151" s="7" t="inlineStr">
+        <is>
+          <t>Jan Vidar Haugstulen</t>
+        </is>
+      </c>
+      <c r="D151" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutteringsansvarlig, Eliteakademiet</t>
+        </is>
+      </c>
+      <c r="E151" s="7" t="inlineStr">
+        <is>
+          <t>Rekrutacja do akademii</t>
+        </is>
+      </c>
+      <c r="F151" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G151" s="7" t="inlineStr">
+        <is>
+          <t>tel. 913 32 753</t>
+        </is>
+      </c>
+      <c r="H151" s="8" t="inlineStr">
+        <is>
+          <t>https://www.godset.no/utvikling/eliteakademiet</t>
+        </is>
+      </c>
+      <c r="I151" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J151" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K151" s="7" t="inlineStr">
+        <is>
+          <t>Znana akademia wprowadzająca młodzież do 1. zespołu</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B152" s="7" t="inlineStr">
+        <is>
+          <t>FK Bodø/Glimt</t>
+        </is>
+      </c>
+      <c r="C152" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E152" s="7" t="inlineStr">
+        <is>
+          <t>Kontakt ogólny</t>
+        </is>
+      </c>
+      <c r="F152" s="7" t="inlineStr"/>
+      <c r="G152" s="7" t="inlineStr">
+        <is>
+          <t>bg@glimt.no</t>
+        </is>
+      </c>
+      <c r="H152" s="8" t="inlineStr">
+        <is>
+          <t>https://x.com/Glimt</t>
+        </is>
+      </c>
+      <c r="I152" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J152" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K152" s="7" t="inlineStr">
+        <is>
+          <t>Brak publicznego maila akademii</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="7" t="inlineStr">
+        <is>
+          <t>Norwegia</t>
+        </is>
+      </c>
+      <c r="B153" s="7" t="inlineStr">
+        <is>
+          <t>SK Brann</t>
+        </is>
+      </c>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D153" s="7" t="inlineStr">
+        <is>
+          <t>Akademiet</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
+          <t>Akademia</t>
+        </is>
+      </c>
+      <c r="F153" s="7" t="inlineStr">
+        <is>
+          <t>ukryty na stronie (ochrona antyspamowa) – skopiuj ze strony</t>
+        </is>
+      </c>
+      <c r="G153" s="7" t="inlineStr">
+        <is>
+          <t>tel. +47 55 59 85 00</t>
+        </is>
+      </c>
+      <c r="H153" s="8" t="inlineStr">
+        <is>
+          <t>https://www.brann.no/lag/akademiet/ansatte</t>
+        </is>
+      </c>
+      <c r="I153" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J153" s="7" t="inlineStr">
+        <is>
+          <t>Częściowo – brak maila osoby</t>
+        </is>
+      </c>
+      <c r="K153" s="7" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="7" t="inlineStr">
+        <is>
+          <t>Słowacja</t>
+        </is>
+      </c>
+      <c r="B154" s="7" t="inlineStr">
+        <is>
+          <t>MŠK Žilina</t>
+        </is>
+      </c>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
+          <t>Viktor Miko</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="inlineStr">
+        <is>
+          <t>Skauting U7–U12</t>
+        </is>
+      </c>
+      <c r="E154" s="7" t="inlineStr">
+        <is>
+          <t>Nabór i scouting najmłodszych</t>
+        </is>
+      </c>
+      <c r="F154" s="7" t="inlineStr">
+        <is>
+          <t>Viktor.Miko@mskzilina.sk</t>
+        </is>
+      </c>
+      <c r="G154" s="7" t="inlineStr">
+        <is>
+          <t>mskzilina@mskzilina.sk; +421 41 54 24 958</t>
+        </is>
+      </c>
+      <c r="H154" s="8" t="inlineStr">
+        <is>
+          <t>http://mskzilina.sk/nabor</t>
+        </is>
+      </c>
+      <c r="I154" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J154" s="7" t="inlineStr">
+        <is>
+          <t>Zweryfikowany</t>
+        </is>
+      </c>
+      <c r="K154" s="7" t="inlineStr">
+        <is>
+          <t>Jedna z najbardziej znanych akademii w Europie Środkowej</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="7" t="inlineStr">
+        <is>
+          <t>Słowenia</t>
+        </is>
+      </c>
+      <c r="B155" s="7" t="inlineStr">
+        <is>
+          <t>NK Maribor</t>
+        </is>
+      </c>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>Danijel Širec</t>
+        </is>
+      </c>
+      <c r="D155" s="7" t="inlineStr">
+        <is>
+          <t>Vodja skavtske službe (szef scoutingu)</t>
+        </is>
+      </c>
+      <c r="E155" s="7" t="inlineStr">
+        <is>
+          <t>Scouting akademii</t>
+        </is>
+      </c>
+      <c r="F155" s="7" t="inlineStr"/>
+      <c r="G155" s="7" t="inlineStr">
+        <is>
           <t>nogometna.sola@nkmaribor.com; 02 620 97 05</t>
         </is>
       </c>
-      <c r="H148" s="8" t="inlineStr">
+      <c r="H155" s="8" t="inlineStr">
         <is>
           <t>https://www.nkmaribor.com/footballSchool/basic/contact</t>
         </is>
       </c>
-      <c r="I148" s="9" t="n">
+      <c r="I155" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="J148" s="7" t="inlineStr">
+      <c r="J155" s="7" t="inlineStr">
         <is>
           <t>Zweryfikowany</t>
         </is>
       </c>
-      <c r="K148" s="7" t="inlineStr">
+      <c r="K155" s="7" t="inlineStr">
         <is>
           <t>Dyrektor szkółki: Sebastijan Harc; dyr. sportowy: Boštjan Kreft</t>
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" s="7" t="inlineStr">
+        <is>
+          <t>Szkocja</t>
+        </is>
+      </c>
+      <c r="B156" s="7" t="inlineStr">
+        <is>
+          <t>Celtic FC</t>
+        </is>
+      </c>
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>Celtic FC Academy – trials</t>
+        </is>
+      </c>
+      <c r="E156" s="7" t="inlineStr">
+        <is>
+          <t>Zgłoszenia zawodników</t>
+        </is>
+      </c>
+      <c r="F156" s="7" t="inlineStr"/>
+      <c r="G156" s="7" t="inlineStr">
+        <is>
+          <t>youthtrials@celticfc.co.uk</t>
+        </is>
+      </c>
+      <c r="H156" s="8" t="inlineStr">
+        <is>
+          <t>https://www.celticfc.com/academy/academy-faqs</t>
+        </is>
+      </c>
+      <c r="I156" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J156" s="7" t="inlineStr">
+        <is>
+          <t>Do potwierdzenia</t>
+        </is>
+      </c>
+      <c r="K156" s="7" t="inlineStr">
+        <is>
+          <t>CIES: czołówka pressingu (12,4). Adres z FAQ akademii – potwierdzić</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K148"/>
-  <conditionalFormatting sqref="A2:K148">
+  <autoFilter ref="A1:K156"/>
+  <conditionalFormatting sqref="A2:K156">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Zweryfikowany"</formula>
     </cfRule>
@@ -8701,13 +9132,13 @@
       <formula>$J2="Do potwierdzenia"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I148">
+  <conditionalFormatting sqref="I2:I156">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>$I2=1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Zweryfikowany,Częściowo – brak maila osoby,Do potwierdzenia"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8766,117 +9197,125 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H145" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H147" r:id="rId164"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H148" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H149" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H150" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H151" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H152" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H153" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H154" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H155" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H156" r:id="rId173"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9105,7 +9544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -10106,15 +10545,239 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Saldo transferów netto 2015–2024 (mln €)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Benfica +816, Ajax +473, RB Salzburg +401, LOSC Lille +391, Sporting +345</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Wszystkie w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Saldo transferów netto 2015–2024 (mln €)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>6–10</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Monaco +305, Porto +296, Braga +279, Dinamo Zagrzeb +255, PSV +250</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>Wszystkie w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Saldo transferów netto 2015–2024 (mln €)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>11–15</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>AZ +224, FC Nordsjælland +219, KRC Genk +211, Udinese +208, Atalanta +206</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Wszystkie w arkuszu Kontakty</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Saldo transferów netto 2015–2024 (mln €)</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>16–20</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Athletico Paranaense +200, Lyon +196, Palmeiras +194, Szachtar +190, Fluminense +186</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Lyon, Szachtar w Kontaktach; kluby brazylijskie poza zakresem</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Pressing wysokiej intensywności na mecz (28 lig, 2023/24)</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Man. City 15,2; Leverkusen 13,9; Columbus Crew 13,5; PSG 12,6; Malmö FF 12,4</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Europejskie w Kontaktach</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Pressing wysokiej intensywności na mecz (28 lig, 2023/24)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>5–10</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Southampton 12,4; Celtic 12,4; Barcelona 12,3; PSV 12,3; Dinamo Zagrzeb 12,3</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Wszystkie w Kontaktach</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Pressing wysokiej intensywności na mecz (28 lig, 2023/24)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>11–19</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Tottenham 12,2; Czornomoreć 12,2; Bayern 12,1; Chelsea 12,1; Ajax 12,0; Leeds 11,9; Sunderland 11,9; Monaco 11,8; Gent 11,7; Häcken 11,7</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>różne</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Europejskie (bez Czornomorca) w Kontaktach</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Źródła: CIES Football Observatory – Weekly Post 529 (training clubs), Weekly Post 540 (most profitable academies), 2026; Monthly Report 99 (II 2025); Monthly Report 98 (XII 2024) – ranking zawodników U21, nie akademii; wymieniono tylko kluby podane w publikacjach o raporcie. football-observatory.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>